<commit_message>
El Excel agrupa las inversiones bajo su cuenta y suma el total de cada cuenta
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>MIS INVERSIONES · MOVIMIENTOS: DE DÓNDE VIENE EL DINERO</t>
   </si>
@@ -38,7 +38,7 @@
     <t>Saldo</t>
   </si>
   <si>
-    <t>Cada cuenta y cada inversión, por separado; abajo, el total de cada titular y el TOTAL de todo junto.</t>
+    <t>Resumen de cada cuenta, con lo invertido en cada inversión debajo; después, el total de cada cuenta, el de cada titular y el TOTAL.</t>
   </si>
   <si>
     <t>MOVIMIENTOS</t>
@@ -59,7 +59,7 @@
     <t>Importe</t>
   </si>
   <si>
-    <t>Cuenta o inversión</t>
+    <t>Cuenta e inversiones</t>
   </si>
   <si>
     <t>Titular</t>
@@ -83,27 +83,27 @@
     <t>Marta</t>
   </si>
   <si>
+    <t>Vanguard Global Stock Index</t>
+  </si>
+  <si>
+    <t>Fidelity MSCI World Index</t>
+  </si>
+  <si>
+    <t>Cartera indexada Metal</t>
+  </si>
+  <si>
+    <t>Depósito 12 meses</t>
+  </si>
+  <si>
+    <t>Plan de pensiones indexado global</t>
+  </si>
+  <si>
     <t>Cuenta nómina · BBVA</t>
   </si>
   <si>
     <t>Cuenta ahorro · ING</t>
   </si>
   <si>
-    <t>Vanguard Global Stock Index</t>
-  </si>
-  <si>
-    <t>Fidelity MSCI World Index</t>
-  </si>
-  <si>
-    <t>Cartera indexada Metal</t>
-  </si>
-  <si>
-    <t>Depósito 12 meses</t>
-  </si>
-  <si>
-    <t>Plan de pensiones indexado global</t>
-  </si>
-  <si>
     <t>Fondo indexado</t>
   </si>
   <si>
@@ -113,6 +113,9 @@
     <t>Depósito ahorro</t>
   </si>
   <si>
+    <t>Total MyInvestor</t>
+  </si>
+  <si>
     <t>Total Marta</t>
   </si>
   <si>
@@ -122,7 +125,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Para añadir un producto: escribe su nombre (y su titular) en una fila libre del resumen. Para quitarlo: borra su fila.</t>
+    <t>Para añadir un producto: escribe su nombre (y su titular) en una fila libre, debajo de la cuenta desde la que lo pagas. Para quitarlo: borra su fila.</t>
   </si>
   <si>
     <t>El saldo de las inversiones es su valor de hoy: escríbelo tú en la celda amarilla. «Exterior» es el dinero que entra o sale de fuera; «Interés», lo que paga el banco o la inversión (rentabilidad, no dinero aportado).</t>
@@ -137,7 +140,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -190,14 +193,11 @@
       <sz val="10"/>
     </font>
     <font>
+      <b/>
+      <color rgb="FF0F172A"/>
       <sz val="10"/>
     </font>
     <font>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -259,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -290,24 +290,36 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -717,11 +729,12 @@
     <col min="2" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="2" customWidth="1"/>
-    <col min="6" max="6" width="27" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -890,7 +903,7 @@
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="11"/>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="18" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="15" t="s">
@@ -905,9 +918,7 @@
       <c r="J9" s="16">
         <f>IF($F9="","",IF(AND($H9=0,$K9=0),"",$K9-$H9))</f>
       </c>
-      <c r="K9" s="16">
-        <f>IF($F9="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F9)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F9))</f>
-      </c>
+      <c r="K9" s="19"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
@@ -916,7 +927,7 @@
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="11"/>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="18" t="s">
         <v>23</v>
       </c>
       <c r="G10" s="15" t="s">
@@ -931,9 +942,7 @@
       <c r="J10" s="16">
         <f>IF($F10="","",IF(AND($H10=0,$K10=0),"",$K10-$H10))</f>
       </c>
-      <c r="K10" s="16">
-        <f>IF($F10="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F10)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F10))</f>
-      </c>
+      <c r="K10" s="19"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
@@ -942,7 +951,7 @@
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="18" t="s">
         <v>24</v>
       </c>
       <c r="G11" s="15" t="s">
@@ -957,7 +966,7 @@
       <c r="J11" s="16">
         <f>IF($F11="","",IF(AND($H11=0,$K11=0),"",$K11-$H11))</f>
       </c>
-      <c r="K11" s="18"/>
+      <c r="K11" s="19"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
@@ -966,7 +975,7 @@
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G12" s="15" t="s">
@@ -981,7 +990,7 @@
       <c r="J12" s="16">
         <f>IF($F12="","",IF(AND($H12=0,$K12=0),"",$K12-$H12))</f>
       </c>
-      <c r="K12" s="18"/>
+      <c r="K12" s="19"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
@@ -990,7 +999,7 @@
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="18" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="15" t="s">
@@ -1005,7 +1014,7 @@
       <c r="J13" s="16">
         <f>IF($F13="","",IF(AND($H13=0,$K13=0),"",$K13-$H13))</f>
       </c>
-      <c r="K13" s="18"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
@@ -1014,12 +1023,8 @@
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
-      <c r="F14" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="F14" s="20"/>
+      <c r="G14" s="21"/>
       <c r="H14" s="16">
         <f>IF($F14="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F14)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F14)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F14,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F14,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1029,7 +1034,7 @@
       <c r="J14" s="16">
         <f>IF($F14="","",IF(AND($H14=0,$K14=0),"",$K14-$H14))</f>
       </c>
-      <c r="K14" s="18"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
@@ -1038,12 +1043,8 @@
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
-      <c r="F15" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="F15" s="20"/>
+      <c r="G15" s="21"/>
       <c r="H15" s="16">
         <f>IF($F15="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F15)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F15)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F15,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F15,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1053,7 +1054,7 @@
       <c r="J15" s="16">
         <f>IF($F15="","",IF(AND($H15=0,$K15=0),"",$K15-$H15))</f>
       </c>
-      <c r="K15" s="18"/>
+      <c r="K15" s="19"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
@@ -1062,12 +1063,8 @@
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
-      <c r="F16" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>30</v>
-      </c>
+      <c r="F16" s="20"/>
+      <c r="G16" s="21"/>
       <c r="H16" s="16">
         <f>IF($F16="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F16)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F16)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F16,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F16,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1077,7 +1074,7 @@
       <c r="J16" s="16">
         <f>IF($F16="","",IF(AND($H16=0,$K16=0),"",$K16-$H16))</f>
       </c>
-      <c r="K16" s="18"/>
+      <c r="K16" s="19"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
@@ -1087,10 +1084,10 @@
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="F17" s="14" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="H17" s="16">
         <f>IF($F17="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F17)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F17)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F17,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F17,$C$6:$C$205,"Interés"))</f>
@@ -1101,7 +1098,9 @@
       <c r="J17" s="16">
         <f>IF($F17="","",IF(AND($H17=0,$K17=0),"",$K17-$H17))</f>
       </c>
-      <c r="K17" s="18"/>
+      <c r="K17" s="16">
+        <f>IF($F17="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F17)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F17))</f>
+      </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
@@ -1110,8 +1109,12 @@
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="20"/>
+      <c r="F18" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="H18" s="16">
         <f>IF($F18="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F18)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F18)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F18,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F18,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1121,7 +1124,9 @@
       <c r="J18" s="16">
         <f>IF($F18="","",IF(AND($H18=0,$K18=0),"",$K18-$H18))</f>
       </c>
-      <c r="K18" s="18"/>
+      <c r="K18" s="16">
+        <f>IF($F18="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F18)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F18))</f>
+      </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
@@ -1130,8 +1135,12 @@
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="20"/>
+      <c r="F19" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="H19" s="16">
         <f>IF($F19="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F19)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F19)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F19,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F19,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1141,7 +1150,7 @@
       <c r="J19" s="16">
         <f>IF($F19="","",IF(AND($H19=0,$K19=0),"",$K19-$H19))</f>
       </c>
-      <c r="K19" s="18"/>
+      <c r="K19" s="19"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
@@ -1150,8 +1159,12 @@
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="11"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
+      <c r="F20" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="H20" s="16">
         <f>IF($F20="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F20)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F20)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F20,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F20,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1161,7 +1174,7 @@
       <c r="J20" s="16">
         <f>IF($F20="","",IF(AND($H20=0,$K20=0),"",$K20-$H20))</f>
       </c>
-      <c r="K20" s="18"/>
+      <c r="K20" s="19"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
@@ -1170,8 +1183,8 @@
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="21"/>
       <c r="H21" s="16">
         <f>IF($F21="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F21)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F21)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F21,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F21,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1181,7 +1194,7 @@
       <c r="J21" s="16">
         <f>IF($F21="","",IF(AND($H21=0,$K21=0),"",$K21-$H21))</f>
       </c>
-      <c r="K21" s="18"/>
+      <c r="K21" s="19"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
@@ -1190,8 +1203,8 @@
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="21"/>
       <c r="H22" s="16">
         <f>IF($F22="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F22)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F22)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F22,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F22,$C$6:$C$205,"Interés"))</f>
       </c>
@@ -1201,35 +1214,39 @@
       <c r="J22" s="16">
         <f>IF($F22="","",IF(AND($H22=0,$K22=0),"",$K22-$H22))</f>
       </c>
-      <c r="K22" s="18"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K22" s="19"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>46317</v>
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="16">
-        <f>IF($F23="","",SUMIFS($D$6:$D$205,$C$6:$C$205,$F23)-SUMIFS($D$6:$D$205,$B$6:$B$205,$F23)-SUMIFS($D$6:$D$205,$C$6:$C$205,$F23,$B$6:$B$205,"Interés")+SUMIFS($D$6:$D$205,$B$6:$B$205,$F23,$C$6:$C$205,"Interés"))</f>
-      </c>
-      <c r="I23" s="17">
-        <f>IF($F23="","",IF($H23=0,"",$J23/$H23))</f>
-      </c>
-      <c r="J23" s="16">
-        <f>IF($F23="","",IF(AND($H23=0,$K23=0),"",$K23-$H23))</f>
-      </c>
-      <c r="K23" s="18"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>46317</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
+      <c r="F24" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="23"/>
+      <c r="H24" s="24">
+        <f>IF(SUM($H$8:$H$16)=0,"",SUM($H$8:$H$16))</f>
+      </c>
+      <c r="I24" s="25">
+        <f>IF($H24=0,"",$J24/$H24)</f>
+      </c>
+      <c r="J24" s="24">
+        <f>IF(SUM($J$8:$J$16)=0,"",SUM($J$8:$J$16))</f>
+      </c>
+      <c r="K24" s="24">
+        <f>IF(SUM($K$8:$K$16)=0,"",SUM($K$8:$K$16))</f>
+      </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
@@ -1238,23 +1255,23 @@
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="11"/>
-      <c r="F25" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="G25" s="22" t="s">
+      <c r="F25" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="G25" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H25" s="23">
-        <f>SUMIF($G$6:$G$23,$G25,$H$6:$H$23)</f>
-      </c>
-      <c r="I25" s="24">
+      <c r="H25" s="24">
+        <f>IF(SUMIFS($H$6:$H$22,$G$6:$G$22,$G25)=0,"",SUMIFS($H$6:$H$22,$G$6:$G$22,$G25))</f>
+      </c>
+      <c r="I25" s="25">
         <f>IF($H25=0,"",$J25/$H25)</f>
       </c>
-      <c r="J25" s="23">
-        <f>SUMIF($G$6:$G$23,$G25,$J$6:$J$23)</f>
-      </c>
-      <c r="K25" s="23">
-        <f>SUMIF($G$6:$G$23,$G25,$K$6:$K$23)</f>
+      <c r="J25" s="24">
+        <f>IF(SUMIFS($J$6:$J$22,$G$6:$G$22,$G25)=0,"",SUMIFS($J$6:$J$22,$G$6:$G$22,$G25))</f>
+      </c>
+      <c r="K25" s="24">
+        <f>IF(SUMIFS($K$6:$K$22,$G$6:$G$22,$G25)=0,"",SUMIFS($K$6:$K$22,$G$6:$G$22,$G25))</f>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1264,23 +1281,23 @@
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
-      <c r="F26" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="22" t="s">
+      <c r="F26" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="H26" s="23">
-        <f>SUMIF($G$6:$G$23,$G26,$H$6:$H$23)</f>
-      </c>
-      <c r="I26" s="24">
+      <c r="H26" s="24">
+        <f>IF(SUMIFS($H$6:$H$22,$G$6:$G$22,$G26)=0,"",SUMIFS($H$6:$H$22,$G$6:$G$22,$G26))</f>
+      </c>
+      <c r="I26" s="25">
         <f>IF($H26=0,"",$J26/$H26)</f>
       </c>
-      <c r="J26" s="23">
-        <f>SUMIF($G$6:$G$23,$G26,$J$6:$J$23)</f>
-      </c>
-      <c r="K26" s="23">
-        <f>SUMIF($G$6:$G$23,$G26,$K$6:$K$23)</f>
+      <c r="J26" s="24">
+        <f>IF(SUMIFS($J$6:$J$22,$G$6:$G$22,$G26)=0,"",SUMIFS($J$6:$J$22,$G$6:$G$22,$G26))</f>
+      </c>
+      <c r="K26" s="24">
+        <f>IF(SUMIFS($K$6:$K$22,$G$6:$G$22,$G26)=0,"",SUMIFS($K$6:$K$22,$G$6:$G$22,$G26))</f>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1290,21 +1307,21 @@
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="11"/>
-      <c r="F27" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="G27" s="25"/>
-      <c r="H27" s="26">
-        <f>SUM($H$6:$H$23)</f>
-      </c>
-      <c r="I27" s="27">
+      <c r="F27" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="G27" s="27"/>
+      <c r="H27" s="28">
+        <f>IF(SUM($H$6:$H$22)=0,"",SUM($H$6:$H$22))</f>
+      </c>
+      <c r="I27" s="29">
         <f>IF($H27=0,"",$J27/$H27)</f>
       </c>
-      <c r="J27" s="26">
-        <f>SUM($J$6:$J$23)</f>
-      </c>
-      <c r="K27" s="26">
-        <f>SUM($K$6:$K$23)</f>
+      <c r="J27" s="28">
+        <f>IF(SUM($J$6:$J$22)=0,"",SUM($J$6:$J$22))</f>
+      </c>
+      <c r="K27" s="28">
+        <f>IF(SUM($K$6:$K$22)=0,"",SUM($K$6:$K$22))</f>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1316,34 +1333,34 @@
       <c r="D28" s="11"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
+      <c r="A29" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="28"/>
+      <c r="A30" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="30"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
@@ -2767,7 +2784,7 @@
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J23">
+  <conditionalFormatting sqref="I6:J22">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
@@ -2777,10 +2794,10 @@
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="B6:B205">
-      <formula1>$F$6:$F$23</formula1>
+      <formula1>$F$6:$F$22</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C6:C205">
-      <formula1>$F$6:$F$23</formula1>
+      <formula1>$F$6:$F$22</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" sqref="D6:D205">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
El color de cada fila lo marca su titular: también en las inversiones que añadas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -141,7 +141,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -212,10 +212,6 @@
     </font>
     <font>
       <color rgb="FFEA580C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -320,7 +316,7 @@
     <xf numFmtId="166" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -328,10 +324,10 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -349,7 +345,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="7">
     <dxf>
       <font>
         <color rgb="FF0F172A"/>
@@ -389,6 +385,16 @@
       <font>
         <color rgb="FFFFFFFF"/>
         <sz val="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF2447B8"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFEA580C"/>
       </font>
     </dxf>
     <dxf>
@@ -1881,11 +1887,19 @@
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F9:F23">
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="7">
+      <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I6:J23">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
El gráfico del Excel, como el modelo: dos barras por titular (aportado neto y beneficio-pérdida), con el importe encima
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -8,7 +8,7 @@
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$23),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$K43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$K47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>MIS INVERSIONES · MOVIMIENTOS: DE DÓNDE VIENE EL DINERO</t>
   </si>
@@ -117,10 +117,10 @@
     <t>Total MyInvestor</t>
   </si>
   <si>
+    <t>Total Marta</t>
+  </si>
+  <si>
     <t>Total Fondo ahorro</t>
-  </si>
-  <si>
-    <t>Total Marta</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -426,9 +426,23 @@
   <c:chart>
     <c:title>
       <c:tx>
-        <c:v>Aportado · Rentabilidad · Saldo por cuenta</c:v>
+        <c:v>Aportado neto y beneficio / pérdida por titular</c:v>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -441,25 +455,41 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Aportado</c:v>
+            <c:v>Aportado neto</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1D4ED8"/>
+              <a:srgbClr val="2563EB"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>Movimientos!$F$25:$F$26</c:f>
-            </c:strRef>
+            <c:strLit>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$25:$H$26</c:f>
+              <c:f>Movimientos!$H$26:$H$27</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -467,56 +497,46 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Rentabilidad</c:v>
+            <c:v>Beneficio-pérdida</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="047857"/>
+              <a:srgbClr val="E67E22"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
           <c:cat>
-            <c:strRef>
-              <c:f>Movimientos!$F$25:$F$26</c:f>
-            </c:strRef>
+            <c:strLit>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$25:$J$26</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Saldo</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="EA580C"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Movimientos!$F$25:$F$26</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$K$25:$K$26</c:f>
+              <c:f>Movimientos!$J$26:$J$27</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
         <c:gapWidth val="60"/>
-        <c:overlap val="-10"/>
+        <c:overlap val="-80"/>
         <c:axId val="100000001"/>
         <c:axId val="100000002"/>
       </c:barChart>
@@ -552,12 +572,26 @@
         <c:crossAx val="100000001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:valAx>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -586,7 +620,7 @@
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1491,18 +1525,20 @@
       <c r="F26" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="25"/>
+      <c r="G26" s="28" t="s">
+        <v>21</v>
+      </c>
       <c r="H26" s="26">
-        <f>IFERROR(IF(SUM($H$16:$H$17)=0,"",SUM($H$16:$H$17)),"")</f>
+        <f>IFERROR(IF(SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")),"")</f>
       </c>
       <c r="I26" s="27">
         <f>IFERROR(IF($H26=0,"",$J26/$H26),"")</f>
       </c>
       <c r="J26" s="26">
-        <f>IFERROR(IF(SUM($J$16:$J$17)=0,"",SUM($J$16:$J$17)),"")</f>
+        <f>IFERROR(IF(SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")),"")</f>
       </c>
       <c r="K26" s="26">
-        <f>IFERROR(IF(SUM($K$16:$K$17)=0,"",SUM($K$16:$K$17)),"")</f>
+        <f>IFERROR(IF(SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")),"")</f>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1516,19 +1552,19 @@
         <v>34</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H27" s="26">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($H$6:$H$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
       </c>
       <c r="I27" s="27">
         <f>IFERROR(IF($H27=0,"",$J27/$H27),"")</f>
       </c>
       <c r="J27" s="26">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($J$6:$J$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
       </c>
       <c r="K27" s="26">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($K$6:$K$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
El Excel: sin «Interés», nombres cortos, una sola fila amarilla, 500 movimientos, gráfico en L-O y hoja protegida
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -7,8 +7,8 @@
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$23),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$K47</definedName>
+    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$30),1),1)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O50</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
   <si>
     <t>MIS INVERSIONES · MOVIMIENTOS: DE DÓNDE VIENE EL DINERO</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Importe</t>
   </si>
   <si>
-    <t>Cuenta e inversiones</t>
+    <t>Inversiones</t>
   </si>
   <si>
     <t>Titular</t>
@@ -75,10 +75,7 @@
     <t>Exterior</t>
   </si>
   <si>
-    <t>Interés</t>
-  </si>
-  <si>
-    <t>MyInvestor</t>
+    <t>Cuenta Myinvestor</t>
   </si>
   <si>
     <t>Marta</t>
@@ -96,10 +93,7 @@
     <t>Depósito 12 meses</t>
   </si>
   <si>
-    <t>Plan de pensiones indexado global</t>
-  </si>
-  <si>
-    <t>Cuenta nómina · BBVA</t>
+    <t>Plan de pensiones indexado</t>
   </si>
   <si>
     <t>Cuenta ahorro · ING</t>
@@ -111,13 +105,10 @@
     <t>Fondo ahorro</t>
   </si>
   <si>
-    <t>Depósito ahorro</t>
+    <t>iShares Developed World Index</t>
   </si>
   <si>
-    <t>Total MyInvestor</t>
-  </si>
-  <si>
-    <t>Total Marta</t>
+    <t>Total Cuenta Myinvestor-Marta</t>
   </si>
   <si>
     <t>Total Fondo ahorro</t>
@@ -126,10 +117,10 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Para añadir una inversión: escribe su nombre (y su titular) en una fila libre del final. Para quitarla: borra su fila. Entra al momento en los desplegables.</t>
+    <t>Para añadir una inversión: escribe su nombre (y su titular) en la fila amarilla; al rellenarla sale la siguiente. Para quitarla: borra su nombre y desaparece. Entra al momento en los desplegables.</t>
   </si>
   <si>
-    <t>En las inversiones se escribe la rentabilidad en % (la celda amarilla, como en la app) y el saldo se calcula solo. «Exterior» es el dinero que entra o sale de fuera; «Interés», lo que paga el banco (rentabilidad, no dinero aportado).</t>
+    <t>En las inversiones se escribe la rentabilidad en % (la celda amarilla, como en la app) y el saldo se calcula solo. «Exterior» es el dinero que entra o sale de fuera. La hoja está protegida: solo se puede escribir en los movimientos, en las filas nuevas y en el %.</t>
   </si>
 </sst>
 </file>
@@ -141,7 +132,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -199,9 +190,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
-    </font>
-    <font>
       <color rgb="FF2447B8"/>
       <sz val="10"/>
     </font>
@@ -215,11 +203,19 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,11 +242,6 @@
         <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFBEB"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -273,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -299,39 +290,64 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -340,12 +356,14 @@
     <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="12">
     <dxf>
       <font>
         <color rgb="FF0F172A"/>
@@ -386,6 +404,61 @@
         <color rgb="FFFFFFFF"/>
         <sz val="10"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0F172A"/>
+        <sz val="10"/>
+      </font>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8DEE9"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0F172A"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFBEB"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8DEE9"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+        <sz val="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFBEB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFBEB"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -489,7 +562,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$26:$H$27</c:f>
+              <c:f>Movimientos!$H$32:$H$33</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -531,7 +604,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$26:$J$27</c:f>
+              <c:f>Movimientos!$J$32:$J$33</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -612,15 +685,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -969,7 +1042,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K505"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -982,6 +1055,7 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="15" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1108,14 +1182,24 @@
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="11"/>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
+      <c r="G7" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="16">
+        <f>IFERROR(IF($F7="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F7)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F7)),"")</f>
+      </c>
+      <c r="I7" s="17">
+        <f>IFERROR(IF($F7="","",IF($H7=0,"",$J7/$H7)),"")</f>
+      </c>
+      <c r="J7" s="16">
+        <f>IFERROR(IF($F7="","",$K7-$H7),"")</f>
+      </c>
+      <c r="K7" s="16">
+        <f>IFERROR(IF($F7="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F7)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F7)),"")</f>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
@@ -1124,23 +1208,21 @@
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="11"/>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="15" t="s">
-        <v>21</v>
-      </c>
       <c r="H8" s="16">
-        <f>IFERROR(IF($F8="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F8)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F8)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F8,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F8,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I8" s="17">
-        <f>IFERROR(IF($F8="","",IF($H8=0,"",$J8/$H8)),"")</f>
-      </c>
+        <f>IFERROR(IF($F8="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F8)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F8)),"")</f>
+      </c>
+      <c r="I8" s="19"/>
       <c r="J8" s="16">
         <f>IFERROR(IF($F8="","",$K8-$H8),"")</f>
       </c>
       <c r="K8" s="16">
-        <f>IFERROR(IF($F8="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F8)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F8)),"")</f>
+        <f>IFERROR(IF($F8="","",IF($H8=0,"",IF($I8="",$H8,$H8*(1+$I8)))),"")</f>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1150,20 +1232,20 @@
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="11"/>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="20" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="16">
-        <f>IFERROR(IF($F9="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F9)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F9)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F9,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F9,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I9" s="19"/>
-      <c r="J9" s="16">
+        <v>20</v>
+      </c>
+      <c r="H9" s="21">
+        <f>IFERROR(IF($F9="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F9)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F9)),"")</f>
+      </c>
+      <c r="I9" s="22"/>
+      <c r="J9" s="21">
         <f>IFERROR(IF($F9="","",$K9-$H9),"")</f>
       </c>
-      <c r="K9" s="16">
+      <c r="K9" s="21">
         <f>IFERROR(IF($F9="","",IF($H9=0,"",IF($I9="",$H9,$H9*(1+$I9)))),"")</f>
       </c>
     </row>
@@ -1174,20 +1256,20 @@
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="11"/>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="20" t="s">
         <v>23</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10" s="16">
-        <f>IFERROR(IF($F10="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F10)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F10)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F10,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F10,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I10" s="19"/>
-      <c r="J10" s="16">
+        <v>20</v>
+      </c>
+      <c r="H10" s="21">
+        <f>IFERROR(IF($F10="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F10)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F10)),"")</f>
+      </c>
+      <c r="I10" s="22"/>
+      <c r="J10" s="21">
         <f>IFERROR(IF($F10="","",$K10-$H10),"")</f>
       </c>
-      <c r="K10" s="16">
+      <c r="K10" s="21">
         <f>IFERROR(IF($F10="","",IF($H10=0,"",IF($I10="",$H10,$H10*(1+$I10)))),"")</f>
       </c>
     </row>
@@ -1198,20 +1280,20 @@
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="20" t="s">
         <v>24</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="16">
-        <f>IFERROR(IF($F11="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F11)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F11)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F11,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F11,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I11" s="19"/>
-      <c r="J11" s="16">
+        <v>20</v>
+      </c>
+      <c r="H11" s="21">
+        <f>IFERROR(IF($F11="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F11)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F11)),"")</f>
+      </c>
+      <c r="I11" s="22"/>
+      <c r="J11" s="21">
         <f>IFERROR(IF($F11="","",$K11-$H11),"")</f>
       </c>
-      <c r="K11" s="16">
+      <c r="K11" s="21">
         <f>IFERROR(IF($F11="","",IF($H11=0,"",IF($I11="",$H11,$H11*(1+$I11)))),"")</f>
       </c>
     </row>
@@ -1222,20 +1304,20 @@
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="20" t="s">
         <v>25</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="16">
-        <f>IFERROR(IF($F12="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F12)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F12)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F12,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F12,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I12" s="19"/>
-      <c r="J12" s="16">
+        <v>20</v>
+      </c>
+      <c r="H12" s="21">
+        <f>IFERROR(IF($F12="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F12)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F12)),"")</f>
+      </c>
+      <c r="I12" s="22"/>
+      <c r="J12" s="21">
         <f>IFERROR(IF($F12="","",$K12-$H12),"")</f>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="21">
         <f>IFERROR(IF($F12="","",IF($H12=0,"",IF($I12="",$H12,$H12*(1+$I12)))),"")</f>
       </c>
     </row>
@@ -1246,21 +1328,23 @@
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="23" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="16">
-        <f>IFERROR(IF($F13="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F13)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F13)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F13,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F13,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I13" s="19"/>
-      <c r="J13" s="16">
+        <v>20</v>
+      </c>
+      <c r="H13" s="21">
+        <f>IFERROR(IF($F13="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)),"")</f>
+      </c>
+      <c r="I13" s="24">
+        <f>IFERROR(IF($F13="","",IF($H13=0,"",$J13/$H13)),"")</f>
+      </c>
+      <c r="J13" s="21">
         <f>IFERROR(IF($F13="","",$K13-$H13),"")</f>
       </c>
-      <c r="K13" s="16">
-        <f>IFERROR(IF($F13="","",IF($H13=0,"",IF($I13="",$H13,$H13*(1+$I13)))),"")</f>
+      <c r="K13" s="21">
+        <f>IFERROR(IF($F13="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)),"")</f>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1270,23 +1354,21 @@
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="25" t="s">
         <v>27</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" s="16">
-        <f>IFERROR(IF($F14="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F14)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F14)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F14,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F14,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I14" s="17">
-        <f>IFERROR(IF($F14="","",IF($H14=0,"",$J14/$H14)),"")</f>
-      </c>
-      <c r="J14" s="16">
+        <v>28</v>
+      </c>
+      <c r="H14" s="26">
+        <f>IFERROR(IF($F14="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)),"")</f>
+      </c>
+      <c r="I14" s="27"/>
+      <c r="J14" s="26">
         <f>IFERROR(IF($F14="","",$K14-$H14),"")</f>
       </c>
-      <c r="K14" s="16">
-        <f>IFERROR(IF($F14="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F14)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F14)),"")</f>
+      <c r="K14" s="26">
+        <f>IFERROR(IF($F14="","",IF($H14=0,"",IF($I14="",$H14,$H14*(1+$I14)))),"")</f>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1296,23 +1378,21 @@
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" s="16">
-        <f>IFERROR(IF($F15="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F15)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F15)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F15,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F15,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I15" s="17">
-        <f>IFERROR(IF($F15="","",IF($H15=0,"",$J15/$H15)),"")</f>
-      </c>
-      <c r="J15" s="16">
+      <c r="H15" s="26">
+        <f>IFERROR(IF($F15="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15)),"")</f>
+      </c>
+      <c r="I15" s="27"/>
+      <c r="J15" s="26">
         <f>IFERROR(IF($F15="","",$K15-$H15),"")</f>
       </c>
-      <c r="K15" s="16">
-        <f>IFERROR(IF($F15="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F15)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F15)),"")</f>
+      <c r="K15" s="26">
+        <f>IFERROR(IF($F15="","",IF($H15=0,"",IF($I15="",$H15,$H15*(1+$I15)))),"")</f>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1322,20 +1402,16 @@
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
-      <c r="F16" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" s="16">
-        <f>IFERROR(IF($F16="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F16)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F16)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F16,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F16,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I16" s="19"/>
-      <c r="J16" s="16">
+      <c r="F16" s="28"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="30">
+        <f>IFERROR(IF($F16="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)),"")</f>
+      </c>
+      <c r="I16" s="31"/>
+      <c r="J16" s="30">
         <f>IFERROR(IF($F16="","",$K16-$H16),"")</f>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="30">
         <f>IFERROR(IF($F16="","",IF($H16=0,"",IF($I16="",$H16,$H16*(1+$I16)))),"")</f>
       </c>
     </row>
@@ -1346,20 +1422,16 @@
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
-      <c r="F17" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H17" s="16">
-        <f>IFERROR(IF($F17="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F17)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F17)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F17,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F17,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I17" s="19"/>
-      <c r="J17" s="16">
+      <c r="F17" s="28"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="30">
+        <f>IFERROR(IF($F17="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)),"")</f>
+      </c>
+      <c r="I17" s="31"/>
+      <c r="J17" s="30">
         <f>IFERROR(IF($F17="","",$K17-$H17),"")</f>
       </c>
-      <c r="K17" s="16">
+      <c r="K17" s="30">
         <f>IFERROR(IF($F17="","",IF($H17=0,"",IF($I17="",$H17,$H17*(1+$I17)))),"")</f>
       </c>
     </row>
@@ -1370,16 +1442,16 @@
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="16">
-        <f>IFERROR(IF($F18="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F18)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F18)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F18,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F18,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I18" s="19"/>
-      <c r="J18" s="16">
+      <c r="F18" s="28"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="30">
+        <f>IFERROR(IF($F18="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18)),"")</f>
+      </c>
+      <c r="I18" s="31"/>
+      <c r="J18" s="30">
         <f>IFERROR(IF($F18="","",$K18-$H18),"")</f>
       </c>
-      <c r="K18" s="16">
+      <c r="K18" s="30">
         <f>IFERROR(IF($F18="","",IF($H18=0,"",IF($I18="",$H18,$H18*(1+$I18)))),"")</f>
       </c>
     </row>
@@ -1390,16 +1462,16 @@
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="16">
-        <f>IFERROR(IF($F19="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F19)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F19)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F19,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F19,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I19" s="19"/>
-      <c r="J19" s="16">
+      <c r="F19" s="28"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30">
+        <f>IFERROR(IF($F19="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19)),"")</f>
+      </c>
+      <c r="I19" s="31"/>
+      <c r="J19" s="30">
         <f>IFERROR(IF($F19="","",$K19-$H19),"")</f>
       </c>
-      <c r="K19" s="16">
+      <c r="K19" s="30">
         <f>IFERROR(IF($F19="","",IF($H19=0,"",IF($I19="",$H19,$H19*(1+$I19)))),"")</f>
       </c>
     </row>
@@ -1410,16 +1482,16 @@
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="11"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="16">
-        <f>IFERROR(IF($F20="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F20)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F20)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F20,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F20,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="16">
+      <c r="F20" s="28"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="30">
+        <f>IFERROR(IF($F20="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F20)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F20)),"")</f>
+      </c>
+      <c r="I20" s="31"/>
+      <c r="J20" s="30">
         <f>IFERROR(IF($F20="","",$K20-$H20),"")</f>
       </c>
-      <c r="K20" s="16">
+      <c r="K20" s="30">
         <f>IFERROR(IF($F20="","",IF($H20=0,"",IF($I20="",$H20,$H20*(1+$I20)))),"")</f>
       </c>
     </row>
@@ -1430,16 +1502,16 @@
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="16">
-        <f>IFERROR(IF($F21="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F21)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F21)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F21,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F21,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I21" s="19"/>
-      <c r="J21" s="16">
+      <c r="F21" s="28"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="30">
+        <f>IFERROR(IF($F21="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F21)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F21)),"")</f>
+      </c>
+      <c r="I21" s="31"/>
+      <c r="J21" s="30">
         <f>IFERROR(IF($F21="","",$K21-$H21),"")</f>
       </c>
-      <c r="K21" s="16">
+      <c r="K21" s="30">
         <f>IFERROR(IF($F21="","",IF($H21=0,"",IF($I21="",$H21,$H21*(1+$I21)))),"")</f>
       </c>
     </row>
@@ -1450,16 +1522,16 @@
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="16">
-        <f>IFERROR(IF($F22="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F22)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F22)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F22,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F22,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I22" s="19"/>
-      <c r="J22" s="16">
+      <c r="F22" s="28"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="30">
+        <f>IFERROR(IF($F22="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F22)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F22)),"")</f>
+      </c>
+      <c r="I22" s="31"/>
+      <c r="J22" s="30">
         <f>IFERROR(IF($F22="","",$K22-$H22),"")</f>
       </c>
-      <c r="K22" s="16">
+      <c r="K22" s="30">
         <f>IFERROR(IF($F22="","",IF($H22=0,"",IF($I22="",$H22,$H22*(1+$I22)))),"")</f>
       </c>
     </row>
@@ -1470,26 +1542,38 @@
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="16">
-        <f>IFERROR(IF($F23="","",SUMIFS($D$6:$D$65,$C$6:$C$65,$F23)-SUMIFS($D$6:$D$65,$B$6:$B$65,$F23)-SUMIFS($D$6:$D$65,$C$6:$C$65,$F23,$B$6:$B$65,"Interés")+SUMIFS($D$6:$D$65,$B$6:$B$65,$F23,$C$6:$C$65,"Interés")),"")</f>
-      </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="16">
+      <c r="F23" s="28"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="30">
+        <f>IFERROR(IF($F23="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F23)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F23)),"")</f>
+      </c>
+      <c r="I23" s="31"/>
+      <c r="J23" s="30">
         <f>IFERROR(IF($F23="","",$K23-$H23),"")</f>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="30">
         <f>IFERROR(IF($F23="","",IF($H23=0,"",IF($I23="",$H23,$H23*(1+$I23)))),"")</f>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>46317</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="30">
+        <f>IFERROR(IF($F24="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F24)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F24)),"")</f>
+      </c>
+      <c r="I24" s="31"/>
+      <c r="J24" s="30">
+        <f>IFERROR(IF($F24="","",$K24-$H24),"")</f>
+      </c>
+      <c r="K24" s="30">
+        <f>IFERROR(IF($F24="","",IF($H24=0,"",IF($I24="",$H24,$H24*(1+$I24)))),"")</f>
+      </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
@@ -1498,21 +1582,17 @@
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="11"/>
-      <c r="F25" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="26">
-        <f>IFERROR(IF(SUM($H$8:$H$13)=0,"",SUM($H$8:$H$13)),"")</f>
-      </c>
-      <c r="I25" s="27">
-        <f>IFERROR(IF($H25=0,"",$J25/$H25),"")</f>
-      </c>
-      <c r="J25" s="26">
-        <f>IFERROR(IF(SUM($J$8:$J$13)=0,"",SUM($J$8:$J$13)),"")</f>
-      </c>
-      <c r="K25" s="26">
-        <f>IFERROR(IF(SUM($K$8:$K$13)=0,"",SUM($K$8:$K$13)),"")</f>
+      <c r="F25" s="28"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="30">
+        <f>IFERROR(IF($F25="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F25)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F25)),"")</f>
+      </c>
+      <c r="I25" s="31"/>
+      <c r="J25" s="30">
+        <f>IFERROR(IF($F25="","",$K25-$H25),"")</f>
+      </c>
+      <c r="K25" s="30">
+        <f>IFERROR(IF($F25="","",IF($H25=0,"",IF($I25="",$H25,$H25*(1+$I25)))),"")</f>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1522,23 +1602,17 @@
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
-      <c r="F26" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26" s="26">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($H$6:$H$23,$G$6:$G$23,"Marta")),"")</f>
-      </c>
-      <c r="I26" s="27">
-        <f>IFERROR(IF($H26=0,"",$J26/$H26),"")</f>
-      </c>
-      <c r="J26" s="26">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($J$6:$J$23,$G$6:$G$23,"Marta")),"")</f>
-      </c>
-      <c r="K26" s="26">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")=0,"",SUMIFS($K$6:$K$23,$G$6:$G$23,"Marta")),"")</f>
+      <c r="F26" s="28"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="30">
+        <f>IFERROR(IF($F26="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F26)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F26)),"")</f>
+      </c>
+      <c r="I26" s="31"/>
+      <c r="J26" s="30">
+        <f>IFERROR(IF($F26="","",$K26-$H26),"")</f>
+      </c>
+      <c r="K26" s="30">
+        <f>IFERROR(IF($F26="","",IF($H26=0,"",IF($I26="",$H26,$H26*(1+$I26)))),"")</f>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1548,110 +1622,162 @@
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="11"/>
-      <c r="F27" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="G27" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="H27" s="26">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="I27" s="27">
-        <f>IFERROR(IF($H27=0,"",$J27/$H27),"")</f>
-      </c>
-      <c r="J27" s="26">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="K27" s="26">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$23,$G$6:$G$23,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$23,$G$6:$G$23,"Fondo ahorro")),"")</f>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F27" s="28"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30">
+        <f>IFERROR(IF($F27="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F27)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F27)),"")</f>
+      </c>
+      <c r="I27" s="31"/>
+      <c r="J27" s="30">
+        <f>IFERROR(IF($F27="","",$K27-$H27),"")</f>
+      </c>
+      <c r="K27" s="30">
+        <f>IFERROR(IF($F27="","",IF($H27=0,"",IF($I27="",$H27,$H27*(1+$I27)))),"")</f>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>46317</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="11"/>
-      <c r="F28" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="F28" s="28"/>
       <c r="G28" s="29"/>
       <c r="H28" s="30">
-        <f>IFERROR(IF(SUM($H$6:$H$23)=0,"",SUM($H$6:$H$23)),"")</f>
-      </c>
-      <c r="I28" s="31">
-        <f>IFERROR(IF($H28=0,"",$J28/$H28),"")</f>
-      </c>
+        <f>IFERROR(IF($F28="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F28)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F28)),"")</f>
+      </c>
+      <c r="I28" s="31"/>
       <c r="J28" s="30">
-        <f>IFERROR(IF(SUM($J$6:$J$23)=0,"",SUM($J$6:$J$23)),"")</f>
+        <f>IFERROR(IF($F28="","",$K28-$H28),"")</f>
       </c>
       <c r="K28" s="30">
-        <f>IFERROR(IF(SUM($K$6:$K$23)=0,"",SUM($K$6:$K$23)),"")</f>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <f>IFERROR(IF($F28="","",IF($H28=0,"",IF($I28="",$H28,$H28*(1+$I28)))),"")</f>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>46317</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="11"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="30">
+        <f>IFERROR(IF($F29="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F29)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F29)),"")</f>
+      </c>
+      <c r="I29" s="31"/>
+      <c r="J29" s="30">
+        <f>IFERROR(IF($F29="","",$K29-$H29),"")</f>
+      </c>
+      <c r="K29" s="30">
+        <f>IFERROR(IF($F29="","",IF($H29=0,"",IF($I29="",$H29,$H29*(1+$I29)))),"")</f>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="32"/>
-      <c r="K31" s="32"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="11"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="30">
+        <f>IFERROR(IF($F30="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F30)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F30)),"")</f>
+      </c>
+      <c r="I30" s="31"/>
+      <c r="J30" s="30">
+        <f>IFERROR(IF($F30="","",$K30-$H30),"")</f>
+      </c>
+      <c r="K30" s="30">
+        <f>IFERROR(IF($F30="","",IF($H30=0,"",IF($I30="",$H30,$H30*(1+$I30)))),"")</f>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="11"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>46317</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
       <c r="D32" s="11"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F32" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="G32" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H32" s="34">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($H$6:$H$30,$G$6:$G$30,"Marta")),"")</f>
+      </c>
+      <c r="I32" s="35">
+        <f>IFERROR(IF($H32=0,"",$J32/$H32),"")</f>
+      </c>
+      <c r="J32" s="34">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($J$6:$J$30,$G$6:$G$30,"Marta")),"")</f>
+      </c>
+      <c r="K32" s="34">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($K$6:$K$30,$G$6:$G$30,"Marta")),"")</f>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>46317</v>
       </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F33" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H33" s="34">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="I33" s="35">
+        <f>IFERROR(IF($H33=0,"",$J33/$H33),"")</f>
+      </c>
+      <c r="J33" s="34">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="K33" s="34">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="9">
         <v>46317</v>
       </c>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="11"/>
+      <c r="F34" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="G34" s="36"/>
+      <c r="H34" s="37">
+        <f>IFERROR(IF(SUM($H$6:$H$30)=0,"",SUM($H$6:$H$30)),"")</f>
+      </c>
+      <c r="I34" s="38">
+        <f>IFERROR(IF($H34=0,"",$J34/$H34),"")</f>
+      </c>
+      <c r="J34" s="37">
+        <f>IFERROR(IF(SUM($J$6:$J$30)=0,"",SUM($J$6:$J$30)),"")</f>
+      </c>
+      <c r="K34" s="37">
+        <f>IFERROR(IF(SUM($K$6:$K$30)=0,"",SUM($K$6:$K$30)),"")</f>
+      </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="9">
@@ -1661,21 +1787,35 @@
       <c r="C35" s="10"/>
       <c r="D35" s="11"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="11"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="11"/>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="39"/>
+      <c r="K36" s="39"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="39"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="39"/>
+      <c r="K37" s="39"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="9">
@@ -1901,7 +2041,3528 @@
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
     </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="11"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="11"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="11"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="11"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="11"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="11"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B72" s="10"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="11"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="11"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="11"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="11"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="11"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="11"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="11"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="11"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B80" s="10"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="11"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="11"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B82" s="10"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="11"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B83" s="10"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="11"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B84" s="10"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="11"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="11"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="11"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B87" s="10"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="11"/>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B88" s="10"/>
+      <c r="C88" s="10"/>
+      <c r="D88" s="11"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B89" s="10"/>
+      <c r="C89" s="10"/>
+      <c r="D89" s="11"/>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B90" s="10"/>
+      <c r="C90" s="10"/>
+      <c r="D90" s="11"/>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B91" s="10"/>
+      <c r="C91" s="10"/>
+      <c r="D91" s="11"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B92" s="10"/>
+      <c r="C92" s="10"/>
+      <c r="D92" s="11"/>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B93" s="10"/>
+      <c r="C93" s="10"/>
+      <c r="D93" s="11"/>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B94" s="10"/>
+      <c r="C94" s="10"/>
+      <c r="D94" s="11"/>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B95" s="10"/>
+      <c r="C95" s="10"/>
+      <c r="D95" s="11"/>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B96" s="10"/>
+      <c r="C96" s="10"/>
+      <c r="D96" s="11"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B97" s="10"/>
+      <c r="C97" s="10"/>
+      <c r="D97" s="11"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B98" s="10"/>
+      <c r="C98" s="10"/>
+      <c r="D98" s="11"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B99" s="10"/>
+      <c r="C99" s="10"/>
+      <c r="D99" s="11"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B100" s="10"/>
+      <c r="C100" s="10"/>
+      <c r="D100" s="11"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B101" s="10"/>
+      <c r="C101" s="10"/>
+      <c r="D101" s="11"/>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B102" s="10"/>
+      <c r="C102" s="10"/>
+      <c r="D102" s="11"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B103" s="10"/>
+      <c r="C103" s="10"/>
+      <c r="D103" s="11"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B104" s="10"/>
+      <c r="C104" s="10"/>
+      <c r="D104" s="11"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B105" s="10"/>
+      <c r="C105" s="10"/>
+      <c r="D105" s="11"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B106" s="10"/>
+      <c r="C106" s="10"/>
+      <c r="D106" s="11"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B107" s="10"/>
+      <c r="C107" s="10"/>
+      <c r="D107" s="11"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B108" s="10"/>
+      <c r="C108" s="10"/>
+      <c r="D108" s="11"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B109" s="10"/>
+      <c r="C109" s="10"/>
+      <c r="D109" s="11"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B110" s="10"/>
+      <c r="C110" s="10"/>
+      <c r="D110" s="11"/>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B111" s="10"/>
+      <c r="C111" s="10"/>
+      <c r="D111" s="11"/>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B112" s="10"/>
+      <c r="C112" s="10"/>
+      <c r="D112" s="11"/>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B113" s="10"/>
+      <c r="C113" s="10"/>
+      <c r="D113" s="11"/>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B114" s="10"/>
+      <c r="C114" s="10"/>
+      <c r="D114" s="11"/>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B115" s="10"/>
+      <c r="C115" s="10"/>
+      <c r="D115" s="11"/>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B116" s="10"/>
+      <c r="C116" s="10"/>
+      <c r="D116" s="11"/>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B117" s="10"/>
+      <c r="C117" s="10"/>
+      <c r="D117" s="11"/>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B118" s="10"/>
+      <c r="C118" s="10"/>
+      <c r="D118" s="11"/>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B119" s="10"/>
+      <c r="C119" s="10"/>
+      <c r="D119" s="11"/>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B120" s="10"/>
+      <c r="C120" s="10"/>
+      <c r="D120" s="11"/>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B121" s="10"/>
+      <c r="C121" s="10"/>
+      <c r="D121" s="11"/>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B122" s="10"/>
+      <c r="C122" s="10"/>
+      <c r="D122" s="11"/>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B123" s="10"/>
+      <c r="C123" s="10"/>
+      <c r="D123" s="11"/>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B124" s="10"/>
+      <c r="C124" s="10"/>
+      <c r="D124" s="11"/>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B125" s="10"/>
+      <c r="C125" s="10"/>
+      <c r="D125" s="11"/>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B126" s="10"/>
+      <c r="C126" s="10"/>
+      <c r="D126" s="11"/>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B127" s="10"/>
+      <c r="C127" s="10"/>
+      <c r="D127" s="11"/>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B128" s="10"/>
+      <c r="C128" s="10"/>
+      <c r="D128" s="11"/>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B129" s="10"/>
+      <c r="C129" s="10"/>
+      <c r="D129" s="11"/>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B130" s="10"/>
+      <c r="C130" s="10"/>
+      <c r="D130" s="11"/>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B131" s="10"/>
+      <c r="C131" s="10"/>
+      <c r="D131" s="11"/>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B132" s="10"/>
+      <c r="C132" s="10"/>
+      <c r="D132" s="11"/>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B133" s="10"/>
+      <c r="C133" s="10"/>
+      <c r="D133" s="11"/>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B134" s="10"/>
+      <c r="C134" s="10"/>
+      <c r="D134" s="11"/>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B135" s="10"/>
+      <c r="C135" s="10"/>
+      <c r="D135" s="11"/>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B136" s="10"/>
+      <c r="C136" s="10"/>
+      <c r="D136" s="11"/>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B137" s="10"/>
+      <c r="C137" s="10"/>
+      <c r="D137" s="11"/>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B138" s="10"/>
+      <c r="C138" s="10"/>
+      <c r="D138" s="11"/>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B139" s="10"/>
+      <c r="C139" s="10"/>
+      <c r="D139" s="11"/>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B140" s="10"/>
+      <c r="C140" s="10"/>
+      <c r="D140" s="11"/>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B141" s="10"/>
+      <c r="C141" s="10"/>
+      <c r="D141" s="11"/>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B142" s="10"/>
+      <c r="C142" s="10"/>
+      <c r="D142" s="11"/>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B143" s="10"/>
+      <c r="C143" s="10"/>
+      <c r="D143" s="11"/>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B144" s="10"/>
+      <c r="C144" s="10"/>
+      <c r="D144" s="11"/>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B145" s="10"/>
+      <c r="C145" s="10"/>
+      <c r="D145" s="11"/>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B146" s="10"/>
+      <c r="C146" s="10"/>
+      <c r="D146" s="11"/>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B147" s="10"/>
+      <c r="C147" s="10"/>
+      <c r="D147" s="11"/>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B148" s="10"/>
+      <c r="C148" s="10"/>
+      <c r="D148" s="11"/>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B149" s="10"/>
+      <c r="C149" s="10"/>
+      <c r="D149" s="11"/>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A150" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B150" s="10"/>
+      <c r="C150" s="10"/>
+      <c r="D150" s="11"/>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B151" s="10"/>
+      <c r="C151" s="10"/>
+      <c r="D151" s="11"/>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A152" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B152" s="10"/>
+      <c r="C152" s="10"/>
+      <c r="D152" s="11"/>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B153" s="10"/>
+      <c r="C153" s="10"/>
+      <c r="D153" s="11"/>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B154" s="10"/>
+      <c r="C154" s="10"/>
+      <c r="D154" s="11"/>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B155" s="10"/>
+      <c r="C155" s="10"/>
+      <c r="D155" s="11"/>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B156" s="10"/>
+      <c r="C156" s="10"/>
+      <c r="D156" s="11"/>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B157" s="10"/>
+      <c r="C157" s="10"/>
+      <c r="D157" s="11"/>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A158" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B158" s="10"/>
+      <c r="C158" s="10"/>
+      <c r="D158" s="11"/>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A159" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B159" s="10"/>
+      <c r="C159" s="10"/>
+      <c r="D159" s="11"/>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B160" s="10"/>
+      <c r="C160" s="10"/>
+      <c r="D160" s="11"/>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B161" s="10"/>
+      <c r="C161" s="10"/>
+      <c r="D161" s="11"/>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A162" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B162" s="10"/>
+      <c r="C162" s="10"/>
+      <c r="D162" s="11"/>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B163" s="10"/>
+      <c r="C163" s="10"/>
+      <c r="D163" s="11"/>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A164" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B164" s="10"/>
+      <c r="C164" s="10"/>
+      <c r="D164" s="11"/>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B165" s="10"/>
+      <c r="C165" s="10"/>
+      <c r="D165" s="11"/>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A166" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B166" s="10"/>
+      <c r="C166" s="10"/>
+      <c r="D166" s="11"/>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A167" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B167" s="10"/>
+      <c r="C167" s="10"/>
+      <c r="D167" s="11"/>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A168" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B168" s="10"/>
+      <c r="C168" s="10"/>
+      <c r="D168" s="11"/>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B169" s="10"/>
+      <c r="C169" s="10"/>
+      <c r="D169" s="11"/>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B170" s="10"/>
+      <c r="C170" s="10"/>
+      <c r="D170" s="11"/>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A171" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B171" s="10"/>
+      <c r="C171" s="10"/>
+      <c r="D171" s="11"/>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A172" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B172" s="10"/>
+      <c r="C172" s="10"/>
+      <c r="D172" s="11"/>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A173" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B173" s="10"/>
+      <c r="C173" s="10"/>
+      <c r="D173" s="11"/>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A174" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B174" s="10"/>
+      <c r="C174" s="10"/>
+      <c r="D174" s="11"/>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A175" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B175" s="10"/>
+      <c r="C175" s="10"/>
+      <c r="D175" s="11"/>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A176" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B176" s="10"/>
+      <c r="C176" s="10"/>
+      <c r="D176" s="11"/>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A177" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B177" s="10"/>
+      <c r="C177" s="10"/>
+      <c r="D177" s="11"/>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B178" s="10"/>
+      <c r="C178" s="10"/>
+      <c r="D178" s="11"/>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B179" s="10"/>
+      <c r="C179" s="10"/>
+      <c r="D179" s="11"/>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B180" s="10"/>
+      <c r="C180" s="10"/>
+      <c r="D180" s="11"/>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B181" s="10"/>
+      <c r="C181" s="10"/>
+      <c r="D181" s="11"/>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B182" s="10"/>
+      <c r="C182" s="10"/>
+      <c r="D182" s="11"/>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B183" s="10"/>
+      <c r="C183" s="10"/>
+      <c r="D183" s="11"/>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B184" s="10"/>
+      <c r="C184" s="10"/>
+      <c r="D184" s="11"/>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B185" s="10"/>
+      <c r="C185" s="10"/>
+      <c r="D185" s="11"/>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A186" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B186" s="10"/>
+      <c r="C186" s="10"/>
+      <c r="D186" s="11"/>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B187" s="10"/>
+      <c r="C187" s="10"/>
+      <c r="D187" s="11"/>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B188" s="10"/>
+      <c r="C188" s="10"/>
+      <c r="D188" s="11"/>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A189" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B189" s="10"/>
+      <c r="C189" s="10"/>
+      <c r="D189" s="11"/>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A190" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B190" s="10"/>
+      <c r="C190" s="10"/>
+      <c r="D190" s="11"/>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A191" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B191" s="10"/>
+      <c r="C191" s="10"/>
+      <c r="D191" s="11"/>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A192" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B192" s="10"/>
+      <c r="C192" s="10"/>
+      <c r="D192" s="11"/>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A193" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B193" s="10"/>
+      <c r="C193" s="10"/>
+      <c r="D193" s="11"/>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A194" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B194" s="10"/>
+      <c r="C194" s="10"/>
+      <c r="D194" s="11"/>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A195" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B195" s="10"/>
+      <c r="C195" s="10"/>
+      <c r="D195" s="11"/>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A196" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B196" s="10"/>
+      <c r="C196" s="10"/>
+      <c r="D196" s="11"/>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A197" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B197" s="10"/>
+      <c r="C197" s="10"/>
+      <c r="D197" s="11"/>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A198" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B198" s="10"/>
+      <c r="C198" s="10"/>
+      <c r="D198" s="11"/>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A199" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B199" s="10"/>
+      <c r="C199" s="10"/>
+      <c r="D199" s="11"/>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A200" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B200" s="10"/>
+      <c r="C200" s="10"/>
+      <c r="D200" s="11"/>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A201" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B201" s="10"/>
+      <c r="C201" s="10"/>
+      <c r="D201" s="11"/>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A202" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B202" s="10"/>
+      <c r="C202" s="10"/>
+      <c r="D202" s="11"/>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A203" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B203" s="10"/>
+      <c r="C203" s="10"/>
+      <c r="D203" s="11"/>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A204" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B204" s="10"/>
+      <c r="C204" s="10"/>
+      <c r="D204" s="11"/>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A205" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B205" s="10"/>
+      <c r="C205" s="10"/>
+      <c r="D205" s="11"/>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A206" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B206" s="10"/>
+      <c r="C206" s="10"/>
+      <c r="D206" s="11"/>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A207" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B207" s="10"/>
+      <c r="C207" s="10"/>
+      <c r="D207" s="11"/>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A208" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B208" s="10"/>
+      <c r="C208" s="10"/>
+      <c r="D208" s="11"/>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A209" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B209" s="10"/>
+      <c r="C209" s="10"/>
+      <c r="D209" s="11"/>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A210" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B210" s="10"/>
+      <c r="C210" s="10"/>
+      <c r="D210" s="11"/>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A211" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B211" s="10"/>
+      <c r="C211" s="10"/>
+      <c r="D211" s="11"/>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A212" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B212" s="10"/>
+      <c r="C212" s="10"/>
+      <c r="D212" s="11"/>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A213" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B213" s="10"/>
+      <c r="C213" s="10"/>
+      <c r="D213" s="11"/>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A214" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B214" s="10"/>
+      <c r="C214" s="10"/>
+      <c r="D214" s="11"/>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A215" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B215" s="10"/>
+      <c r="C215" s="10"/>
+      <c r="D215" s="11"/>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A216" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B216" s="10"/>
+      <c r="C216" s="10"/>
+      <c r="D216" s="11"/>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A217" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B217" s="10"/>
+      <c r="C217" s="10"/>
+      <c r="D217" s="11"/>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A218" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B218" s="10"/>
+      <c r="C218" s="10"/>
+      <c r="D218" s="11"/>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A219" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B219" s="10"/>
+      <c r="C219" s="10"/>
+      <c r="D219" s="11"/>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A220" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B220" s="10"/>
+      <c r="C220" s="10"/>
+      <c r="D220" s="11"/>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A221" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B221" s="10"/>
+      <c r="C221" s="10"/>
+      <c r="D221" s="11"/>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A222" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B222" s="10"/>
+      <c r="C222" s="10"/>
+      <c r="D222" s="11"/>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A223" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B223" s="10"/>
+      <c r="C223" s="10"/>
+      <c r="D223" s="11"/>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A224" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B224" s="10"/>
+      <c r="C224" s="10"/>
+      <c r="D224" s="11"/>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A225" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B225" s="10"/>
+      <c r="C225" s="10"/>
+      <c r="D225" s="11"/>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A226" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B226" s="10"/>
+      <c r="C226" s="10"/>
+      <c r="D226" s="11"/>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A227" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B227" s="10"/>
+      <c r="C227" s="10"/>
+      <c r="D227" s="11"/>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A228" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B228" s="10"/>
+      <c r="C228" s="10"/>
+      <c r="D228" s="11"/>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A229" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B229" s="10"/>
+      <c r="C229" s="10"/>
+      <c r="D229" s="11"/>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A230" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B230" s="10"/>
+      <c r="C230" s="10"/>
+      <c r="D230" s="11"/>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A231" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B231" s="10"/>
+      <c r="C231" s="10"/>
+      <c r="D231" s="11"/>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A232" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B232" s="10"/>
+      <c r="C232" s="10"/>
+      <c r="D232" s="11"/>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A233" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B233" s="10"/>
+      <c r="C233" s="10"/>
+      <c r="D233" s="11"/>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A234" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B234" s="10"/>
+      <c r="C234" s="10"/>
+      <c r="D234" s="11"/>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A235" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B235" s="10"/>
+      <c r="C235" s="10"/>
+      <c r="D235" s="11"/>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A236" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B236" s="10"/>
+      <c r="C236" s="10"/>
+      <c r="D236" s="11"/>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A237" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B237" s="10"/>
+      <c r="C237" s="10"/>
+      <c r="D237" s="11"/>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A238" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B238" s="10"/>
+      <c r="C238" s="10"/>
+      <c r="D238" s="11"/>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A239" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B239" s="10"/>
+      <c r="C239" s="10"/>
+      <c r="D239" s="11"/>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A240" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B240" s="10"/>
+      <c r="C240" s="10"/>
+      <c r="D240" s="11"/>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A241" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B241" s="10"/>
+      <c r="C241" s="10"/>
+      <c r="D241" s="11"/>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A242" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B242" s="10"/>
+      <c r="C242" s="10"/>
+      <c r="D242" s="11"/>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A243" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B243" s="10"/>
+      <c r="C243" s="10"/>
+      <c r="D243" s="11"/>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A244" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B244" s="10"/>
+      <c r="C244" s="10"/>
+      <c r="D244" s="11"/>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A245" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B245" s="10"/>
+      <c r="C245" s="10"/>
+      <c r="D245" s="11"/>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A246" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B246" s="10"/>
+      <c r="C246" s="10"/>
+      <c r="D246" s="11"/>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A247" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B247" s="10"/>
+      <c r="C247" s="10"/>
+      <c r="D247" s="11"/>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A248" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B248" s="10"/>
+      <c r="C248" s="10"/>
+      <c r="D248" s="11"/>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A249" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B249" s="10"/>
+      <c r="C249" s="10"/>
+      <c r="D249" s="11"/>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A250" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B250" s="10"/>
+      <c r="C250" s="10"/>
+      <c r="D250" s="11"/>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A251" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B251" s="10"/>
+      <c r="C251" s="10"/>
+      <c r="D251" s="11"/>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A252" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B252" s="10"/>
+      <c r="C252" s="10"/>
+      <c r="D252" s="11"/>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A253" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B253" s="10"/>
+      <c r="C253" s="10"/>
+      <c r="D253" s="11"/>
+    </row>
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A254" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B254" s="10"/>
+      <c r="C254" s="10"/>
+      <c r="D254" s="11"/>
+    </row>
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A255" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B255" s="10"/>
+      <c r="C255" s="10"/>
+      <c r="D255" s="11"/>
+    </row>
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A256" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B256" s="10"/>
+      <c r="C256" s="10"/>
+      <c r="D256" s="11"/>
+    </row>
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A257" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B257" s="10"/>
+      <c r="C257" s="10"/>
+      <c r="D257" s="11"/>
+    </row>
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A258" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B258" s="10"/>
+      <c r="C258" s="10"/>
+      <c r="D258" s="11"/>
+    </row>
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A259" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B259" s="10"/>
+      <c r="C259" s="10"/>
+      <c r="D259" s="11"/>
+    </row>
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A260" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B260" s="10"/>
+      <c r="C260" s="10"/>
+      <c r="D260" s="11"/>
+    </row>
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A261" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B261" s="10"/>
+      <c r="C261" s="10"/>
+      <c r="D261" s="11"/>
+    </row>
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A262" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B262" s="10"/>
+      <c r="C262" s="10"/>
+      <c r="D262" s="11"/>
+    </row>
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A263" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B263" s="10"/>
+      <c r="C263" s="10"/>
+      <c r="D263" s="11"/>
+    </row>
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A264" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B264" s="10"/>
+      <c r="C264" s="10"/>
+      <c r="D264" s="11"/>
+    </row>
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A265" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B265" s="10"/>
+      <c r="C265" s="10"/>
+      <c r="D265" s="11"/>
+    </row>
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A266" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B266" s="10"/>
+      <c r="C266" s="10"/>
+      <c r="D266" s="11"/>
+    </row>
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A267" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B267" s="10"/>
+      <c r="C267" s="10"/>
+      <c r="D267" s="11"/>
+    </row>
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A268" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B268" s="10"/>
+      <c r="C268" s="10"/>
+      <c r="D268" s="11"/>
+    </row>
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A269" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B269" s="10"/>
+      <c r="C269" s="10"/>
+      <c r="D269" s="11"/>
+    </row>
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A270" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B270" s="10"/>
+      <c r="C270" s="10"/>
+      <c r="D270" s="11"/>
+    </row>
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A271" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B271" s="10"/>
+      <c r="C271" s="10"/>
+      <c r="D271" s="11"/>
+    </row>
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A272" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B272" s="10"/>
+      <c r="C272" s="10"/>
+      <c r="D272" s="11"/>
+    </row>
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A273" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B273" s="10"/>
+      <c r="C273" s="10"/>
+      <c r="D273" s="11"/>
+    </row>
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A274" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B274" s="10"/>
+      <c r="C274" s="10"/>
+      <c r="D274" s="11"/>
+    </row>
+    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A275" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B275" s="10"/>
+      <c r="C275" s="10"/>
+      <c r="D275" s="11"/>
+    </row>
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A276" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B276" s="10"/>
+      <c r="C276" s="10"/>
+      <c r="D276" s="11"/>
+    </row>
+    <row r="277" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A277" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B277" s="10"/>
+      <c r="C277" s="10"/>
+      <c r="D277" s="11"/>
+    </row>
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A278" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B278" s="10"/>
+      <c r="C278" s="10"/>
+      <c r="D278" s="11"/>
+    </row>
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A279" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B279" s="10"/>
+      <c r="C279" s="10"/>
+      <c r="D279" s="11"/>
+    </row>
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A280" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B280" s="10"/>
+      <c r="C280" s="10"/>
+      <c r="D280" s="11"/>
+    </row>
+    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A281" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B281" s="10"/>
+      <c r="C281" s="10"/>
+      <c r="D281" s="11"/>
+    </row>
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A282" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B282" s="10"/>
+      <c r="C282" s="10"/>
+      <c r="D282" s="11"/>
+    </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A283" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B283" s="10"/>
+      <c r="C283" s="10"/>
+      <c r="D283" s="11"/>
+    </row>
+    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A284" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B284" s="10"/>
+      <c r="C284" s="10"/>
+      <c r="D284" s="11"/>
+    </row>
+    <row r="285" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A285" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B285" s="10"/>
+      <c r="C285" s="10"/>
+      <c r="D285" s="11"/>
+    </row>
+    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A286" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B286" s="10"/>
+      <c r="C286" s="10"/>
+      <c r="D286" s="11"/>
+    </row>
+    <row r="287" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A287" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B287" s="10"/>
+      <c r="C287" s="10"/>
+      <c r="D287" s="11"/>
+    </row>
+    <row r="288" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A288" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B288" s="10"/>
+      <c r="C288" s="10"/>
+      <c r="D288" s="11"/>
+    </row>
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A289" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B289" s="10"/>
+      <c r="C289" s="10"/>
+      <c r="D289" s="11"/>
+    </row>
+    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A290" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B290" s="10"/>
+      <c r="C290" s="10"/>
+      <c r="D290" s="11"/>
+    </row>
+    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A291" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B291" s="10"/>
+      <c r="C291" s="10"/>
+      <c r="D291" s="11"/>
+    </row>
+    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A292" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B292" s="10"/>
+      <c r="C292" s="10"/>
+      <c r="D292" s="11"/>
+    </row>
+    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A293" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B293" s="10"/>
+      <c r="C293" s="10"/>
+      <c r="D293" s="11"/>
+    </row>
+    <row r="294" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A294" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B294" s="10"/>
+      <c r="C294" s="10"/>
+      <c r="D294" s="11"/>
+    </row>
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A295" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B295" s="10"/>
+      <c r="C295" s="10"/>
+      <c r="D295" s="11"/>
+    </row>
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A296" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B296" s="10"/>
+      <c r="C296" s="10"/>
+      <c r="D296" s="11"/>
+    </row>
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A297" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B297" s="10"/>
+      <c r="C297" s="10"/>
+      <c r="D297" s="11"/>
+    </row>
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A298" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B298" s="10"/>
+      <c r="C298" s="10"/>
+      <c r="D298" s="11"/>
+    </row>
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A299" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B299" s="10"/>
+      <c r="C299" s="10"/>
+      <c r="D299" s="11"/>
+    </row>
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A300" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B300" s="10"/>
+      <c r="C300" s="10"/>
+      <c r="D300" s="11"/>
+    </row>
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A301" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B301" s="10"/>
+      <c r="C301" s="10"/>
+      <c r="D301" s="11"/>
+    </row>
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A302" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B302" s="10"/>
+      <c r="C302" s="10"/>
+      <c r="D302" s="11"/>
+    </row>
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A303" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B303" s="10"/>
+      <c r="C303" s="10"/>
+      <c r="D303" s="11"/>
+    </row>
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A304" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B304" s="10"/>
+      <c r="C304" s="10"/>
+      <c r="D304" s="11"/>
+    </row>
+    <row r="305" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A305" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B305" s="10"/>
+      <c r="C305" s="10"/>
+      <c r="D305" s="11"/>
+    </row>
+    <row r="306" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A306" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B306" s="10"/>
+      <c r="C306" s="10"/>
+      <c r="D306" s="11"/>
+    </row>
+    <row r="307" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A307" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B307" s="10"/>
+      <c r="C307" s="10"/>
+      <c r="D307" s="11"/>
+    </row>
+    <row r="308" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A308" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B308" s="10"/>
+      <c r="C308" s="10"/>
+      <c r="D308" s="11"/>
+    </row>
+    <row r="309" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A309" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B309" s="10"/>
+      <c r="C309" s="10"/>
+      <c r="D309" s="11"/>
+    </row>
+    <row r="310" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A310" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B310" s="10"/>
+      <c r="C310" s="10"/>
+      <c r="D310" s="11"/>
+    </row>
+    <row r="311" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A311" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B311" s="10"/>
+      <c r="C311" s="10"/>
+      <c r="D311" s="11"/>
+    </row>
+    <row r="312" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A312" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B312" s="10"/>
+      <c r="C312" s="10"/>
+      <c r="D312" s="11"/>
+    </row>
+    <row r="313" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A313" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B313" s="10"/>
+      <c r="C313" s="10"/>
+      <c r="D313" s="11"/>
+    </row>
+    <row r="314" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A314" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B314" s="10"/>
+      <c r="C314" s="10"/>
+      <c r="D314" s="11"/>
+    </row>
+    <row r="315" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A315" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B315" s="10"/>
+      <c r="C315" s="10"/>
+      <c r="D315" s="11"/>
+    </row>
+    <row r="316" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A316" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B316" s="10"/>
+      <c r="C316" s="10"/>
+      <c r="D316" s="11"/>
+    </row>
+    <row r="317" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A317" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B317" s="10"/>
+      <c r="C317" s="10"/>
+      <c r="D317" s="11"/>
+    </row>
+    <row r="318" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A318" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B318" s="10"/>
+      <c r="C318" s="10"/>
+      <c r="D318" s="11"/>
+    </row>
+    <row r="319" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A319" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B319" s="10"/>
+      <c r="C319" s="10"/>
+      <c r="D319" s="11"/>
+    </row>
+    <row r="320" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A320" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B320" s="10"/>
+      <c r="C320" s="10"/>
+      <c r="D320" s="11"/>
+    </row>
+    <row r="321" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A321" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B321" s="10"/>
+      <c r="C321" s="10"/>
+      <c r="D321" s="11"/>
+    </row>
+    <row r="322" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A322" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B322" s="10"/>
+      <c r="C322" s="10"/>
+      <c r="D322" s="11"/>
+    </row>
+    <row r="323" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A323" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B323" s="10"/>
+      <c r="C323" s="10"/>
+      <c r="D323" s="11"/>
+    </row>
+    <row r="324" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A324" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B324" s="10"/>
+      <c r="C324" s="10"/>
+      <c r="D324" s="11"/>
+    </row>
+    <row r="325" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A325" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B325" s="10"/>
+      <c r="C325" s="10"/>
+      <c r="D325" s="11"/>
+    </row>
+    <row r="326" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A326" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B326" s="10"/>
+      <c r="C326" s="10"/>
+      <c r="D326" s="11"/>
+    </row>
+    <row r="327" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A327" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B327" s="10"/>
+      <c r="C327" s="10"/>
+      <c r="D327" s="11"/>
+    </row>
+    <row r="328" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A328" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B328" s="10"/>
+      <c r="C328" s="10"/>
+      <c r="D328" s="11"/>
+    </row>
+    <row r="329" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A329" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B329" s="10"/>
+      <c r="C329" s="10"/>
+      <c r="D329" s="11"/>
+    </row>
+    <row r="330" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A330" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B330" s="10"/>
+      <c r="C330" s="10"/>
+      <c r="D330" s="11"/>
+    </row>
+    <row r="331" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A331" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B331" s="10"/>
+      <c r="C331" s="10"/>
+      <c r="D331" s="11"/>
+    </row>
+    <row r="332" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A332" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B332" s="10"/>
+      <c r="C332" s="10"/>
+      <c r="D332" s="11"/>
+    </row>
+    <row r="333" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A333" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B333" s="10"/>
+      <c r="C333" s="10"/>
+      <c r="D333" s="11"/>
+    </row>
+    <row r="334" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A334" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B334" s="10"/>
+      <c r="C334" s="10"/>
+      <c r="D334" s="11"/>
+    </row>
+    <row r="335" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A335" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B335" s="10"/>
+      <c r="C335" s="10"/>
+      <c r="D335" s="11"/>
+    </row>
+    <row r="336" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A336" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B336" s="10"/>
+      <c r="C336" s="10"/>
+      <c r="D336" s="11"/>
+    </row>
+    <row r="337" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A337" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B337" s="10"/>
+      <c r="C337" s="10"/>
+      <c r="D337" s="11"/>
+    </row>
+    <row r="338" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A338" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B338" s="10"/>
+      <c r="C338" s="10"/>
+      <c r="D338" s="11"/>
+    </row>
+    <row r="339" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A339" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B339" s="10"/>
+      <c r="C339" s="10"/>
+      <c r="D339" s="11"/>
+    </row>
+    <row r="340" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A340" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B340" s="10"/>
+      <c r="C340" s="10"/>
+      <c r="D340" s="11"/>
+    </row>
+    <row r="341" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A341" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B341" s="10"/>
+      <c r="C341" s="10"/>
+      <c r="D341" s="11"/>
+    </row>
+    <row r="342" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A342" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B342" s="10"/>
+      <c r="C342" s="10"/>
+      <c r="D342" s="11"/>
+    </row>
+    <row r="343" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A343" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B343" s="10"/>
+      <c r="C343" s="10"/>
+      <c r="D343" s="11"/>
+    </row>
+    <row r="344" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A344" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B344" s="10"/>
+      <c r="C344" s="10"/>
+      <c r="D344" s="11"/>
+    </row>
+    <row r="345" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A345" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B345" s="10"/>
+      <c r="C345" s="10"/>
+      <c r="D345" s="11"/>
+    </row>
+    <row r="346" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A346" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B346" s="10"/>
+      <c r="C346" s="10"/>
+      <c r="D346" s="11"/>
+    </row>
+    <row r="347" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A347" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B347" s="10"/>
+      <c r="C347" s="10"/>
+      <c r="D347" s="11"/>
+    </row>
+    <row r="348" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A348" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B348" s="10"/>
+      <c r="C348" s="10"/>
+      <c r="D348" s="11"/>
+    </row>
+    <row r="349" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A349" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B349" s="10"/>
+      <c r="C349" s="10"/>
+      <c r="D349" s="11"/>
+    </row>
+    <row r="350" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A350" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B350" s="10"/>
+      <c r="C350" s="10"/>
+      <c r="D350" s="11"/>
+    </row>
+    <row r="351" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A351" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B351" s="10"/>
+      <c r="C351" s="10"/>
+      <c r="D351" s="11"/>
+    </row>
+    <row r="352" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A352" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B352" s="10"/>
+      <c r="C352" s="10"/>
+      <c r="D352" s="11"/>
+    </row>
+    <row r="353" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A353" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B353" s="10"/>
+      <c r="C353" s="10"/>
+      <c r="D353" s="11"/>
+    </row>
+    <row r="354" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A354" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B354" s="10"/>
+      <c r="C354" s="10"/>
+      <c r="D354" s="11"/>
+    </row>
+    <row r="355" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A355" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B355" s="10"/>
+      <c r="C355" s="10"/>
+      <c r="D355" s="11"/>
+    </row>
+    <row r="356" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A356" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B356" s="10"/>
+      <c r="C356" s="10"/>
+      <c r="D356" s="11"/>
+    </row>
+    <row r="357" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A357" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B357" s="10"/>
+      <c r="C357" s="10"/>
+      <c r="D357" s="11"/>
+    </row>
+    <row r="358" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A358" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B358" s="10"/>
+      <c r="C358" s="10"/>
+      <c r="D358" s="11"/>
+    </row>
+    <row r="359" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A359" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B359" s="10"/>
+      <c r="C359" s="10"/>
+      <c r="D359" s="11"/>
+    </row>
+    <row r="360" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A360" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B360" s="10"/>
+      <c r="C360" s="10"/>
+      <c r="D360" s="11"/>
+    </row>
+    <row r="361" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A361" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B361" s="10"/>
+      <c r="C361" s="10"/>
+      <c r="D361" s="11"/>
+    </row>
+    <row r="362" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A362" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B362" s="10"/>
+      <c r="C362" s="10"/>
+      <c r="D362" s="11"/>
+    </row>
+    <row r="363" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A363" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B363" s="10"/>
+      <c r="C363" s="10"/>
+      <c r="D363" s="11"/>
+    </row>
+    <row r="364" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A364" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B364" s="10"/>
+      <c r="C364" s="10"/>
+      <c r="D364" s="11"/>
+    </row>
+    <row r="365" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A365" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B365" s="10"/>
+      <c r="C365" s="10"/>
+      <c r="D365" s="11"/>
+    </row>
+    <row r="366" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A366" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B366" s="10"/>
+      <c r="C366" s="10"/>
+      <c r="D366" s="11"/>
+    </row>
+    <row r="367" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A367" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B367" s="10"/>
+      <c r="C367" s="10"/>
+      <c r="D367" s="11"/>
+    </row>
+    <row r="368" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A368" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B368" s="10"/>
+      <c r="C368" s="10"/>
+      <c r="D368" s="11"/>
+    </row>
+    <row r="369" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A369" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B369" s="10"/>
+      <c r="C369" s="10"/>
+      <c r="D369" s="11"/>
+    </row>
+    <row r="370" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A370" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B370" s="10"/>
+      <c r="C370" s="10"/>
+      <c r="D370" s="11"/>
+    </row>
+    <row r="371" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A371" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B371" s="10"/>
+      <c r="C371" s="10"/>
+      <c r="D371" s="11"/>
+    </row>
+    <row r="372" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A372" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B372" s="10"/>
+      <c r="C372" s="10"/>
+      <c r="D372" s="11"/>
+    </row>
+    <row r="373" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A373" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B373" s="10"/>
+      <c r="C373" s="10"/>
+      <c r="D373" s="11"/>
+    </row>
+    <row r="374" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A374" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B374" s="10"/>
+      <c r="C374" s="10"/>
+      <c r="D374" s="11"/>
+    </row>
+    <row r="375" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A375" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B375" s="10"/>
+      <c r="C375" s="10"/>
+      <c r="D375" s="11"/>
+    </row>
+    <row r="376" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A376" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B376" s="10"/>
+      <c r="C376" s="10"/>
+      <c r="D376" s="11"/>
+    </row>
+    <row r="377" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A377" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B377" s="10"/>
+      <c r="C377" s="10"/>
+      <c r="D377" s="11"/>
+    </row>
+    <row r="378" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A378" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B378" s="10"/>
+      <c r="C378" s="10"/>
+      <c r="D378" s="11"/>
+    </row>
+    <row r="379" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A379" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B379" s="10"/>
+      <c r="C379" s="10"/>
+      <c r="D379" s="11"/>
+    </row>
+    <row r="380" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A380" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B380" s="10"/>
+      <c r="C380" s="10"/>
+      <c r="D380" s="11"/>
+    </row>
+    <row r="381" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A381" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B381" s="10"/>
+      <c r="C381" s="10"/>
+      <c r="D381" s="11"/>
+    </row>
+    <row r="382" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A382" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B382" s="10"/>
+      <c r="C382" s="10"/>
+      <c r="D382" s="11"/>
+    </row>
+    <row r="383" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A383" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B383" s="10"/>
+      <c r="C383" s="10"/>
+      <c r="D383" s="11"/>
+    </row>
+    <row r="384" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A384" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B384" s="10"/>
+      <c r="C384" s="10"/>
+      <c r="D384" s="11"/>
+    </row>
+    <row r="385" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A385" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B385" s="10"/>
+      <c r="C385" s="10"/>
+      <c r="D385" s="11"/>
+    </row>
+    <row r="386" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A386" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B386" s="10"/>
+      <c r="C386" s="10"/>
+      <c r="D386" s="11"/>
+    </row>
+    <row r="387" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A387" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B387" s="10"/>
+      <c r="C387" s="10"/>
+      <c r="D387" s="11"/>
+    </row>
+    <row r="388" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A388" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B388" s="10"/>
+      <c r="C388" s="10"/>
+      <c r="D388" s="11"/>
+    </row>
+    <row r="389" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A389" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B389" s="10"/>
+      <c r="C389" s="10"/>
+      <c r="D389" s="11"/>
+    </row>
+    <row r="390" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A390" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B390" s="10"/>
+      <c r="C390" s="10"/>
+      <c r="D390" s="11"/>
+    </row>
+    <row r="391" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A391" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B391" s="10"/>
+      <c r="C391" s="10"/>
+      <c r="D391" s="11"/>
+    </row>
+    <row r="392" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A392" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B392" s="10"/>
+      <c r="C392" s="10"/>
+      <c r="D392" s="11"/>
+    </row>
+    <row r="393" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A393" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B393" s="10"/>
+      <c r="C393" s="10"/>
+      <c r="D393" s="11"/>
+    </row>
+    <row r="394" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A394" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B394" s="10"/>
+      <c r="C394" s="10"/>
+      <c r="D394" s="11"/>
+    </row>
+    <row r="395" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A395" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B395" s="10"/>
+      <c r="C395" s="10"/>
+      <c r="D395" s="11"/>
+    </row>
+    <row r="396" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A396" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B396" s="10"/>
+      <c r="C396" s="10"/>
+      <c r="D396" s="11"/>
+    </row>
+    <row r="397" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A397" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B397" s="10"/>
+      <c r="C397" s="10"/>
+      <c r="D397" s="11"/>
+    </row>
+    <row r="398" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A398" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B398" s="10"/>
+      <c r="C398" s="10"/>
+      <c r="D398" s="11"/>
+    </row>
+    <row r="399" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A399" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B399" s="10"/>
+      <c r="C399" s="10"/>
+      <c r="D399" s="11"/>
+    </row>
+    <row r="400" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A400" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B400" s="10"/>
+      <c r="C400" s="10"/>
+      <c r="D400" s="11"/>
+    </row>
+    <row r="401" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A401" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B401" s="10"/>
+      <c r="C401" s="10"/>
+      <c r="D401" s="11"/>
+    </row>
+    <row r="402" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A402" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B402" s="10"/>
+      <c r="C402" s="10"/>
+      <c r="D402" s="11"/>
+    </row>
+    <row r="403" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A403" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B403" s="10"/>
+      <c r="C403" s="10"/>
+      <c r="D403" s="11"/>
+    </row>
+    <row r="404" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A404" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B404" s="10"/>
+      <c r="C404" s="10"/>
+      <c r="D404" s="11"/>
+    </row>
+    <row r="405" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A405" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B405" s="10"/>
+      <c r="C405" s="10"/>
+      <c r="D405" s="11"/>
+    </row>
+    <row r="406" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A406" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B406" s="10"/>
+      <c r="C406" s="10"/>
+      <c r="D406" s="11"/>
+    </row>
+    <row r="407" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A407" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B407" s="10"/>
+      <c r="C407" s="10"/>
+      <c r="D407" s="11"/>
+    </row>
+    <row r="408" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A408" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B408" s="10"/>
+      <c r="C408" s="10"/>
+      <c r="D408" s="11"/>
+    </row>
+    <row r="409" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A409" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B409" s="10"/>
+      <c r="C409" s="10"/>
+      <c r="D409" s="11"/>
+    </row>
+    <row r="410" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A410" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B410" s="10"/>
+      <c r="C410" s="10"/>
+      <c r="D410" s="11"/>
+    </row>
+    <row r="411" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A411" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B411" s="10"/>
+      <c r="C411" s="10"/>
+      <c r="D411" s="11"/>
+    </row>
+    <row r="412" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A412" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B412" s="10"/>
+      <c r="C412" s="10"/>
+      <c r="D412" s="11"/>
+    </row>
+    <row r="413" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A413" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B413" s="10"/>
+      <c r="C413" s="10"/>
+      <c r="D413" s="11"/>
+    </row>
+    <row r="414" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A414" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B414" s="10"/>
+      <c r="C414" s="10"/>
+      <c r="D414" s="11"/>
+    </row>
+    <row r="415" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A415" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B415" s="10"/>
+      <c r="C415" s="10"/>
+      <c r="D415" s="11"/>
+    </row>
+    <row r="416" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A416" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B416" s="10"/>
+      <c r="C416" s="10"/>
+      <c r="D416" s="11"/>
+    </row>
+    <row r="417" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A417" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B417" s="10"/>
+      <c r="C417" s="10"/>
+      <c r="D417" s="11"/>
+    </row>
+    <row r="418" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A418" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B418" s="10"/>
+      <c r="C418" s="10"/>
+      <c r="D418" s="11"/>
+    </row>
+    <row r="419" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A419" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B419" s="10"/>
+      <c r="C419" s="10"/>
+      <c r="D419" s="11"/>
+    </row>
+    <row r="420" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A420" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B420" s="10"/>
+      <c r="C420" s="10"/>
+      <c r="D420" s="11"/>
+    </row>
+    <row r="421" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A421" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B421" s="10"/>
+      <c r="C421" s="10"/>
+      <c r="D421" s="11"/>
+    </row>
+    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A422" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B422" s="10"/>
+      <c r="C422" s="10"/>
+      <c r="D422" s="11"/>
+    </row>
+    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A423" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B423" s="10"/>
+      <c r="C423" s="10"/>
+      <c r="D423" s="11"/>
+    </row>
+    <row r="424" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A424" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B424" s="10"/>
+      <c r="C424" s="10"/>
+      <c r="D424" s="11"/>
+    </row>
+    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A425" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B425" s="10"/>
+      <c r="C425" s="10"/>
+      <c r="D425" s="11"/>
+    </row>
+    <row r="426" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A426" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B426" s="10"/>
+      <c r="C426" s="10"/>
+      <c r="D426" s="11"/>
+    </row>
+    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A427" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B427" s="10"/>
+      <c r="C427" s="10"/>
+      <c r="D427" s="11"/>
+    </row>
+    <row r="428" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A428" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B428" s="10"/>
+      <c r="C428" s="10"/>
+      <c r="D428" s="11"/>
+    </row>
+    <row r="429" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A429" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B429" s="10"/>
+      <c r="C429" s="10"/>
+      <c r="D429" s="11"/>
+    </row>
+    <row r="430" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A430" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B430" s="10"/>
+      <c r="C430" s="10"/>
+      <c r="D430" s="11"/>
+    </row>
+    <row r="431" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A431" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B431" s="10"/>
+      <c r="C431" s="10"/>
+      <c r="D431" s="11"/>
+    </row>
+    <row r="432" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A432" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B432" s="10"/>
+      <c r="C432" s="10"/>
+      <c r="D432" s="11"/>
+    </row>
+    <row r="433" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A433" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B433" s="10"/>
+      <c r="C433" s="10"/>
+      <c r="D433" s="11"/>
+    </row>
+    <row r="434" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A434" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B434" s="10"/>
+      <c r="C434" s="10"/>
+      <c r="D434" s="11"/>
+    </row>
+    <row r="435" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A435" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B435" s="10"/>
+      <c r="C435" s="10"/>
+      <c r="D435" s="11"/>
+    </row>
+    <row r="436" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A436" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B436" s="10"/>
+      <c r="C436" s="10"/>
+      <c r="D436" s="11"/>
+    </row>
+    <row r="437" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A437" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B437" s="10"/>
+      <c r="C437" s="10"/>
+      <c r="D437" s="11"/>
+    </row>
+    <row r="438" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A438" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B438" s="10"/>
+      <c r="C438" s="10"/>
+      <c r="D438" s="11"/>
+    </row>
+    <row r="439" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A439" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B439" s="10"/>
+      <c r="C439" s="10"/>
+      <c r="D439" s="11"/>
+    </row>
+    <row r="440" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A440" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B440" s="10"/>
+      <c r="C440" s="10"/>
+      <c r="D440" s="11"/>
+    </row>
+    <row r="441" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A441" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B441" s="10"/>
+      <c r="C441" s="10"/>
+      <c r="D441" s="11"/>
+    </row>
+    <row r="442" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A442" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B442" s="10"/>
+      <c r="C442" s="10"/>
+      <c r="D442" s="11"/>
+    </row>
+    <row r="443" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A443" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B443" s="10"/>
+      <c r="C443" s="10"/>
+      <c r="D443" s="11"/>
+    </row>
+    <row r="444" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A444" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B444" s="10"/>
+      <c r="C444" s="10"/>
+      <c r="D444" s="11"/>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A445" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B445" s="10"/>
+      <c r="C445" s="10"/>
+      <c r="D445" s="11"/>
+    </row>
+    <row r="446" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A446" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B446" s="10"/>
+      <c r="C446" s="10"/>
+      <c r="D446" s="11"/>
+    </row>
+    <row r="447" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A447" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B447" s="10"/>
+      <c r="C447" s="10"/>
+      <c r="D447" s="11"/>
+    </row>
+    <row r="448" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A448" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B448" s="10"/>
+      <c r="C448" s="10"/>
+      <c r="D448" s="11"/>
+    </row>
+    <row r="449" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A449" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B449" s="10"/>
+      <c r="C449" s="10"/>
+      <c r="D449" s="11"/>
+    </row>
+    <row r="450" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A450" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B450" s="10"/>
+      <c r="C450" s="10"/>
+      <c r="D450" s="11"/>
+    </row>
+    <row r="451" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A451" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B451" s="10"/>
+      <c r="C451" s="10"/>
+      <c r="D451" s="11"/>
+    </row>
+    <row r="452" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A452" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B452" s="10"/>
+      <c r="C452" s="10"/>
+      <c r="D452" s="11"/>
+    </row>
+    <row r="453" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A453" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B453" s="10"/>
+      <c r="C453" s="10"/>
+      <c r="D453" s="11"/>
+    </row>
+    <row r="454" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A454" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B454" s="10"/>
+      <c r="C454" s="10"/>
+      <c r="D454" s="11"/>
+    </row>
+    <row r="455" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A455" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B455" s="10"/>
+      <c r="C455" s="10"/>
+      <c r="D455" s="11"/>
+    </row>
+    <row r="456" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A456" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B456" s="10"/>
+      <c r="C456" s="10"/>
+      <c r="D456" s="11"/>
+    </row>
+    <row r="457" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A457" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B457" s="10"/>
+      <c r="C457" s="10"/>
+      <c r="D457" s="11"/>
+    </row>
+    <row r="458" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A458" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B458" s="10"/>
+      <c r="C458" s="10"/>
+      <c r="D458" s="11"/>
+    </row>
+    <row r="459" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A459" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B459" s="10"/>
+      <c r="C459" s="10"/>
+      <c r="D459" s="11"/>
+    </row>
+    <row r="460" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A460" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B460" s="10"/>
+      <c r="C460" s="10"/>
+      <c r="D460" s="11"/>
+    </row>
+    <row r="461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A461" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B461" s="10"/>
+      <c r="C461" s="10"/>
+      <c r="D461" s="11"/>
+    </row>
+    <row r="462" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A462" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B462" s="10"/>
+      <c r="C462" s="10"/>
+      <c r="D462" s="11"/>
+    </row>
+    <row r="463" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A463" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B463" s="10"/>
+      <c r="C463" s="10"/>
+      <c r="D463" s="11"/>
+    </row>
+    <row r="464" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A464" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B464" s="10"/>
+      <c r="C464" s="10"/>
+      <c r="D464" s="11"/>
+    </row>
+    <row r="465" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A465" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B465" s="10"/>
+      <c r="C465" s="10"/>
+      <c r="D465" s="11"/>
+    </row>
+    <row r="466" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A466" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B466" s="10"/>
+      <c r="C466" s="10"/>
+      <c r="D466" s="11"/>
+    </row>
+    <row r="467" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A467" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B467" s="10"/>
+      <c r="C467" s="10"/>
+      <c r="D467" s="11"/>
+    </row>
+    <row r="468" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A468" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B468" s="10"/>
+      <c r="C468" s="10"/>
+      <c r="D468" s="11"/>
+    </row>
+    <row r="469" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A469" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B469" s="10"/>
+      <c r="C469" s="10"/>
+      <c r="D469" s="11"/>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A470" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B470" s="10"/>
+      <c r="C470" s="10"/>
+      <c r="D470" s="11"/>
+    </row>
+    <row r="471" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A471" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B471" s="10"/>
+      <c r="C471" s="10"/>
+      <c r="D471" s="11"/>
+    </row>
+    <row r="472" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A472" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B472" s="10"/>
+      <c r="C472" s="10"/>
+      <c r="D472" s="11"/>
+    </row>
+    <row r="473" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A473" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B473" s="10"/>
+      <c r="C473" s="10"/>
+      <c r="D473" s="11"/>
+    </row>
+    <row r="474" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A474" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B474" s="10"/>
+      <c r="C474" s="10"/>
+      <c r="D474" s="11"/>
+    </row>
+    <row r="475" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A475" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B475" s="10"/>
+      <c r="C475" s="10"/>
+      <c r="D475" s="11"/>
+    </row>
+    <row r="476" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A476" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B476" s="10"/>
+      <c r="C476" s="10"/>
+      <c r="D476" s="11"/>
+    </row>
+    <row r="477" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A477" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B477" s="10"/>
+      <c r="C477" s="10"/>
+      <c r="D477" s="11"/>
+    </row>
+    <row r="478" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A478" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B478" s="10"/>
+      <c r="C478" s="10"/>
+      <c r="D478" s="11"/>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B479" s="10"/>
+      <c r="C479" s="10"/>
+      <c r="D479" s="11"/>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B480" s="10"/>
+      <c r="C480" s="10"/>
+      <c r="D480" s="11"/>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B481" s="10"/>
+      <c r="C481" s="10"/>
+      <c r="D481" s="11"/>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B482" s="10"/>
+      <c r="C482" s="10"/>
+      <c r="D482" s="11"/>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B483" s="10"/>
+      <c r="C483" s="10"/>
+      <c r="D483" s="11"/>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B484" s="10"/>
+      <c r="C484" s="10"/>
+      <c r="D484" s="11"/>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B485" s="10"/>
+      <c r="C485" s="10"/>
+      <c r="D485" s="11"/>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B486" s="10"/>
+      <c r="C486" s="10"/>
+      <c r="D486" s="11"/>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B487" s="10"/>
+      <c r="C487" s="10"/>
+      <c r="D487" s="11"/>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B488" s="10"/>
+      <c r="C488" s="10"/>
+      <c r="D488" s="11"/>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B489" s="10"/>
+      <c r="C489" s="10"/>
+      <c r="D489" s="11"/>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B490" s="10"/>
+      <c r="C490" s="10"/>
+      <c r="D490" s="11"/>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B491" s="10"/>
+      <c r="C491" s="10"/>
+      <c r="D491" s="11"/>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A492" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B492" s="10"/>
+      <c r="C492" s="10"/>
+      <c r="D492" s="11"/>
+    </row>
+    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A493" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B493" s="10"/>
+      <c r="C493" s="10"/>
+      <c r="D493" s="11"/>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A494" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B494" s="10"/>
+      <c r="C494" s="10"/>
+      <c r="D494" s="11"/>
+    </row>
+    <row r="495" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A495" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B495" s="10"/>
+      <c r="C495" s="10"/>
+      <c r="D495" s="11"/>
+    </row>
+    <row r="496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A496" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B496" s="10"/>
+      <c r="C496" s="10"/>
+      <c r="D496" s="11"/>
+    </row>
+    <row r="497" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A497" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B497" s="10"/>
+      <c r="C497" s="10"/>
+      <c r="D497" s="11"/>
+    </row>
+    <row r="498" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A498" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B498" s="10"/>
+      <c r="C498" s="10"/>
+      <c r="D498" s="11"/>
+    </row>
+    <row r="499" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A499" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B499" s="10"/>
+      <c r="C499" s="10"/>
+      <c r="D499" s="11"/>
+    </row>
+    <row r="500" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A500" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B500" s="10"/>
+      <c r="C500" s="10"/>
+      <c r="D500" s="11"/>
+    </row>
+    <row r="501" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A501" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B501" s="10"/>
+      <c r="C501" s="10"/>
+      <c r="D501" s="11"/>
+    </row>
+    <row r="502" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A502" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B502" s="10"/>
+      <c r="C502" s="10"/>
+      <c r="D502" s="11"/>
+    </row>
+    <row r="503" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A503" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B503" s="10"/>
+      <c r="C503" s="10"/>
+      <c r="D503" s="11"/>
+    </row>
+    <row r="504" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A504" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B504" s="10"/>
+      <c r="C504" s="10"/>
+      <c r="D504" s="11"/>
+    </row>
+    <row r="505" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A505" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B505" s="10"/>
+      <c r="C505" s="10"/>
+      <c r="D505" s="11"/>
+    </row>
   </sheetData>
+  <sheetProtection sheet="1"/>
   <mergeCells count="8">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:D3"/>
@@ -1909,10 +5570,10 @@
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:K4"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A37:K37"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:D65">
+  <conditionalFormatting sqref="A6:D505">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($D5&lt;&gt;"",$D6="")</formula>
     </cfRule>
@@ -1923,30 +5584,49 @@
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F23">
-    <cfRule type="expression" dxfId="3" priority="6">
+  <conditionalFormatting sqref="F16:K30">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$F16&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>AND($F15&lt;&gt;"",$F16="")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>$F15=""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I16:I30">
+    <cfRule type="expression" dxfId="6" priority="4">
+      <formula>$F16&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="5">
+      <formula>AND($F15&lt;&gt;"",$F16="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9:F30">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J23">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="I6:J30">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="B6:B65">
+    <dataValidation type="list" allowBlank="1" sqref="B6:B505">
       <formula1>ListaNombres</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C6:C65">
+    <dataValidation type="list" allowBlank="1" sqref="C6:C505">
       <formula1>ListaNombres</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" sqref="D6:D65">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" sqref="D6:D505">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
El Excel: gráfico visible, nombres repetidos distintos, Myinvestor → Cuenta Myinvestor, una fila de separación y poder borrar filas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -7,8 +7,8 @@
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$30),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O50</definedName>
+    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$17),1),1)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -499,23 +499,26 @@
   <c:chart>
     <c:title>
       <c:tx>
-        <c:v>Aportado neto y beneficio / pérdida por titular</c:v>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="334155"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000"/>
+              <a:t>Aportado neto y beneficio / pérdida por titular</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
       </c:tx>
       <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -562,7 +565,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$32:$H$33</c:f>
+              <c:f>Movimientos!$H$19:$H$20</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -604,7 +607,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$32:$J$33</c:f>
+              <c:f>Movimientos!$J$19:$J$20</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -687,13 +690,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1435,25 +1438,13 @@
         <f>IFERROR(IF($F17="","",IF($H17=0,"",IF($I17="",$H17,$H17*(1+$I17)))),"")</f>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>46317</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="30">
-        <f>IFERROR(IF($F18="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18)),"")</f>
-      </c>
-      <c r="I18" s="31"/>
-      <c r="J18" s="30">
-        <f>IFERROR(IF($F18="","",$K18-$H18),"")</f>
-      </c>
-      <c r="K18" s="30">
-        <f>IFERROR(IF($F18="","",IF($H18=0,"",IF($I18="",$H18,$H18*(1+$I18)))),"")</f>
-      </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
@@ -1462,17 +1453,23 @@
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="30">
-        <f>IFERROR(IF($F19="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19)),"")</f>
-      </c>
-      <c r="I19" s="31"/>
-      <c r="J19" s="30">
-        <f>IFERROR(IF($F19="","",$K19-$H19),"")</f>
-      </c>
-      <c r="K19" s="30">
-        <f>IFERROR(IF($F19="","",IF($H19=0,"",IF($I19="",$H19,$H19*(1+$I19)))),"")</f>
+      <c r="F19" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" s="34">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")),"")</f>
+      </c>
+      <c r="I19" s="35">
+        <f>IFERROR(IF($H19=0,"",$J19/$H19),"")</f>
+      </c>
+      <c r="J19" s="34">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($J$6:$J$17,$G$6:$G$17,"Marta")),"")</f>
+      </c>
+      <c r="K19" s="34">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($K$6:$K$17,$G$6:$G$17,"Marta")),"")</f>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1482,218 +1479,134 @@
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="11"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="30">
-        <f>IFERROR(IF($F20="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F20)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F20)),"")</f>
-      </c>
-      <c r="I20" s="31"/>
-      <c r="J20" s="30">
-        <f>IFERROR(IF($F20="","",$K20-$H20),"")</f>
-      </c>
-      <c r="K20" s="30">
-        <f>IFERROR(IF($F20="","",IF($H20=0,"",IF($I20="",$H20,$H20*(1+$I20)))),"")</f>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F20" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="34">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="I20" s="35">
+        <f>IFERROR(IF($H20=0,"",$J20/$H20),"")</f>
+      </c>
+      <c r="J20" s="34">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="K20" s="34">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>46317</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="30">
-        <f>IFERROR(IF($F21="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F21)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F21)),"")</f>
-      </c>
-      <c r="I21" s="31"/>
-      <c r="J21" s="30">
-        <f>IFERROR(IF($F21="","",$K21-$H21),"")</f>
-      </c>
-      <c r="K21" s="30">
-        <f>IFERROR(IF($F21="","",IF($H21=0,"",IF($I21="",$H21,$H21*(1+$I21)))),"")</f>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F21" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="G21" s="36"/>
+      <c r="H21" s="37">
+        <f>IFERROR(IF(SUM($H$6:$H$17)=0,"",SUM($H$6:$H$17)),"")</f>
+      </c>
+      <c r="I21" s="38">
+        <f>IFERROR(IF($H21=0,"",$J21/$H21),"")</f>
+      </c>
+      <c r="J21" s="37">
+        <f>IFERROR(IF(SUM($J$6:$J$17)=0,"",SUM($J$6:$J$17)),"")</f>
+      </c>
+      <c r="K21" s="37">
+        <f>IFERROR(IF(SUM($K$6:$K$17)=0,"",SUM($K$6:$K$17)),"")</f>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>46317</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="30">
-        <f>IFERROR(IF($F22="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F22)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F22)),"")</f>
-      </c>
-      <c r="I22" s="31"/>
-      <c r="J22" s="30">
-        <f>IFERROR(IF($F22="","",$K22-$H22),"")</f>
-      </c>
-      <c r="K22" s="30">
-        <f>IFERROR(IF($F22="","",IF($H22=0,"",IF($I22="",$H22,$H22*(1+$I22)))),"")</f>
-      </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="30">
-        <f>IFERROR(IF($F23="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F23)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F23)),"")</f>
-      </c>
-      <c r="I23" s="31"/>
-      <c r="J23" s="30">
-        <f>IFERROR(IF($F23="","",$K23-$H23),"")</f>
-      </c>
-      <c r="K23" s="30">
-        <f>IFERROR(IF($F23="","",IF($H23=0,"",IF($I23="",$H23,$H23*(1+$I23)))),"")</f>
-      </c>
+      <c r="A23" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="39"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="29"/>
-      <c r="H24" s="30">
-        <f>IFERROR(IF($F24="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F24)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F24)),"")</f>
-      </c>
-      <c r="I24" s="31"/>
-      <c r="J24" s="30">
-        <f>IFERROR(IF($F24="","",$K24-$H24),"")</f>
-      </c>
-      <c r="K24" s="30">
-        <f>IFERROR(IF($F24="","",IF($H24=0,"",IF($I24="",$H24,$H24*(1+$I24)))),"")</f>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="39"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="39"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>46317</v>
       </c>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="11"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="30">
-        <f>IFERROR(IF($F25="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F25)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F25)),"")</f>
-      </c>
-      <c r="I25" s="31"/>
-      <c r="J25" s="30">
-        <f>IFERROR(IF($F25="","",$K25-$H25),"")</f>
-      </c>
-      <c r="K25" s="30">
-        <f>IFERROR(IF($F25="","",IF($H25=0,"",IF($I25="",$H25,$H25*(1+$I25)))),"")</f>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>46317</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="30">
-        <f>IFERROR(IF($F26="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F26)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F26)),"")</f>
-      </c>
-      <c r="I26" s="31"/>
-      <c r="J26" s="30">
-        <f>IFERROR(IF($F26="","",$K26-$H26),"")</f>
-      </c>
-      <c r="K26" s="30">
-        <f>IFERROR(IF($F26="","",IF($H26=0,"",IF($I26="",$H26,$H26*(1+$I26)))),"")</f>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>46317</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="11"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="30">
-        <f>IFERROR(IF($F27="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F27)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F27)),"")</f>
-      </c>
-      <c r="I27" s="31"/>
-      <c r="J27" s="30">
-        <f>IFERROR(IF($F27="","",$K27-$H27),"")</f>
-      </c>
-      <c r="K27" s="30">
-        <f>IFERROR(IF($F27="","",IF($H27=0,"",IF($I27="",$H27,$H27*(1+$I27)))),"")</f>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>46317</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="11"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="30">
-        <f>IFERROR(IF($F28="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F28)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F28)),"")</f>
-      </c>
-      <c r="I28" s="31"/>
-      <c r="J28" s="30">
-        <f>IFERROR(IF($F28="","",$K28-$H28),"")</f>
-      </c>
-      <c r="K28" s="30">
-        <f>IFERROR(IF($F28="","",IF($H28=0,"",IF($I28="",$H28,$H28*(1+$I28)))),"")</f>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>46317</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="11"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="30">
-        <f>IFERROR(IF($F29="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F29)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F29)),"")</f>
-      </c>
-      <c r="I29" s="31"/>
-      <c r="J29" s="30">
-        <f>IFERROR(IF($F29="","",$K29-$H29),"")</f>
-      </c>
-      <c r="K29" s="30">
-        <f>IFERROR(IF($F29="","",IF($H29=0,"",IF($I29="",$H29,$H29*(1+$I29)))),"")</f>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="9">
         <v>46317</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="11"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="30">
-        <f>IFERROR(IF($F30="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F30)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F30)),"")</f>
-      </c>
-      <c r="I30" s="31"/>
-      <c r="J30" s="30">
-        <f>IFERROR(IF($F30="","",$K30-$H30),"")</f>
-      </c>
-      <c r="K30" s="30">
-        <f>IFERROR(IF($F30="","",IF($H30=0,"",IF($I30="",$H30,$H30*(1+$I30)))),"")</f>
-      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
@@ -1703,81 +1616,29 @@
       <c r="C31" s="10"/>
       <c r="D31" s="11"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>46317</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
       <c r="D32" s="11"/>
-      <c r="F32" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="G32" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="H32" s="34">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($H$6:$H$30,$G$6:$G$30,"Marta")),"")</f>
-      </c>
-      <c r="I32" s="35">
-        <f>IFERROR(IF($H32=0,"",$J32/$H32),"")</f>
-      </c>
-      <c r="J32" s="34">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($J$6:$J$30,$G$6:$G$30,"Marta")),"")</f>
-      </c>
-      <c r="K32" s="34">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$30,$G$6:$G$30,"Marta")=0,"",SUMIFS($K$6:$K$30,$G$6:$G$30,"Marta")),"")</f>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>46317</v>
       </c>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
-      <c r="F33" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="G33" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="H33" s="34">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="I33" s="35">
-        <f>IFERROR(IF($H33=0,"",$J33/$H33),"")</f>
-      </c>
-      <c r="J33" s="34">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="K33" s="34">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$30,$G$6:$G$30,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$30,$G$6:$G$30,"Fondo ahorro")),"")</f>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="9">
         <v>46317</v>
       </c>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="11"/>
-      <c r="F34" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="G34" s="36"/>
-      <c r="H34" s="37">
-        <f>IFERROR(IF(SUM($H$6:$H$30)=0,"",SUM($H$6:$H$30)),"")</f>
-      </c>
-      <c r="I34" s="38">
-        <f>IFERROR(IF($H34=0,"",$J34/$H34),"")</f>
-      </c>
-      <c r="J34" s="37">
-        <f>IFERROR(IF(SUM($J$6:$J$30)=0,"",SUM($J$6:$J$30)),"")</f>
-      </c>
-      <c r="K34" s="37">
-        <f>IFERROR(IF(SUM($K$6:$K$30)=0,"",SUM($K$6:$K$30)),"")</f>
-      </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="9">
@@ -1787,35 +1648,21 @@
       <c r="C35" s="10"/>
       <c r="D35" s="11"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="39" t="s">
-        <v>33</v>
-      </c>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
-      <c r="J36" s="39"/>
-      <c r="K36" s="39"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="B37" s="39"/>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="39"/>
-      <c r="H37" s="39"/>
-      <c r="I37" s="39"/>
-      <c r="J37" s="39"/>
-      <c r="K37" s="39"/>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="11"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="11"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="9">
@@ -5562,7 +5409,7 @@
       <c r="D505" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
+  <sheetProtection sheet="1" objects="0" scenarios="0" selectLockedCells="0" selectUnlockedCells="0" formatCells="0" formatRows="0" insertRows="0" deleteRows="0"/>
   <mergeCells count="8">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:D3"/>
@@ -5570,8 +5417,8 @@
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:K4"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A24:K24"/>
   </mergeCells>
   <conditionalFormatting sqref="A6:D505">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -5584,7 +5431,7 @@
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16:K30">
+  <conditionalFormatting sqref="F16:K17">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>$F16&lt;&gt;""</formula>
     </cfRule>
@@ -5595,7 +5442,7 @@
       <formula>$F15=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I16:I30">
+  <conditionalFormatting sqref="I16:I17">
     <cfRule type="expression" dxfId="6" priority="4">
       <formula>$F16&lt;&gt;""</formula>
     </cfRule>
@@ -5603,7 +5450,7 @@
       <formula>AND($F15&lt;&gt;"",$F16="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F30">
+  <conditionalFormatting sqref="F9:F17">
     <cfRule type="expression" dxfId="8" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
@@ -5611,7 +5458,7 @@
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J30">
+  <conditionalFormatting sqref="I6:J17">
     <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
El Excel: siete filas nuevas, gráficos en la página 2 (con el del Fondo ahorro), el flujo del dinero en la 3, título Myinvestor y lo que queda a cero desaparece
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -8,7 +8,7 @@
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$17),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O128</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
   <si>
-    <t>MIS INVERSIONES · MOVIMIENTOS: DE DÓNDE VIENE EL DINERO</t>
+    <t>Myinvestor</t>
   </si>
   <si>
     <t>Escribe cada movimiento: fecha, de dónde sale (De), a dónde va (A) e importe. Solo se ve una fila: al rellenarla, se abre la siguiente.</t>
@@ -363,7 +363,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <font>
         <color rgb="FF0F172A"/>
@@ -459,6 +459,12 @@
           <fgColor rgb="FFFFFBEB"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+        <sz val="10"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -684,24 +690,424 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="334155"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000"/>
+              <a:t>Marta: inversión por inversión</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Aportado neto</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Vanguard Global Stock Index</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Fidelity MSCI World Index</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Cartera indexada Metal</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Depósito 12 meses</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Plan de pensiones indexado</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$H$8:$H$12</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Beneficio-pérdida</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E67E22"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="5"/>
+              <c:pt idx="0">
+                <c:v>Vanguard Global Stock Index</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Fidelity MSCI World Index</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Cartera indexada Metal</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Depósito 12 meses</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Plan de pensiones indexado</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$J$8:$J$12</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="-80"/>
+        <c:axId val="100000001"/>
+        <c:axId val="100000002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="100000001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100000002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="D8DEE9"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="334155"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000"/>
+              <a:t>Fondo ahorro: inversión por inversión</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Aportado neto</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>Fondo indexado</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>iShares Developed World Index</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$H$14:$H$15</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Beneficio-pérdida</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E67E22"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="2"/>
+              <c:pt idx="0">
+                <c:v>Fondo indexado</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>iShares Developed World Index</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$J$14:$J$15</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="-80"/>
+        <c:axId val="100000001"/>
+        <c:axId val="100000002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="100000001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100000002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="D8DEE9"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Grafico"/>
+        <xdr:cNvPr id="2" name="Grafico 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -714,6 +1120,1292 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Grafico 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Grafico 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>127</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="1" name="Flujo del dinero"/>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="15182850" cy="6667500"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="15182850" cy="6667500"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="1" name="Titulo del flujo"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="14859000" cy="304800"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F172A"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F172A"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Flujo del dinero: de dónde llega, por dónde pasa y a dónde va</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="De 1"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1047750" y="381000"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="64748B"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Exterior</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="Flecha 1"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3981450" y="457200"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="4" name="A 1"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="381000"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="5" name="De 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1047750" y="1104900"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="64748B"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Exterior</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="6" name="Flecha 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3981450" y="1181100"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="7" name="A 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="1104900"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Fondo indexado</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="De 3"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1047750" y="1828800"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="64748B"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Exterior</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="9" name="Flecha 3"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3981450" y="1905000"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="10" name="A 3"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="1828800"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>iShares Developed World Index</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="De 4"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="2552700"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="Flecha 4"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8934450" y="2628900"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="13" name="A 4"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10953750" y="2552700"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="0F766E"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Vanguard Global Stock Index</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="14" name="De 5"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="3276600"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="15" name="Flecha 5"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8934450" y="3352800"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="16" name="A 5"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10953750" y="3276600"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="0F766E"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Fidelity MSCI World Index</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="17" name="De 6"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="4000500"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="18" name="Flecha 6"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8934450" y="4076700"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="19" name="A 6"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10953750" y="4000500"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="0F766E"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cartera indexada Metal</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="20" name="De 7"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="4724400"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="21" name="Flecha 7"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8934450" y="4800600"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="22" name="A 7"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10953750" y="4724400"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="0F766E"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Depósito 12 meses</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="23" name="De 8"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6000750" y="5448300"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="1D4ED8"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cuenta Myinvestor</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="24" name="Flecha 8"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8934450" y="5524500"/>
+            <a:ext cx="1943100" cy="285750"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst>
+              <a:gd name="adj1" fmla="50000"/>
+              <a:gd name="adj2" fmla="50000"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="F1F5F9"/>
+          </a:solidFill>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="CBD5E1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="1D4ED8"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="25" name="A 8"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10953750" y="5448300"/>
+            <a:ext cx="2857500" cy="438150"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst>
+              <a:gd name="adj" fmla="16667"/>
+            </a:avLst>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="0F766E"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+            <a:noAutofit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Plan de pensiones indexado</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1192,16 +2884,16 @@
         <v>20</v>
       </c>
       <c r="H7" s="16">
-        <f>IFERROR(IF($F7="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F7)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F7)),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
       </c>
       <c r="I7" s="17">
-        <f>IFERROR(IF($F7="","",IF($H7=0,"",$J7/$H7)),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",IF(OR($H7=0,$H7=""),"",$J7/$H7))),"")</f>
       </c>
       <c r="J7" s="16">
-        <f>IFERROR(IF($F7="","",$K7-$H7),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
       </c>
       <c r="K7" s="16">
-        <f>IFERROR(IF($F7="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F7)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F7)),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1218,14 +2910,14 @@
         <v>20</v>
       </c>
       <c r="H8" s="16">
-        <f>IFERROR(IF($F8="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F8)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F8)),"")</f>
+        <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index"))),"")</f>
       </c>
       <c r="I8" s="19"/>
       <c r="J8" s="16">
-        <f>IFERROR(IF($F8="","",$K8-$H8),"")</f>
+        <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",IF(OR($H8="",$K8=""),"",$K8-$H8))),"")</f>
       </c>
       <c r="K8" s="16">
-        <f>IFERROR(IF($F8="","",IF($H8=0,"",IF($I8="",$H8,$H8*(1+$I8)))),"")</f>
+        <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",IF(OR($H8="",$H8=0),"",IF($I8="",$H8,$H8*(1+$I8))))),"")</f>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1242,14 +2934,14 @@
         <v>20</v>
       </c>
       <c r="H9" s="21">
-        <f>IFERROR(IF($F9="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F9)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F9)),"")</f>
+        <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index"))),"")</f>
       </c>
       <c r="I9" s="22"/>
       <c r="J9" s="21">
-        <f>IFERROR(IF($F9="","",$K9-$H9),"")</f>
+        <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",IF(OR($H9="",$K9=""),"",$K9-$H9))),"")</f>
       </c>
       <c r="K9" s="21">
-        <f>IFERROR(IF($F9="","",IF($H9=0,"",IF($I9="",$H9,$H9*(1+$I9)))),"")</f>
+        <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",IF(OR($H9="",$H9=0),"",IF($I9="",$H9,$H9*(1+$I9))))),"")</f>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1266,14 +2958,14 @@
         <v>20</v>
       </c>
       <c r="H10" s="21">
-        <f>IFERROR(IF($F10="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F10)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F10)),"")</f>
+        <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal"))),"")</f>
       </c>
       <c r="I10" s="22"/>
       <c r="J10" s="21">
-        <f>IFERROR(IF($F10="","",$K10-$H10),"")</f>
+        <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",IF(OR($H10="",$K10=""),"",$K10-$H10))),"")</f>
       </c>
       <c r="K10" s="21">
-        <f>IFERROR(IF($F10="","",IF($H10=0,"",IF($I10="",$H10,$H10*(1+$I10)))),"")</f>
+        <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",IF(OR($H10="",$H10=0),"",IF($I10="",$H10,$H10*(1+$I10))))),"")</f>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1290,14 +2982,14 @@
         <v>20</v>
       </c>
       <c r="H11" s="21">
-        <f>IFERROR(IF($F11="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F11)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F11)),"")</f>
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses"))),"")</f>
       </c>
       <c r="I11" s="22"/>
       <c r="J11" s="21">
-        <f>IFERROR(IF($F11="","",$K11-$H11),"")</f>
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",IF(OR($H11="",$K11=""),"",$K11-$H11))),"")</f>
       </c>
       <c r="K11" s="21">
-        <f>IFERROR(IF($F11="","",IF($H11=0,"",IF($I11="",$H11,$H11*(1+$I11)))),"")</f>
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",IF(OR($H11="",$H11=0),"",IF($I11="",$H11,$H11*(1+$I11))))),"")</f>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1314,14 +3006,14 @@
         <v>20</v>
       </c>
       <c r="H12" s="21">
-        <f>IFERROR(IF($F12="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F12)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F12)),"")</f>
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado"))),"")</f>
       </c>
       <c r="I12" s="22"/>
       <c r="J12" s="21">
-        <f>IFERROR(IF($F12="","",$K12-$H12),"")</f>
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",IF(OR($H12="",$K12=""),"",$K12-$H12))),"")</f>
       </c>
       <c r="K12" s="21">
-        <f>IFERROR(IF($F12="","",IF($H12=0,"",IF($I12="",$H12,$H12*(1+$I12)))),"")</f>
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",IF(OR($H12="",$H12=0),"",IF($I12="",$H12,$H12*(1+$I12))))),"")</f>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1338,16 +3030,16 @@
         <v>20</v>
       </c>
       <c r="H13" s="21">
-        <f>IFERROR(IF($F13="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)),"")</f>
+        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING"))),"")</f>
       </c>
       <c r="I13" s="24">
-        <f>IFERROR(IF($F13="","",IF($H13=0,"",$J13/$H13)),"")</f>
+        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",IF(OR($H13=0,$H13=""),"",$J13/$H13))),"")</f>
       </c>
       <c r="J13" s="21">
-        <f>IFERROR(IF($F13="","",$K13-$H13),"")</f>
+        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",IF(OR($H13="",$K13=""),"",$K13-$H13))),"")</f>
       </c>
       <c r="K13" s="21">
-        <f>IFERROR(IF($F13="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)),"")</f>
+        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING"))),"")</f>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1364,14 +3056,14 @@
         <v>28</v>
       </c>
       <c r="H14" s="26">
-        <f>IFERROR(IF($F14="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)),"")</f>
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
       </c>
       <c r="I14" s="27"/>
       <c r="J14" s="26">
-        <f>IFERROR(IF($F14="","",$K14-$H14),"")</f>
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H14="",$K14=""),"",$K14-$H14))),"")</f>
       </c>
       <c r="K14" s="26">
-        <f>IFERROR(IF($F14="","",IF($H14=0,"",IF($I14="",$H14,$H14*(1+$I14)))),"")</f>
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H14="",$H14=0),"",IF($I14="",$H14,$H14*(1+$I14))))),"")</f>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1388,14 +3080,14 @@
         <v>28</v>
       </c>
       <c r="H15" s="26">
-        <f>IFERROR(IF($F15="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15)),"")</f>
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
       </c>
       <c r="I15" s="27"/>
       <c r="J15" s="26">
-        <f>IFERROR(IF($F15="","",$K15-$H15),"")</f>
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H15="",$K15=""),"",$K15-$H15))),"")</f>
       </c>
       <c r="K15" s="26">
-        <f>IFERROR(IF($F15="","",IF($H15=0,"",IF($I15="",$H15,$H15*(1+$I15)))),"")</f>
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H15="",$H15=0),"",IF($I15="",$H15,$H15*(1+$I15))))),"")</f>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1408,14 +3100,14 @@
       <c r="F16" s="28"/>
       <c r="G16" s="29"/>
       <c r="H16" s="30">
-        <f>IFERROR(IF($F16="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)),"")</f>
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16))),"")</f>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="30">
-        <f>IFERROR(IF($F16="","",$K16-$H16),"")</f>
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$K16=""),"",$K16-$H16))),"")</f>
       </c>
       <c r="K16" s="30">
-        <f>IFERROR(IF($F16="","",IF($H16=0,"",IF($I16="",$H16,$H16*(1+$I16)))),"")</f>
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$H16=0),"",IF($I16="",$H16,$H16*(1+$I16))))),"")</f>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1428,14 +3120,14 @@
       <c r="F17" s="28"/>
       <c r="G17" s="29"/>
       <c r="H17" s="30">
-        <f>IFERROR(IF($F17="","",SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)),"")</f>
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17))),"")</f>
       </c>
       <c r="I17" s="31"/>
       <c r="J17" s="30">
-        <f>IFERROR(IF($F17="","",$K17-$H17),"")</f>
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$K17=""),"",$K17-$H17))),"")</f>
       </c>
       <c r="K17" s="30">
-        <f>IFERROR(IF($F17="","",IF($H17=0,"",IF($I17="",$H17,$H17*(1+$I17)))),"")</f>
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$H17=0),"",IF($I17="",$H17,$H17*(1+$I17))))),"")</f>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -5450,19 +7142,24 @@
       <formula>AND($F15&lt;&gt;"",$F16="")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F7:K15">
+    <cfRule type="expression" dxfId="8" priority="1">
+      <formula>$H7=""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F9:F17">
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="10" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:J17">
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5478,7 +7175,11 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="26" min="0" max="16383" man="1"/>
+    <brk id="92" min="0" max="16383" man="1"/>
+  </rowBreaks>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Los gráficos y el flujo del dinero, en dos hojas aparte («Gráficos» y «Flujo»), cada una con su dibujo
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -5,18 +5,22 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Gráficos" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Flujo" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$17),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O128</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O28</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -122,6 +126,18 @@
   <si>
     <t>En las inversiones se escribe la rentabilidad en % (la celda amarilla, como en la app) y el saldo se calcula solo. «Exterior» es el dinero que entra o sale de fuera. La hoja está protegida: solo se puede escribir en los movimientos, en las filas nuevas y en el %.</t>
   </si>
+  <si>
+    <t>Gráficos</t>
+  </si>
+  <si>
+    <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
+  </si>
+  <si>
+    <t>Flujo del dinero: de dónde llega, por dónde pasa y a dónde va</t>
+  </si>
+  <si>
+    <t>Se dibuja con los movimientos de hoy: vuelve a descargar el Excel para tenerlo al día.</t>
+  </si>
 </sst>
 </file>
 
@@ -132,7 +148,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -214,6 +230,11 @@
       <b/>
       <sz val="10"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="16"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -264,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -358,6 +379,9 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1096,13 +1120,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1126,13 +1150,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1156,13 +1180,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>88</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1182,1230 +1206,1521 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>127</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="1" name="Flujo del dinero"/>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="De 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="15182850" cy="6667500"/>
-          <a:chOff x="0" y="0"/>
-          <a:chExt cx="15182850" cy="6667500"/>
+          <a:ext cx="2857500" cy="438150"/>
         </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="1" name="Titulo del flujo"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="14859000" cy="304800"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="64748B"/>
+        </a:solidFill>
+        <a:ln>
           <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="0F172A"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="0F172A"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Flujo del dinero: de dónde llega, por dónde pasa y a dónde va</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="2" name="De 1"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1047750" y="381000"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Exterior</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Flecha 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="64748B"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Exterior</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="3" name="Flecha 1"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="3981450" y="457200"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="A 1"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>215900</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="De 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="64748B"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Exterior</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Flecha 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="4" name="A 1"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="381000"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>215900</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="A 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Fondo indexado</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="De 3"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="64748B"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Exterior</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Flecha 3"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="5" name="De 2"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1047750" y="1104900"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="A 3"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>iShares Developed World Index</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="De 4"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>215900</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>247650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Flecha 4"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="64748B"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Exterior</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="6" name="Flecha 2"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="3981450" y="1181100"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="A 4"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="0F766E"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Vanguard Global Stock Index</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="De 5"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Flecha 5"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="7" name="A 2"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="1104900"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="A 5"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="0F766E"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Fidelity MSCI World Index</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>247650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="De 6"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="Flecha 6"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Fondo indexado</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="8" name="De 3"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1047750" y="1828800"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>247650</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="A 6"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="0F766E"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cartera indexada Metal</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="De 7"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Flecha 7"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="64748B"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Exterior</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="9" name="Flecha 3"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="3981450" y="1905000"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="A 7"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="0F766E"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Depósito 12 meses</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>241300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="De 8"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="1D4ED8"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Cuenta Myinvestor</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Flecha 8"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1943100" cy="285750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst>
+            <a:gd name="adj1" fmla="50000"/>
+            <a:gd name="adj2" fmla="50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F1F5F9"/>
+        </a:solidFill>
+        <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
+            <a:srgbClr val="CBD5E1"/>
           </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="10" name="A 3"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="1828800"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>iShares Developed World Index</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="11" name="De 4"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="2552700"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="12" name="Flecha 4"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="8934450" y="2628900"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
-          </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="13" name="A 4"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10953750" y="2552700"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="0F766E"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Vanguard Global Stock Index</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="14" name="De 5"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="3276600"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="15" name="Flecha 5"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="8934450" y="3352800"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
-          </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="16" name="A 5"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10953750" y="3276600"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="0F766E"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Fidelity MSCI World Index</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="17" name="De 6"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="4000500"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="18" name="Flecha 6"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="8934450" y="4076700"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
-          </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="19" name="A 6"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10953750" y="4000500"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="0F766E"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cartera indexada Metal</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="20" name="De 7"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="4724400"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="21" name="Flecha 7"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="8934450" y="4800600"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
-          </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="22" name="A 7"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10953750" y="4724400"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="0F766E"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Depósito 12 meses</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="23" name="De 8"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="6000750" y="5448300"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="1D4ED8"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Cuenta Myinvestor</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="24" name="Flecha 8"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="8934450" y="5524500"/>
-            <a:ext cx="1943100" cy="285750"/>
-          </a:xfrm>
-          <a:prstGeom prst="rightArrow">
-            <a:avLst>
-              <a:gd name="adj1" fmla="50000"/>
-              <a:gd name="adj2" fmla="50000"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="F1F5F9"/>
-          </a:solidFill>
-          <a:ln w="9525">
-            <a:solidFill>
-              <a:srgbClr val="CBD5E1"/>
-            </a:solidFill>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="900" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="1D4ED8"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="25" name="A 8"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10953750" y="5448300"/>
-            <a:ext cx="2857500" cy="438150"/>
-          </a:xfrm>
-          <a:prstGeom prst="roundRect">
-            <a:avLst>
-              <a:gd name="adj" fmla="16667"/>
-            </a:avLst>
-          </a:prstGeom>
-          <a:solidFill>
-            <a:srgbClr val="0F766E"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr">
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Plan de pensiones indexado</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-    </xdr:grpSp>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="1D4ED8"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t/>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>241300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="A 8"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2857500" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="16667"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="0F766E"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr">
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Plan de pensiones indexado</a:t>
+          </a:r>
+          <a:endParaRPr/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -7175,11 +7490,204 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="26" min="0" max="16383" man="1"/>
-    <brk id="92" min="0" max="16383" man="1"/>
-  </rowBreaks>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF1D4ED8"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O52"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="15" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF1D4ED8"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O28"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="15" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dos gráficos (uno por titular) a la mitad de tamaño y el flujo del dinero pintado con celdas en su hoja
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -12,15 +12,15 @@
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$17),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O52</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O20</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="43">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -138,6 +138,18 @@
   <si>
     <t>Se dibuja con los movimientos de hoy: vuelve a descargar el Excel para tenerlo al día.</t>
   </si>
+  <si>
+    <t>De dónde llega</t>
+  </si>
+  <si>
+    <t>Por dónde pasa</t>
+  </si>
+  <si>
+    <t>A dónde va</t>
+  </si>
+  <si>
+    <t>▶</t>
+  </si>
 </sst>
 </file>
 
@@ -148,7 +160,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -235,8 +247,18 @@
       <color rgb="FF0F172A"/>
       <sz val="16"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF64748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF94A3B8"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,6 +285,16 @@
         <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF64748B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -285,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -382,6 +414,21 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,7 +589,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Aportado neto y beneficio / pérdida por titular</a:t>
+              <a:t>Marta: cuentas e inversiones</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -584,18 +631,33 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="2"/>
+              <c:ptCount val="7"/>
               <c:pt idx="0">
-                <c:v>Marta</c:v>
+                <c:v>Cuenta Myinvestor</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Fondo ahorro</c:v>
+                <c:v>Vanguard Global Stock Index</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Fidelity MSCI World Index</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Cartera indexada Metal</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Depósito 12 meses</c:v>
+              </c:pt>
+              <c:pt idx="5">
+                <c:v>Plan de pensiones indexado</c:v>
+              </c:pt>
+              <c:pt idx="6">
+                <c:v>Cuenta ahorro · ING</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$19:$H$20</c:f>
+              <c:f>Movimientos!$H$7:$H$13</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -626,18 +688,33 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="2"/>
+              <c:ptCount val="7"/>
               <c:pt idx="0">
-                <c:v>Marta</c:v>
+                <c:v>Cuenta Myinvestor</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Fondo ahorro</c:v>
+                <c:v>Vanguard Global Stock Index</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Fidelity MSCI World Index</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Cartera indexada Metal</c:v>
+              </c:pt>
+              <c:pt idx="4">
+                <c:v>Depósito 12 meses</c:v>
+              </c:pt>
+              <c:pt idx="5">
+                <c:v>Plan de pensiones indexado</c:v>
+              </c:pt>
+              <c:pt idx="6">
+                <c:v>Cuenta ahorro · ING</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$19:$J$20</c:f>
+              <c:f>Movimientos!$J$7:$J$13</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -733,216 +810,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Marta: inversión por inversión</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Aportado neto</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="2563EB"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="5"/>
-              <c:pt idx="0">
-                <c:v>Vanguard Global Stock Index</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>Fidelity MSCI World Index</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>Cartera indexada Metal</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Depósito 12 meses</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>Plan de pensiones indexado</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$H$8:$H$12</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Beneficio-pérdida</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="E67E22"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="5"/>
-              <c:pt idx="0">
-                <c:v>Vanguard Global Stock Index</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>Fidelity MSCI World Index</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>Cartera indexada Metal</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Depósito 12 meses</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>Plan de pensiones indexado</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$J$8:$J$12</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="-80"/>
-        <c:axId val="100000001"/>
-        <c:axId val="100000002"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="100000001"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000002"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="100000002"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000001"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln>
-      <a:solidFill>
-        <a:srgbClr val="D8DEE9"/>
-      </a:solidFill>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="334155"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Fondo ahorro: inversión por inversión</a:t>
+              <a:t>Fondo ahorro: inversiones</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -1124,9 +992,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1148,15 +1016,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1174,1553 +1042,6 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Grafico 3"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="De 1"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="64748B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Exterior</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>838200</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Flecha 1"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="A 1"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>215900</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>146050</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="De 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="64748B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Exterior</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>838200</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Flecha 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>215900</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>146050</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="A 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Fondo indexado</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="De 3"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="64748B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Exterior</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>838200</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Flecha 3"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="A 3"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>iShares Developed World Index</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="De 4"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>215900</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>247650</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Flecha 4"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="A 4"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="0F766E"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Vanguard Global Stock Index</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="De 5"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Flecha 5"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="A 5"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="0F766E"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Fidelity MSCI World Index</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>247650</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="De 6"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="Flecha 6"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>247650</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="A 6"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="0F766E"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cartera indexada Metal</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="De 7"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="20" name="Flecha 7"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="A 7"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="0F766E"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Depósito 12 meses</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>241300</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="De 8"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="1D4ED8"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Cuenta Myinvestor</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="Flecha 8"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1943100" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rightArrow">
-          <a:avLst>
-            <a:gd name="adj1" fmla="50000"/>
-            <a:gd name="adj2" fmla="50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="F1F5F9"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="CBD5E1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="1D4ED8"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t/>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>241300</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="A 8"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2857500" cy="438150"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst>
-            <a:gd name="adj" fmla="16667"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="0F766E"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" lIns="27432" tIns="18288" rIns="27432" bIns="18288" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:defRPr sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-ES" sz="1000" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Plan de pensiones indexado</a:t>
-          </a:r>
-          <a:endParaRPr/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -7500,7 +5821,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="15" customWidth="1"/>
@@ -7559,41 +5880,6 @@
     <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
@@ -7611,10 +5897,15 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="15" width="15" customWidth="1"/>
+    <col min="1" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -7655,39 +5946,208 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="F3" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="K3" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+    </row>
+    <row r="5" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="45"/>
+      <c r="M6" s="45"/>
+      <c r="N6" s="45"/>
+    </row>
+    <row r="7" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="45"/>
+      <c r="M8" s="45"/>
+      <c r="N8" s="45"/>
+    </row>
+    <row r="9" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F10" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="45"/>
+    </row>
+    <row r="11" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F12" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="K12" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="L12" s="45"/>
+      <c r="M12" s="45"/>
+      <c r="N12" s="45"/>
+    </row>
+    <row r="13" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F14" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="K14" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="L14" s="45"/>
+      <c r="M14" s="45"/>
+      <c r="N14" s="45"/>
+    </row>
+    <row r="15" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F16" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="44"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="45" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="45"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="45"/>
+    </row>
+    <row r="17" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F18" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="K18" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="45"/>
+    </row>
+    <row r="19" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="23">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E8:J8"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="K10:N10"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="K12:N12"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="K16:N16"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="K18:N18"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Gráficos de tres barras por titular (aportado, rentabilidad y saldo) y el flujo con el dinero y los movimientos uno a uno
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -13,14 +13,14 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O29</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -82,13 +82,19 @@
     <t>Cuenta Myinvestor</t>
   </si>
   <si>
+    <t>Vanguard Global Stock Index</t>
+  </si>
+  <si>
     <t>Marta</t>
   </si>
   <si>
-    <t>Vanguard Global Stock Index</t>
+    <t>Fidelity MSCI World Index</t>
   </si>
   <si>
-    <t>Fidelity MSCI World Index</t>
+    <t>Fondo indexado</t>
+  </si>
+  <si>
+    <t>iShares Developed World Index</t>
   </si>
   <si>
     <t>Cartera indexada Metal</t>
@@ -103,13 +109,7 @@
     <t>Cuenta ahorro · ING</t>
   </si>
   <si>
-    <t>Fondo indexado</t>
-  </si>
-  <si>
     <t>Fondo ahorro</t>
-  </si>
-  <si>
-    <t>iShares Developed World Index</t>
   </si>
   <si>
     <t>Total Cuenta Myinvestor-Marta</t>
@@ -148,7 +148,34 @@
     <t>A dónde va</t>
   </si>
   <si>
+    <t>1000,00 €   ▶</t>
+  </si>
+  <si>
+    <t>400,00 €   ▶</t>
+  </si>
+  <si>
+    <t>300,00 €   ▶</t>
+  </si>
+  <si>
+    <t>200,00 €   ▶</t>
+  </si>
+  <si>
+    <t>150,00 €   ▶</t>
+  </si>
+  <si>
     <t>▶</t>
+  </si>
+  <si>
+    <t>Movimientos, uno a uno</t>
+  </si>
+  <si>
+    <t>De</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Total de los 5 movimientos</t>
   </si>
 </sst>
 </file>
@@ -160,7 +187,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -254,8 +281,18 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF94A3B8"/>
-      <sz val="10"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="8">
@@ -317,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -421,7 +458,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -429,6 +466,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -589,7 +650,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Marta: cuentas e inversiones</a:t>
+              <a:t>Marta</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -608,7 +669,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Aportado neto</c:v>
+            <c:v>Aportado</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -631,33 +692,15 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="7"/>
+              <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Cuenta Myinvestor</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>Vanguard Global Stock Index</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>Fidelity MSCI World Index</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Cartera indexada Metal</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>Depósito 12 meses</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>Plan de pensiones indexado</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>Cuenta ahorro · ING</c:v>
+                <c:v>Marta</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$7:$H$13</c:f>
+              <c:f>Movimientos!$H$19</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -665,7 +708,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Beneficio-pérdida</c:v>
+            <c:v>Rentabilidad</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -688,33 +731,54 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="7"/>
+              <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Cuenta Myinvestor</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>Vanguard Global Stock Index</c:v>
-              </c:pt>
-              <c:pt idx="2">
-                <c:v>Fidelity MSCI World Index</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Cartera indexada Metal</c:v>
-              </c:pt>
-              <c:pt idx="4">
-                <c:v>Depósito 12 meses</c:v>
-              </c:pt>
-              <c:pt idx="5">
-                <c:v>Plan de pensiones indexado</c:v>
-              </c:pt>
-              <c:pt idx="6">
-                <c:v>Cuenta ahorro · ING</c:v>
+                <c:v>Marta</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$7:$J$13</c:f>
+              <c:f>Movimientos!$J$19</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Aportado + rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F766E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$K$19</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -810,7 +874,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Fondo ahorro: inversiones</a:t>
+              <a:t>Fondo ahorro</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -829,7 +893,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Aportado neto</c:v>
+            <c:v>Aportado</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -852,18 +916,15 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="2"/>
+              <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Fondo indexado</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>iShares Developed World Index</c:v>
+                <c:v>Fondo ahorro</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$14:$H$15</c:f>
+              <c:f>Movimientos!$H$20</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -871,7 +932,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Beneficio-pérdida</c:v>
+            <c:v>Rentabilidad</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill>
@@ -894,18 +955,54 @@
           </c:dLbls>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="2"/>
+              <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Fondo indexado</c:v>
-              </c:pt>
-              <c:pt idx="1">
-                <c:v>iShares Developed World Index</c:v>
+                <c:v>Fondo ahorro</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$14:$J$15</c:f>
+              <c:f>Movimientos!$J$20</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Aportado + rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F766E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$K$20</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1492,11 +1589,17 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="11"/>
+        <v>46296</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="11">
+        <v>1000</v>
+      </c>
       <c r="F6" s="12" t="s">
         <v>18</v>
       </c>
@@ -1508,16 +1611,22 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="11"/>
+        <v>46297</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="11">
+        <v>300</v>
+      </c>
       <c r="F7" s="14" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H7" s="16">
         <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
@@ -1534,16 +1643,22 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="11"/>
+        <v>46297</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="11">
+        <v>200</v>
+      </c>
       <c r="F8" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="15" t="s">
         <v>21</v>
-      </c>
-      <c r="G8" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="H8" s="16">
         <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index"))),"")</f>
@@ -1558,16 +1673,22 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="11"/>
+        <v>46298</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="11">
+        <v>400</v>
+      </c>
       <c r="F9" s="20" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H9" s="21">
         <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index"))),"")</f>
@@ -1582,16 +1703,22 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="11"/>
+        <v>46300</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="11">
+        <v>150</v>
+      </c>
       <c r="F10" s="20" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H10" s="21">
         <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal"))),"")</f>
@@ -1612,10 +1739,10 @@
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
       <c r="F11" s="20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H11" s="21">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses"))),"")</f>
@@ -1636,10 +1763,10 @@
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
       <c r="F12" s="20" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H12" s="21">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado"))),"")</f>
@@ -1660,10 +1787,10 @@
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
       <c r="F13" s="23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H13" s="21">
         <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING"))),"")</f>
@@ -1686,10 +1813,10 @@
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
       <c r="F14" s="25" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H14" s="26">
         <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
@@ -1710,10 +1837,10 @@
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
       <c r="F15" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="15" t="s">
         <v>29</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>28</v>
       </c>
       <c r="H15" s="26">
         <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
@@ -1785,7 +1912,7 @@
         <v>30</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H19" s="34">
         <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")),"")</f>
@@ -1811,7 +1938,7 @@
         <v>31</v>
       </c>
       <c r="G20" s="33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H20" s="34">
         <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
@@ -5897,7 +6024,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="22" customWidth="1"/>
@@ -5992,7 +6119,7 @@
       <c r="C6" s="42"/>
       <c r="D6" s="42"/>
       <c r="E6" s="43" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -6000,30 +6127,25 @@
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
       <c r="K6" s="45" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L6" s="45"/>
       <c r="M6" s="45"/>
       <c r="N6" s="45"/>
     </row>
     <row r="7" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
+    <row r="8" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F8" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="43" t="s">
+        <v>44</v>
+      </c>
       <c r="K8" s="45" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="L8" s="45"/>
       <c r="M8" s="45"/>
@@ -6038,10 +6160,10 @@
       <c r="H10" s="44"/>
       <c r="I10" s="44"/>
       <c r="J10" s="43" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K10" s="45" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L10" s="45"/>
       <c r="M10" s="45"/>
@@ -6056,10 +6178,10 @@
       <c r="H12" s="44"/>
       <c r="I12" s="44"/>
       <c r="J12" s="43" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="K12" s="45" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L12" s="45"/>
       <c r="M12" s="45"/>
@@ -6073,11 +6195,11 @@
       <c r="G14" s="44"/>
       <c r="H14" s="44"/>
       <c r="I14" s="44"/>
-      <c r="J14" s="43" t="s">
-        <v>42</v>
+      <c r="J14" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="K14" s="45" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="L14" s="45"/>
       <c r="M14" s="45"/>
@@ -6091,11 +6213,11 @@
       <c r="G16" s="44"/>
       <c r="H16" s="44"/>
       <c r="I16" s="44"/>
-      <c r="J16" s="43" t="s">
-        <v>42</v>
+      <c r="J16" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L16" s="45"/>
       <c r="M16" s="45"/>
@@ -6109,11 +6231,11 @@
       <c r="G18" s="44"/>
       <c r="H18" s="44"/>
       <c r="I18" s="44"/>
-      <c r="J18" s="43" t="s">
-        <v>42</v>
+      <c r="J18" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="K18" s="45" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="L18" s="45"/>
       <c r="M18" s="45"/>
@@ -6121,8 +6243,192 @@
     </row>
     <row r="19" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="47" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="47"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="47"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="47"/>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" s="48"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="48"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="49">
+        <v>46296</v>
+      </c>
+      <c r="B24" s="49"/>
+      <c r="C24" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="51">
+        <v>1000</v>
+      </c>
+      <c r="L24" s="51"/>
+      <c r="M24" s="51"/>
+      <c r="N24" s="51"/>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="49">
+        <v>46297</v>
+      </c>
+      <c r="B25" s="49"/>
+      <c r="C25" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="51">
+        <v>300</v>
+      </c>
+      <c r="L25" s="51"/>
+      <c r="M25" s="51"/>
+      <c r="N25" s="51"/>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="49">
+        <v>46297</v>
+      </c>
+      <c r="B26" s="49"/>
+      <c r="C26" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="51">
+        <v>200</v>
+      </c>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="49">
+        <v>46298</v>
+      </c>
+      <c r="B27" s="49"/>
+      <c r="C27" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="H27" s="50"/>
+      <c r="I27" s="50"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="51">
+        <v>400</v>
+      </c>
+      <c r="L27" s="51"/>
+      <c r="M27" s="51"/>
+      <c r="N27" s="51"/>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="49">
+        <v>46300</v>
+      </c>
+      <c r="B28" s="49"/>
+      <c r="C28" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="50"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="50"/>
+      <c r="G28" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28" s="50"/>
+      <c r="I28" s="50"/>
+      <c r="J28" s="50"/>
+      <c r="K28" s="51">
+        <v>150</v>
+      </c>
+      <c r="L28" s="51"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="51"/>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="52" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="52"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="52"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="53">
+        <v>2050</v>
+      </c>
+      <c r="L29" s="53"/>
+      <c r="M29" s="53"/>
+      <c r="N29" s="53"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="49">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A3:D3"/>
@@ -6133,8 +6439,7 @@
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="E6:J6"/>
     <mergeCell ref="K6:N6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="E8:J8"/>
+    <mergeCell ref="F8:I8"/>
     <mergeCell ref="K8:N8"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="K10:N10"/>
@@ -6146,8 +6451,35 @@
     <mergeCell ref="K16:N16"/>
     <mergeCell ref="F18:I18"/>
     <mergeCell ref="K18:N18"/>
+    <mergeCell ref="A22:O22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="K23:N23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K24:N24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="K29:N29"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lo que queda a cero desaparece (y lo de abajo sube), fuera la cuenta nómina y un flujo con un renglón por viaje del dinero
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -9,18 +9,18 @@
     <sheet sheetId="3" name="Flujo" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$17),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O25</definedName>
+    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$14),1),1)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O35</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="53">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -91,22 +91,13 @@
     <t>Fidelity MSCI World Index</t>
   </si>
   <si>
+    <t>Cartera indexada Metal</t>
+  </si>
+  <si>
     <t>Fondo indexado</t>
   </si>
   <si>
     <t>iShares Developed World Index</t>
-  </si>
-  <si>
-    <t>Cartera indexada Metal</t>
-  </si>
-  <si>
-    <t>Depósito 12 meses</t>
-  </si>
-  <si>
-    <t>Plan de pensiones indexado</t>
-  </si>
-  <si>
-    <t>Cuenta ahorro · ING</t>
   </si>
   <si>
     <t>Fondo ahorro</t>
@@ -133,25 +124,40 @@
     <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
   </si>
   <si>
-    <t>Flujo del dinero: de dónde llega, por dónde pasa y a dónde va</t>
+    <t>Flujo del dinero</t>
   </si>
   <si>
-    <t>Se dibuja con los movimientos de hoy: vuelve a descargar el Excel para tenerlo al día.</t>
+    <t>Cada línea es el viaje del dinero: de dónde sale, por dónde pasa y dónde acaba. Se dibuja con los movimientos de hoy: vuelve a descargar el Excel para tenerlo al día.</t>
   </si>
   <si>
-    <t>De dónde llega</t>
+    <t xml:space="preserve">Entra de fuera
+1550,00 €</t>
   </si>
   <si>
-    <t>Por dónde pasa</t>
+    <t xml:space="preserve">Sigue en las cuentas
+380,00 €</t>
   </si>
   <si>
-    <t>A dónde va</t>
+    <t xml:space="preserve">Invertido
+1170,00 €</t>
   </si>
   <si>
-    <t>1000,00 €   ▶</t>
+    <t>DE DÓNDE LLEGA</t>
   </si>
   <si>
-    <t>400,00 €   ▶</t>
+    <t>POR DÓNDE PASA</t>
+  </si>
+  <si>
+    <t>A DÓNDE VA</t>
+  </si>
+  <si>
+    <t>400,00 €   ▶▶▶</t>
+  </si>
+  <si>
+    <t>380,00 €   ▶</t>
+  </si>
+  <si>
+    <t>Sigue en la cuenta</t>
   </si>
   <si>
     <t>300,00 €   ▶</t>
@@ -160,10 +166,10 @@
     <t>200,00 €   ▶</t>
   </si>
   <si>
-    <t>150,00 €   ▶</t>
+    <t>150,00 €   ▶▶▶</t>
   </si>
   <si>
-    <t>▶</t>
+    <t>120,00 €   ▶</t>
   </si>
   <si>
     <t>Movimientos, uno a uno</t>
@@ -175,7 +181,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>Total de los 5 movimientos</t>
+    <t>Total de los 6 movimientos</t>
   </si>
 </sst>
 </file>
@@ -187,7 +193,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -249,11 +255,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF2447B8"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <color rgb="FFEA580C"/>
       <sz val="10"/>
     </font>
@@ -285,9 +286,8 @@
       <sz val="12"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF94A3B8"/>
-      <sz val="12"/>
+      <color rgb="FF64748B"/>
+      <sz val="10"/>
     </font>
     <font>
       <b/>
@@ -354,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -411,32 +411,30 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment indent="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -449,28 +447,37 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -495,7 +502,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+        <sz val="10"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF0F172A"/>
@@ -700,7 +713,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$19</c:f>
+              <c:f>Movimientos!$H$16</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -739,7 +752,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$19</c:f>
+              <c:f>Movimientos!$J$16</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -778,7 +791,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$K$19</c:f>
+              <c:f>Movimientos!$K$16</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -924,7 +937,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$H$20</c:f>
+              <c:f>Movimientos!$H$17</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -963,7 +976,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$J$20</c:f>
+              <c:f>Movimientos!$J$17</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1002,7 +1015,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Movimientos!$K$20</c:f>
+              <c:f>Movimientos!$K$17</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1629,16 +1642,16 @@
         <v>21</v>
       </c>
       <c r="H7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
       </c>
       <c r="I7" s="17">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",IF(OR($H7=0,$H7=""),"",$J7/$H7))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7=0,$H7=""),"",$J7/$H7))),"")</f>
       </c>
       <c r="J7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
       </c>
       <c r="K7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta Myinvestor")+COUNTIF($B$6:$B$505,"Cuenta Myinvestor")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H12&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1676,13 +1689,13 @@
         <v>46298</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="11">
-        <v>400</v>
+        <v>120</v>
       </c>
       <c r="F9" s="20" t="s">
         <v>22</v>
@@ -1703,19 +1716,19 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="11">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>21</v>
@@ -1733,26 +1746,32 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="11"/>
-      <c r="F11" s="20" t="s">
+        <v>46300</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="11">
+        <v>150</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="21">
-        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses"))),"")</f>
-      </c>
-      <c r="I11" s="22"/>
-      <c r="J11" s="21">
-        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",IF(OR($H11="",$K11=""),"",$K11-$H11))),"")</f>
-      </c>
-      <c r="K11" s="21">
-        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Depósito 12 meses")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Depósito 12 meses")&lt;=0),"",IF(OR($H11="",$H11=0),"",IF($I11="",$H11,$H11*(1+$I11))))),"")</f>
+      <c r="H11" s="24">
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
+      </c>
+      <c r="I11" s="25"/>
+      <c r="J11" s="24">
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H11="",$K11=""),"",$K11-$H11))),"")</f>
+      </c>
+      <c r="K11" s="24">
+        <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H11="",$H11=0),"",IF($I11="",$H11,$H11*(1+$I11))))),"")</f>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1762,21 +1781,21 @@
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
-      <c r="F12" s="20" t="s">
-        <v>27</v>
+      <c r="F12" s="23" t="s">
+        <v>25</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="21">
-        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado"))),"")</f>
-      </c>
-      <c r="I12" s="22"/>
-      <c r="J12" s="21">
-        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",IF(OR($H12="",$K12=""),"",$K12-$H12))),"")</f>
-      </c>
-      <c r="K12" s="21">
-        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Plan de pensiones indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Plan de pensiones indexado")&lt;=0),"",IF(OR($H12="",$H12=0),"",IF($I12="",$H12,$H12*(1+$I12))))),"")</f>
+        <v>26</v>
+      </c>
+      <c r="H12" s="24">
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
+      </c>
+      <c r="I12" s="25"/>
+      <c r="J12" s="24">
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H12="",$K12=""),"",$K12-$H12))),"")</f>
+      </c>
+      <c r="K12" s="24">
+        <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H12="",$H12=0),"",IF($I12="",$H12,$H12*(1+$I12))))),"")</f>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1786,23 +1805,17 @@
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
-      <c r="F13" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="21">
-        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING"))),"")</f>
-      </c>
-      <c r="I13" s="24">
-        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",IF(OR($H13=0,$H13=""),"",$J13/$H13))),"")</f>
-      </c>
-      <c r="J13" s="21">
-        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",IF(OR($H13="",$K13=""),"",$K13-$H13))),"")</f>
-      </c>
-      <c r="K13" s="21">
-        <f>IFERROR(IF($F13="","",IF(AND(COUNTIF($C$6:$C$505,"Cuenta ahorro · ING")+COUNTIF($B$6:$B$505,"Cuenta ahorro · ING")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta ahorro · ING")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta ahorro · ING"))),"")</f>
+      <c r="F13" s="26"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="28">
+        <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13))),"")</f>
+      </c>
+      <c r="I13" s="29"/>
+      <c r="J13" s="28">
+        <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",IF(OR($H13="",$K13=""),"",$K13-$H13))),"")</f>
+      </c>
+      <c r="K13" s="28">
+        <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",IF(OR($H13="",$H13=0),"",IF($I13="",$H13,$H13*(1+$I13))))),"")</f>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1812,46 +1825,26 @@
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
-      <c r="F14" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" s="26">
-        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
-      </c>
-      <c r="I14" s="27"/>
-      <c r="J14" s="26">
-        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H14="",$K14=""),"",$K14-$H14))),"")</f>
-      </c>
-      <c r="K14" s="26">
-        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H14="",$H14=0),"",IF($I14="",$H14,$H14*(1+$I14))))),"")</f>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F14" s="26"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28">
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14))),"")</f>
+      </c>
+      <c r="I14" s="29"/>
+      <c r="J14" s="28">
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",IF(OR($H14="",$K14=""),"",$K14-$H14))),"")</f>
+      </c>
+      <c r="K14" s="28">
+        <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",IF(OR($H14="",$H14=0),"",IF($I14="",$H14,$H14*(1+$I14))))),"")</f>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>46317</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
-      <c r="F15" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="26">
-        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
-      </c>
-      <c r="I15" s="27"/>
-      <c r="J15" s="26">
-        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H15="",$K15=""),"",$K15-$H15))),"")</f>
-      </c>
-      <c r="K15" s="26">
-        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H15="",$H15=0),"",IF($I15="",$H15,$H15*(1+$I15))))),"")</f>
-      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
@@ -1860,17 +1853,23 @@
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="30">
-        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16))),"")</f>
-      </c>
-      <c r="I16" s="31"/>
-      <c r="J16" s="30">
-        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$K16=""),"",$K16-$H16))),"")</f>
-      </c>
-      <c r="K16" s="30">
-        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$H16=0),"",IF($I16="",$H16,$H16*(1+$I16))))),"")</f>
+      <c r="F16" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="32">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($H$6:$H$14,$G$6:$G$14,"Marta")),"")</f>
+      </c>
+      <c r="I16" s="33">
+        <f>IFERROR(IF($H16=0,"",$J16/$H16),"")</f>
+      </c>
+      <c r="J16" s="32">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($J$6:$J$14,$G$6:$G$14,"Marta")),"")</f>
+      </c>
+      <c r="K16" s="32">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($K$6:$K$14,$G$6:$G$14,"Marta")),"")</f>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1880,102 +1879,86 @@
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="30">
-        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17))),"")</f>
-      </c>
-      <c r="I17" s="31"/>
-      <c r="J17" s="30">
-        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$K17=""),"",$K17-$H17))),"")</f>
-      </c>
-      <c r="K17" s="30">
-        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$H17=0),"",IF($I17="",$H17,$H17*(1+$I17))))),"")</f>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="32">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="I17" s="33">
+        <f>IFERROR(IF($H17=0,"",$J17/$H17),"")</f>
+      </c>
+      <c r="J17" s="32">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="K17" s="32">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>46317</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F18" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="34"/>
+      <c r="H18" s="35">
+        <f>IFERROR(IF(SUM($H$6:$H$14)=0,"",SUM($H$6:$H$14)),"")</f>
+      </c>
+      <c r="I18" s="36">
+        <f>IFERROR(IF($H18=0,"",$J18/$H18),"")</f>
+      </c>
+      <c r="J18" s="35">
+        <f>IFERROR(IF(SUM($J$6:$J$14)=0,"",SUM($J$6:$J$14)),"")</f>
+      </c>
+      <c r="K18" s="35">
+        <f>IFERROR(IF(SUM($K$6:$K$14)=0,"",SUM($K$6:$K$14)),"")</f>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>46317</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
-      <c r="F19" s="32" t="s">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G19" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="34">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Marta")),"")</f>
-      </c>
-      <c r="I19" s="35">
-        <f>IFERROR(IF($H19=0,"",$J19/$H19),"")</f>
-      </c>
-      <c r="J19" s="34">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($J$6:$J$17,$G$6:$G$17,"Marta")),"")</f>
-      </c>
-      <c r="K19" s="34">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$17,$G$6:$G$17,"Marta")=0,"",SUMIFS($K$6:$K$17,$G$6:$G$17,"Marta")),"")</f>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
-      <c r="F20" s="32" t="s">
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="G20" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="H20" s="34">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="I20" s="35">
-        <f>IFERROR(IF($H20=0,"",$J20/$H20),"")</f>
-      </c>
-      <c r="J20" s="34">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="K20" s="34">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$17,$G$6:$G$17,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$17,$G$6:$G$17,"Fondo ahorro")),"")</f>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="F21" s="36" t="s">
-        <v>32</v>
-      </c>
-      <c r="G21" s="36"/>
-      <c r="H21" s="37">
-        <f>IFERROR(IF(SUM($H$6:$H$17)=0,"",SUM($H$6:$H$17)),"")</f>
-      </c>
-      <c r="I21" s="38">
-        <f>IFERROR(IF($H21=0,"",$J21/$H21),"")</f>
-      </c>
-      <c r="J21" s="37">
-        <f>IFERROR(IF(SUM($J$6:$J$17)=0,"",SUM($J$6:$J$17)),"")</f>
-      </c>
-      <c r="K21" s="37">
-        <f>IFERROR(IF(SUM($K$6:$K$17)=0,"",SUM($K$6:$K$17)),"")</f>
-      </c>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
@@ -1985,35 +1968,21 @@
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="39" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
-      <c r="K23" s="39"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="39"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="39"/>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="11"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
@@ -5872,57 +5841,60 @@
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:K4"/>
-    <mergeCell ref="A23:K23"/>
-    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
   </mergeCells>
   <conditionalFormatting sqref="A6:D505">
     <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND($D6&lt;&gt;"",$D6=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>AND($D5&lt;&gt;"",$D6="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>$D5&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16:K17">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>$F16&lt;&gt;""</formula>
+  <conditionalFormatting sqref="F13:K14">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>$F13&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>AND($F15&lt;&gt;"",$F16="")</formula>
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>AND($F12&lt;&gt;"",$F13="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
-      <formula>$F15=""</formula>
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>$F12=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I16:I17">
-    <cfRule type="expression" dxfId="6" priority="4">
-      <formula>$F16&lt;&gt;""</formula>
+  <conditionalFormatting sqref="I13:I14">
+    <cfRule type="expression" dxfId="7" priority="4">
+      <formula>$F13&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="5">
-      <formula>AND($F15&lt;&gt;"",$F16="")</formula>
+    <cfRule type="expression" dxfId="8" priority="5">
+      <formula>AND($F12&lt;&gt;"",$F13="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F7:K15">
-    <cfRule type="expression" dxfId="8" priority="1">
+  <conditionalFormatting sqref="F7:K12">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>$H7=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F17">
-    <cfRule type="expression" dxfId="9" priority="6">
+  <conditionalFormatting sqref="F9:F14">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="7">
+    <cfRule type="expression" dxfId="11" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J17">
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="I6:J14">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5955,27 +5927,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
+      <c r="A1" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="38"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -6024,7 +5996,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="22" customWidth="1"/>
@@ -6036,27 +6008,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="A1" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="38"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -6073,411 +6045,582 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+    <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="F4" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="K4" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="39"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+    </row>
+    <row r="6" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="F3" s="41" t="s">
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="F7" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="K3" s="41" t="s">
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="K7" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="42"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43" t="s">
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-    </row>
-    <row r="5" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="45" t="s">
-        <v>23</v>
-      </c>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-      <c r="N6" s="45"/>
-    </row>
-    <row r="7" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F8" s="44" t="s">
-        <v>19</v>
-      </c>
+      <c r="F8" s="44"/>
       <c r="G8" s="44"/>
       <c r="H8" s="44"/>
       <c r="I8" s="44"/>
-      <c r="J8" s="43" t="s">
-        <v>44</v>
-      </c>
+      <c r="J8" s="44"/>
       <c r="K8" s="45" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="L8" s="45"/>
       <c r="M8" s="45"/>
       <c r="N8" s="45"/>
     </row>
-    <row r="9" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F10" s="44" t="s">
+    <row r="9" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+    </row>
+    <row r="10" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="43" t="s">
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="K11" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="47"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="43"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="46"/>
+      <c r="K12" s="47"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="47"/>
+      <c r="N12" s="47"/>
+    </row>
+    <row r="13" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="K10" s="45" t="s">
-        <v>22</v>
-      </c>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
-      <c r="N10" s="45"/>
-    </row>
-    <row r="11" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F12" s="44" t="s">
+      <c r="F14" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="K12" s="45" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" s="45"/>
-      <c r="M12" s="45"/>
-      <c r="N12" s="45"/>
-    </row>
-    <row r="13" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F14" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="46" t="s">
-        <v>47</v>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="44" t="s">
+        <v>45</v>
       </c>
       <c r="K14" s="45" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="L14" s="45"/>
       <c r="M14" s="45"/>
       <c r="N14" s="45"/>
     </row>
-    <row r="15" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F16" s="44" t="s">
+    <row r="15" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="43"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+    </row>
+    <row r="16" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="44"/>
-      <c r="H16" s="44"/>
-      <c r="I16" s="44"/>
-      <c r="J16" s="46" t="s">
-        <v>47</v>
-      </c>
-      <c r="K16" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="L16" s="45"/>
-      <c r="M16" s="45"/>
-      <c r="N16" s="45"/>
-    </row>
-    <row r="17" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="22" customHeight="1" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F18" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="44"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="46" t="s">
-        <v>47</v>
-      </c>
-      <c r="K18" s="45" t="s">
-        <v>27</v>
-      </c>
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="K17" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="43"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="45"/>
       <c r="L18" s="45"/>
       <c r="M18" s="45"/>
       <c r="N18" s="45"/>
     </row>
-    <row r="19" ht="5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="22" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="47" t="s">
+    <row r="19" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="F20" s="44"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44"/>
+      <c r="K20" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20" s="45"/>
+      <c r="M20" s="45"/>
+      <c r="N20" s="45"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="43"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="45"/>
+      <c r="L21" s="45"/>
+      <c r="M21" s="45"/>
+      <c r="N21" s="45"/>
+    </row>
+    <row r="22" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="47"/>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="47"/>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="48" t="s">
+      <c r="F23" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="K23" s="45" t="s">
+        <v>23</v>
+      </c>
+      <c r="L23" s="45"/>
+      <c r="M23" s="45"/>
+      <c r="N23" s="45"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="43"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="45"/>
+      <c r="L24" s="45"/>
+      <c r="M24" s="45"/>
+      <c r="N24" s="45"/>
+    </row>
+    <row r="25" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="48"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="48"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="48"/>
+      <c r="M27" s="48"/>
+      <c r="N27" s="48"/>
+      <c r="O27" s="48"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="48"/>
-      <c r="C23" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48" t="s">
+      <c r="B28" s="49"/>
+      <c r="C28" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48"/>
-      <c r="J23" s="48"/>
-      <c r="K23" s="48" t="s">
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" s="49"/>
+      <c r="I28" s="49"/>
+      <c r="J28" s="49"/>
+      <c r="K28" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="L23" s="48"/>
-      <c r="M23" s="48"/>
-      <c r="N23" s="48"/>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="49">
+      <c r="L28" s="49"/>
+      <c r="M28" s="49"/>
+      <c r="N28" s="49"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="50">
         <v>46296</v>
       </c>
-      <c r="B24" s="49"/>
-      <c r="C24" s="50" t="s">
+      <c r="B29" s="50"/>
+      <c r="C29" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="50"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50" t="s">
+      <c r="D29" s="51"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="50"/>
-      <c r="K24" s="51">
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="52">
         <v>1000</v>
       </c>
-      <c r="L24" s="51"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51"/>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="49">
+      <c r="L29" s="52"/>
+      <c r="M29" s="52"/>
+      <c r="N29" s="52"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="50">
         <v>46297</v>
       </c>
-      <c r="B25" s="49"/>
-      <c r="C25" s="50" t="s">
+      <c r="B30" s="50"/>
+      <c r="C30" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50" t="s">
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="51">
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="52">
         <v>300</v>
       </c>
-      <c r="L25" s="51"/>
-      <c r="M25" s="51"/>
-      <c r="N25" s="51"/>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="49">
+      <c r="L30" s="52"/>
+      <c r="M30" s="52"/>
+      <c r="N30" s="52"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="50">
         <v>46297</v>
       </c>
-      <c r="B26" s="49"/>
-      <c r="C26" s="50" t="s">
+      <c r="B31" s="50"/>
+      <c r="C31" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="50"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="50"/>
-      <c r="G26" s="50" t="s">
+      <c r="D31" s="51"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="50"/>
-      <c r="K26" s="51">
+      <c r="H31" s="51"/>
+      <c r="I31" s="51"/>
+      <c r="J31" s="51"/>
+      <c r="K31" s="52">
         <v>200</v>
       </c>
-      <c r="L26" s="51"/>
-      <c r="M26" s="51"/>
-      <c r="N26" s="51"/>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="49">
+      <c r="L31" s="52"/>
+      <c r="M31" s="52"/>
+      <c r="N31" s="52"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="50">
         <v>46298</v>
       </c>
-      <c r="B27" s="49"/>
-      <c r="C27" s="50" t="s">
+      <c r="B32" s="50"/>
+      <c r="C32" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="51"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="51"/>
+      <c r="K32" s="52">
+        <v>120</v>
+      </c>
+      <c r="L32" s="52"/>
+      <c r="M32" s="52"/>
+      <c r="N32" s="52"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="50">
+        <v>46298</v>
+      </c>
+      <c r="B33" s="50"/>
+      <c r="C33" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" s="50"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="50"/>
-      <c r="K27" s="51">
+      <c r="D33" s="51"/>
+      <c r="E33" s="51"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="H33" s="51"/>
+      <c r="I33" s="51"/>
+      <c r="J33" s="51"/>
+      <c r="K33" s="52">
         <v>400</v>
       </c>
-      <c r="L27" s="51"/>
-      <c r="M27" s="51"/>
-      <c r="N27" s="51"/>
-    </row>
-    <row r="28" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="49">
+      <c r="L33" s="52"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="50">
         <v>46300</v>
       </c>
-      <c r="B28" s="49"/>
-      <c r="C28" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
-      <c r="F28" s="50"/>
-      <c r="G28" s="50" t="s">
-        <v>24</v>
-      </c>
-      <c r="H28" s="50"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="51">
+      <c r="B34" s="50"/>
+      <c r="C34" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="51"/>
+      <c r="E34" s="51"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="H34" s="51"/>
+      <c r="I34" s="51"/>
+      <c r="J34" s="51"/>
+      <c r="K34" s="52">
         <v>150</v>
       </c>
-      <c r="L28" s="51"/>
-      <c r="M28" s="51"/>
-      <c r="N28" s="51"/>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="52" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
-      <c r="I29" s="52"/>
-      <c r="J29" s="52"/>
-      <c r="K29" s="53">
-        <v>2050</v>
-      </c>
-      <c r="L29" s="53"/>
-      <c r="M29" s="53"/>
-      <c r="N29" s="53"/>
+      <c r="L34" s="52"/>
+      <c r="M34" s="52"/>
+      <c r="N34" s="52"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="53" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
+      <c r="J35" s="53"/>
+      <c r="K35" s="54">
+        <v>2170</v>
+      </c>
+      <c r="L35" s="54"/>
+      <c r="M35" s="54"/>
+      <c r="N35" s="54"/>
     </row>
   </sheetData>
-  <mergeCells count="49">
+  <mergeCells count="64">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:J6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="K12:N12"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="A22:O22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="K23:N23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K24:N24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="A4:D5"/>
+    <mergeCell ref="F4:I5"/>
+    <mergeCell ref="K4:N5"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="A8:D9"/>
+    <mergeCell ref="E8:J9"/>
+    <mergeCell ref="K8:N9"/>
+    <mergeCell ref="A11:D12"/>
+    <mergeCell ref="F11:I12"/>
+    <mergeCell ref="K11:N12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A14:D15"/>
+    <mergeCell ref="F14:I15"/>
+    <mergeCell ref="K14:N15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="A17:D18"/>
+    <mergeCell ref="F17:I18"/>
+    <mergeCell ref="K17:N18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="A20:D21"/>
+    <mergeCell ref="E20:J21"/>
+    <mergeCell ref="K20:N21"/>
+    <mergeCell ref="A23:D24"/>
+    <mergeCell ref="F23:I24"/>
+    <mergeCell ref="K23:N24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="A27:O27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="K28:N28"/>
-    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
     <mergeCell ref="K29:N29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="K32:N32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="G34:J34"/>
+    <mergeCell ref="K34:N34"/>
+    <mergeCell ref="A35:J35"/>
+    <mergeCell ref="K35:N35"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Ordenar movimientos, limitar salidas y sustituir barras por flujo origen-pasos-final
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -5,22 +5,20 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Gráficos" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Flujo" state="visible" r:id="rId6"/>
+    <sheet sheetId="2" name="Flujo" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$14),1),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O22</definedName>
+    <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Flujo'!$A1:$O35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Flujo'!$A1:$O33</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="58">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -118,16 +116,10 @@
     <t>En las inversiones se escribe la rentabilidad en % (la celda amarilla, como en la app) y el saldo se calcula solo. «Exterior» es el dinero que entra o sale de fuera. La hoja está protegida: solo se puede escribir en los movimientos, en las filas nuevas y en el %.</t>
   </si>
   <si>
-    <t>Gráficos</t>
-  </si>
-  <si>
-    <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
-  </si>
-  <si>
     <t>Flujo del dinero</t>
   </si>
   <si>
-    <t>Cada línea es el viaje del dinero: de dónde sale, por dónde pasa y dónde acaba. Se dibuja con los movimientos de hoy: vuelve a descargar el Excel para tenerlo al día.</t>
+    <t>Gris: lo que llega de fuera · Azul: la cuenta por la que pasa · Verde: donde está hoy. Cada camino es más grueso cuanto más dinero lleva. Se dibuja con los movimientos de hoy.</t>
   </si>
   <si>
     <t xml:space="preserve">Entra de fuera
@@ -142,34 +134,63 @@
 1170,00 €</t>
   </si>
   <si>
-    <t>DE DÓNDE LLEGA</t>
+    <t>ORIGEN</t>
   </si>
   <si>
-    <t>POR DÓNDE PASA</t>
+    <t>PASOS</t>
   </si>
   <si>
-    <t>A DÓNDE VA</t>
+    <t>FINAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exterior
+1550,00 €</t>
+  </si>
+  <si>
+    <t>380,00 €   ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuenta Myinvestor
+1000,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigue en la cuenta
+380,00 €</t>
+  </si>
+  <si>
+    <t>300,00 €   ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanguard Global Stock Index
+300,00 €</t>
+  </si>
+  <si>
+    <t>200,00 €   ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fidelity MSCI World Index
+200,00 €</t>
+  </si>
+  <si>
+    <t>120,00 €   ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartera indexada Metal
+120,00 €</t>
   </si>
   <si>
     <t>400,00 €   ▶▶▶</t>
   </si>
   <si>
-    <t>380,00 €   ▶</t>
-  </si>
-  <si>
-    <t>Sigue en la cuenta</t>
-  </si>
-  <si>
-    <t>300,00 €   ▶</t>
-  </si>
-  <si>
-    <t>200,00 €   ▶</t>
+    <t xml:space="preserve">Fondo indexado
+400,00 €</t>
   </si>
   <si>
     <t>150,00 €   ▶▶▶</t>
   </si>
   <si>
-    <t>120,00 €   ▶</t>
+    <t xml:space="preserve">iShares Developed World Index
+150,00 €</t>
   </si>
   <si>
     <t>Movimientos, uno a uno</t>
@@ -354,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -396,12 +417,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
@@ -462,20 +482,11 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -502,7 +513,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FFFFFFFF"/>
@@ -606,6 +617,13 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFBEB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FFFFFFFF"/>
         <sz val="10"/>
@@ -642,519 +660,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="334155"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Marta</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Aportado</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="2563EB"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Marta</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$H$16</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Rentabilidad</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="E67E22"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Marta</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$J$16</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Aportado + rentabilidad</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="0F766E"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Marta</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$K$16</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="-80"/>
-        <c:axId val="100000001"/>
-        <c:axId val="100000002"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="100000001"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000002"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="100000002"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000001"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln>
-      <a:solidFill>
-        <a:srgbClr val="D8DEE9"/>
-      </a:solidFill>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0">
-                <a:solidFill>
-                  <a:srgbClr val="334155"/>
-                </a:solidFill>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Fondo ahorro</a:t>
-            </a:r>
-            <a:endParaRPr/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Aportado</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="2563EB"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Fondo ahorro</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$H$17</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Rentabilidad</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="E67E22"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Fondo ahorro</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$J$17</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Aportado + rentabilidad</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="0F766E"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:numFmt formatCode="#,##0.00 &quot;€&quot;" sourceLinked="0"/>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Fondo ahorro</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Movimientos!$K$17</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:gapWidth val="60"/>
-        <c:overlap val="-80"/>
-        <c:axId val="100000001"/>
-        <c:axId val="100000002"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="100000001"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000002"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="100000002"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100000001"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln>
-      <a:solidFill>
-        <a:srgbClr val="D8DEE9"/>
-      </a:solidFill>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Grafico 1"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Grafico 2"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1644,14 +1149,12 @@
       <c r="H7" s="16">
         <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
       </c>
-      <c r="I7" s="17">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7=0,$H7=""),"",$J7/$H7))),"")</f>
-      </c>
+      <c r="I7" s="17"/>
       <c r="J7" s="16">
         <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
       </c>
       <c r="K7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$H7=0),"",IF($I7="",$H7,$H7*(1+$I7))))),"")</f>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1676,7 +1179,7 @@
       <c r="H8" s="16">
         <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index"))),"")</f>
       </c>
-      <c r="I8" s="19"/>
+      <c r="I8" s="17"/>
       <c r="J8" s="16">
         <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",IF(OR($H8="",$K8=""),"",$K8-$H8))),"")</f>
       </c>
@@ -1697,20 +1200,20 @@
       <c r="D9" s="11">
         <v>120</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="19" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="20">
         <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index"))),"")</f>
       </c>
-      <c r="I9" s="22"/>
-      <c r="J9" s="21">
+      <c r="I9" s="21"/>
+      <c r="J9" s="20">
         <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",IF(OR($H9="",$K9=""),"",$K9-$H9))),"")</f>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="20">
         <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",IF(OR($H9="",$H9=0),"",IF($I9="",$H9,$H9*(1+$I9))))),"")</f>
       </c>
     </row>
@@ -1727,20 +1230,20 @@
       <c r="D10" s="11">
         <v>400</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="19" t="s">
         <v>23</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="20">
         <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal"))),"")</f>
       </c>
-      <c r="I10" s="22"/>
-      <c r="J10" s="21">
+      <c r="I10" s="21"/>
+      <c r="J10" s="20">
         <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",IF(OR($H10="",$K10=""),"",$K10-$H10))),"")</f>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="20">
         <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",IF(OR($H10="",$H10=0),"",IF($I10="",$H10,$H10*(1+$I10))))),"")</f>
       </c>
     </row>
@@ -1757,20 +1260,20 @@
       <c r="D11" s="11">
         <v>150</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="22" t="s">
         <v>24</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="23">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
       </c>
-      <c r="I11" s="25"/>
-      <c r="J11" s="24">
+      <c r="I11" s="24"/>
+      <c r="J11" s="23">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H11="",$K11=""),"",$K11-$H11))),"")</f>
       </c>
-      <c r="K11" s="24">
+      <c r="K11" s="23">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",IF(OR($H11="",$H11=0),"",IF($I11="",$H11,$H11*(1+$I11))))),"")</f>
       </c>
     </row>
@@ -1781,20 +1284,20 @@
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="11"/>
-      <c r="F12" s="23" t="s">
+      <c r="F12" s="22" t="s">
         <v>25</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="23">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
       </c>
-      <c r="I12" s="25"/>
-      <c r="J12" s="24">
+      <c r="I12" s="24"/>
+      <c r="J12" s="23">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H12="",$K12=""),"",$K12-$H12))),"")</f>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="23">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",IF(OR($H12="",$H12=0),"",IF($I12="",$H12,$H12*(1+$I12))))),"")</f>
       </c>
     </row>
@@ -1805,16 +1308,16 @@
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="28">
+      <c r="F13" s="25"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="27">
         <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13))),"")</f>
       </c>
-      <c r="I13" s="29"/>
-      <c r="J13" s="28">
+      <c r="I13" s="28"/>
+      <c r="J13" s="27">
         <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",IF(OR($H13="",$K13=""),"",$K13-$H13))),"")</f>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="27">
         <f>IFERROR(IF($F13="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F13)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F13)&lt;=0),"",IF(OR($H13="",$H13=0),"",IF($I13="",$H13,$H13*(1+$I13))))),"")</f>
       </c>
     </row>
@@ -1825,26 +1328,38 @@
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="11"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="28">
+      <c r="F14" s="25"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="27">
         <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14))),"")</f>
       </c>
-      <c r="I14" s="29"/>
-      <c r="J14" s="28">
+      <c r="I14" s="28"/>
+      <c r="J14" s="27">
         <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",IF(OR($H14="",$K14=""),"",$K14-$H14))),"")</f>
       </c>
-      <c r="K14" s="28">
+      <c r="K14" s="27">
         <f>IFERROR(IF($F14="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F14)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F14)&lt;=0),"",IF(OR($H14="",$H14=0),"",IF($I14="",$H14,$H14*(1+$I14))))),"")</f>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>46317</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="11"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="27">
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15))),"")</f>
+      </c>
+      <c r="I15" s="28"/>
+      <c r="J15" s="27">
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15)&lt;=0),"",IF(OR($H15="",$K15=""),"",$K15-$H15))),"")</f>
+      </c>
+      <c r="K15" s="27">
+        <f>IFERROR(IF($F15="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F15)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F15)&lt;=0),"",IF(OR($H15="",$H15=0),"",IF($I15="",$H15,$H15*(1+$I15))))),"")</f>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
@@ -1853,23 +1368,17 @@
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
-      <c r="F16" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" s="32">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($H$6:$H$14,$G$6:$G$14,"Marta")),"")</f>
-      </c>
-      <c r="I16" s="33">
-        <f>IFERROR(IF($H16=0,"",$J16/$H16),"")</f>
-      </c>
-      <c r="J16" s="32">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($J$6:$J$14,$G$6:$G$14,"Marta")),"")</f>
-      </c>
-      <c r="K16" s="32">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$14,$G$6:$G$14,"Marta")=0,"",SUMIFS($K$6:$K$14,$G$6:$G$14,"Marta")),"")</f>
+      <c r="F16" s="25"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="27">
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16))),"")</f>
+      </c>
+      <c r="I16" s="28"/>
+      <c r="J16" s="27">
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$K16=""),"",$K16-$H16))),"")</f>
+      </c>
+      <c r="K16" s="27">
+        <f>IFERROR(IF($F16="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F16)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F16)&lt;=0),"",IF(OR($H16="",$H16=0),"",IF($I16="",$H16,$H16*(1+$I16))))),"")</f>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1879,102 +1388,142 @@
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
-      <c r="F17" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="G17" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" s="32">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="I17" s="33">
-        <f>IFERROR(IF($H17=0,"",$J17/$H17),"")</f>
-      </c>
-      <c r="J17" s="32">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
-      </c>
-      <c r="K17" s="32">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$14,$G$6:$G$14,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$14,$G$6:$G$14,"Fondo ahorro")),"")</f>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F17" s="25"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="27">
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17))),"")</f>
+      </c>
+      <c r="I17" s="28"/>
+      <c r="J17" s="27">
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$K17=""),"",$K17-$H17))),"")</f>
+      </c>
+      <c r="K17" s="27">
+        <f>IFERROR(IF($F17="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F17)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F17)&lt;=0),"",IF(OR($H17="",$H17=0),"",IF($I17="",$H17,$H17*(1+$I17))))),"")</f>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>46317</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
-      <c r="F18" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="G18" s="34"/>
-      <c r="H18" s="35">
-        <f>IFERROR(IF(SUM($H$6:$H$14)=0,"",SUM($H$6:$H$14)),"")</f>
-      </c>
-      <c r="I18" s="36">
-        <f>IFERROR(IF($H18=0,"",$J18/$H18),"")</f>
-      </c>
-      <c r="J18" s="35">
-        <f>IFERROR(IF(SUM($J$6:$J$14)=0,"",SUM($J$6:$J$14)),"")</f>
-      </c>
-      <c r="K18" s="35">
-        <f>IFERROR(IF(SUM($K$6:$K$14)=0,"",SUM($K$6:$K$14)),"")</f>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" s="25"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="27">
+        <f>IFERROR(IF($F18="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18))),"")</f>
+      </c>
+      <c r="I18" s="28"/>
+      <c r="J18" s="27">
+        <f>IFERROR(IF($F18="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18)&lt;=0),"",IF(OR($H18="",$K18=""),"",$K18-$H18))),"")</f>
+      </c>
+      <c r="K18" s="27">
+        <f>IFERROR(IF($F18="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F18)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F18)&lt;=0),"",IF(OR($H18="",$H18=0),"",IF($I18="",$H18,$H18*(1+$I18))))),"")</f>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>46317</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="37" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="37"/>
-      <c r="K20" s="37"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="27">
+        <f>IFERROR(IF($F19="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19)&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19))),"")</f>
+      </c>
+      <c r="I19" s="28"/>
+      <c r="J19" s="27">
+        <f>IFERROR(IF($F19="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19)&lt;=0),"",IF(OR($H19="",$K19=""),"",$K19-$H19))),"")</f>
+      </c>
+      <c r="K19" s="27">
+        <f>IFERROR(IF($F19="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,$F19)-SUMIFS($D$6:$D$505,$B$6:$B$505,$F19)&lt;=0),"",IF(OR($H19="",$H19=0),"",IF($I19="",$H19,$H19*(1+$I19))))),"")</f>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="37"/>
-      <c r="K21" s="37"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="9">
+        <v>46317</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="11"/>
+      <c r="F21" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="31">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Marta")),"")</f>
+      </c>
+      <c r="I21" s="32">
+        <f>IFERROR(IF($H21=0,"",$J21/$H21),"")</f>
+      </c>
+      <c r="J21" s="31">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($J$6:$J$19,$G$6:$G$19,"Marta")),"")</f>
+      </c>
+      <c r="K21" s="31">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($K$6:$K$19,$G$6:$G$19,"Marta")),"")</f>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>46317</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F22" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="31">
+        <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="I22" s="32">
+        <f>IFERROR(IF($H22=0,"",$J22/$H22),"")</f>
+      </c>
+      <c r="J22" s="31">
+        <f>IFERROR(IF(SUMIFS($J$6:$J$19,$G$6:$G$19,"Fondo ahorro")=0,"",SUMIFS($J$6:$J$19,$G$6:$G$19,"Fondo ahorro")),"")</f>
+      </c>
+      <c r="K22" s="31">
+        <f>IFERROR(IF(SUMIFS($K$6:$K$19,$G$6:$G$19,"Fondo ahorro")=0,"",SUMIFS($K$6:$K$19,$G$6:$G$19,"Fondo ahorro")),"")</f>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>46317</v>
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
+      <c r="F23" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="G23" s="33"/>
+      <c r="H23" s="34">
+        <f>IFERROR(IF(SUM($H$6:$H$19)=0,"",SUM($H$6:$H$19)),"")</f>
+      </c>
+      <c r="I23" s="35">
+        <f>IFERROR(IF($H23=0,"",$J23/$H23),"")</f>
+      </c>
+      <c r="J23" s="34">
+        <f>IFERROR(IF(SUM($J$6:$J$19)=0,"",SUM($J$6:$J$19)),"")</f>
+      </c>
+      <c r="K23" s="34">
+        <f>IFERROR(IF(SUM($K$6:$K$19)=0,"",SUM($K$6:$K$19)),"")</f>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
@@ -1984,21 +1533,35 @@
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="11"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="11"/>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
+      <c r="J26" s="36"/>
+      <c r="K26" s="36"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
@@ -5841,8 +5404,8 @@
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:K4"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="A6:D505">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -5858,7 +5421,7 @@
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F13:K14">
+  <conditionalFormatting sqref="F13:K19">
     <cfRule type="expression" dxfId="4" priority="1">
       <formula>$F13&lt;&gt;""</formula>
     </cfRule>
@@ -5869,32 +5432,37 @@
       <formula>$F12=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I13:I14">
+  <conditionalFormatting sqref="I7:I12">
     <cfRule type="expression" dxfId="7" priority="4">
+      <formula>AND($F7&lt;&gt;"",$H7&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I13:I19">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>$F13&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>AND($F12&lt;&gt;"",$F13="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F7:K12">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="10" priority="1">
       <formula>$H7=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F14">
-    <cfRule type="expression" dxfId="10" priority="6">
+  <conditionalFormatting sqref="F9:F19">
+    <cfRule type="expression" dxfId="11" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="12" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:J14">
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="I6:J19">
+    <cfRule type="cellIs" dxfId="13" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5905,8 +5473,8 @@
     <dataValidation type="list" allowBlank="1" sqref="C6:C505">
       <formula1>ListaNombres</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" sqref="D6:D505">
-      <formula1>0</formula1>
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="No hay tanto dinero" error="En la cuenta o inversión de la que sale el dinero no queda tanto. Escribe un importe más pequeño o mete antes el dinero desde el Exterior." sqref="D6:D505">
+      <formula1>OR($D6=0,AND($D6&gt;0,OR($B6="Exterior",$D6&lt;=MAX(0,(SUMIFS($D$6:$D6,$C$6:$C6,$B6)-SUMIFS($D$6:$D6,$B$6:$B6,$B6)+$D6)*(1+IFERROR(VLOOKUP($B6,$F$6:$I$19,4,FALSE),0))))))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
@@ -5920,32 +5488,37 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="15" width="15" customWidth="1"/>
+    <col min="1" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+    <row r="1" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>33</v>
       </c>
@@ -5964,599 +5537,573 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-  </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FF1D4ED8"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="3" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-    </row>
     <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="F4" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="K4" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="F4" s="40" t="s">
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="38"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
+      <c r="M5" s="40"/>
+      <c r="N5" s="40"/>
+    </row>
+    <row r="6" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="18" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="K4" s="41" t="s">
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="F7" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="L4" s="41"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="41"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-    </row>
-    <row r="6" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="42" t="s">
+      <c r="G7" s="41"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="K7" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
-      <c r="F7" s="42" t="s">
+      <c r="L7" s="41"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="41"/>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="K7" s="42" t="s">
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+      <c r="F8" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="K8" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="38"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="39"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="38"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="39"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43"/>
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="38"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="38"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="40"/>
+    </row>
+    <row r="13" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="38"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="40"/>
+      <c r="M13" s="40"/>
+      <c r="N13" s="40"/>
+    </row>
+    <row r="14" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="38"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
+      <c r="N14" s="40"/>
+    </row>
+    <row r="15" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="38"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="39"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="39"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="K15" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="L15" s="40"/>
+      <c r="M15" s="40"/>
+      <c r="N15" s="40"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="38"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="40"/>
+      <c r="M16" s="40"/>
+      <c r="N16" s="40"/>
+    </row>
+    <row r="17" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="38"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="39"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="K17" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="40"/>
+      <c r="M17" s="40"/>
+      <c r="N17" s="40"/>
+    </row>
+    <row r="18" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="38"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
+    </row>
+    <row r="19" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="38"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="42" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="L19" s="40"/>
+      <c r="M19" s="40"/>
+      <c r="N19" s="40"/>
+    </row>
+    <row r="20" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="38"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="40"/>
+      <c r="M20" s="40"/>
+      <c r="N20" s="40"/>
+    </row>
+    <row r="21" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="38"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="40"/>
+      <c r="M21" s="40"/>
+      <c r="N21" s="40"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="38"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
+      <c r="N22" s="40"/>
+    </row>
+    <row r="23" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="38"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="42" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="L23" s="40"/>
+      <c r="M23" s="40"/>
+      <c r="N23" s="40"/>
+    </row>
+    <row r="24" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="38"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="42"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="40"/>
+      <c r="M24" s="40"/>
+      <c r="N24" s="40"/>
+    </row>
+    <row r="25" ht="16" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="44"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="44"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="44"/>
+      <c r="O25" s="44"/>
+    </row>
+    <row r="26" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="H26" s="45"/>
+      <c r="I26" s="45"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="L26" s="45"/>
+      <c r="M26" s="45"/>
+      <c r="N26" s="45"/>
+    </row>
+    <row r="27" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="46">
+        <v>46296</v>
+      </c>
+      <c r="B27" s="46"/>
+      <c r="C27" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="44"/>
-      <c r="J8" s="44"/>
-      <c r="K8" s="45" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" s="45"/>
-      <c r="M8" s="45"/>
-      <c r="N8" s="45"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="43"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="45"/>
-      <c r="M9" s="45"/>
-      <c r="N9" s="45"/>
-    </row>
-    <row r="10" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="46" t="s">
+      <c r="D27" s="47"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="K11" s="47" t="s">
-        <v>44</v>
-      </c>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="47"/>
-    </row>
-    <row r="13" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="F14" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="K14" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
-      <c r="N14" s="45"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="43"/>
-      <c r="B15" s="43"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="44"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
-      <c r="N15" s="45"/>
-    </row>
-    <row r="16" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="F17" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-      <c r="J17" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="K17" s="45" t="s">
-        <v>22</v>
-      </c>
-      <c r="L17" s="45"/>
-      <c r="M17" s="45"/>
-      <c r="N17" s="45"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="43"/>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="45"/>
-    </row>
-    <row r="19" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="44" t="s">
-        <v>47</v>
-      </c>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="45" t="s">
-        <v>25</v>
-      </c>
-      <c r="L20" s="45"/>
-      <c r="M20" s="45"/>
-      <c r="N20" s="45"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="43"/>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="44"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="44"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="45"/>
-    </row>
-    <row r="22" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="K23" s="45" t="s">
-        <v>23</v>
-      </c>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="43"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="45"/>
-      <c r="M24" s="45"/>
-      <c r="N24" s="45"/>
-    </row>
-    <row r="25" ht="7" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="47"/>
+      <c r="K27" s="48">
+        <v>1000</v>
+      </c>
       <c r="L27" s="48"/>
       <c r="M27" s="48"/>
       <c r="N27" s="48"/>
-      <c r="O27" s="48"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="49" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" s="49"/>
-      <c r="C28" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" s="49"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="49" t="s">
-        <v>51</v>
-      </c>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="L28" s="49"/>
-      <c r="M28" s="49"/>
-      <c r="N28" s="49"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="50">
-        <v>46296</v>
-      </c>
-      <c r="B29" s="50"/>
-      <c r="C29" s="51" t="s">
+    </row>
+    <row r="28" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="46">
+        <v>46297</v>
+      </c>
+      <c r="B28" s="46"/>
+      <c r="C28" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="48">
+        <v>300</v>
+      </c>
+      <c r="L28" s="48"/>
+      <c r="M28" s="48"/>
+      <c r="N28" s="48"/>
+    </row>
+    <row r="29" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="46">
+        <v>46297</v>
+      </c>
+      <c r="B29" s="46"/>
+      <c r="C29" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="47"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="47"/>
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="48">
+        <v>200</v>
+      </c>
+      <c r="L29" s="48"/>
+      <c r="M29" s="48"/>
+      <c r="N29" s="48"/>
+    </row>
+    <row r="30" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="46">
+        <v>46298</v>
+      </c>
+      <c r="B30" s="46"/>
+      <c r="C30" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="47"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="H30" s="47"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="48">
+        <v>120</v>
+      </c>
+      <c r="L30" s="48"/>
+      <c r="M30" s="48"/>
+      <c r="N30" s="48"/>
+    </row>
+    <row r="31" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="46">
+        <v>46298</v>
+      </c>
+      <c r="B31" s="46"/>
+      <c r="C31" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="51"/>
-      <c r="E29" s="51"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="52">
-        <v>1000</v>
-      </c>
-      <c r="L29" s="52"/>
-      <c r="M29" s="52"/>
-      <c r="N29" s="52"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="50">
-        <v>46297</v>
-      </c>
-      <c r="B30" s="50"/>
-      <c r="C30" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="D30" s="51"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="51"/>
-      <c r="G30" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="H30" s="51"/>
-      <c r="I30" s="51"/>
-      <c r="J30" s="51"/>
-      <c r="K30" s="52">
-        <v>300</v>
-      </c>
-      <c r="L30" s="52"/>
-      <c r="M30" s="52"/>
-      <c r="N30" s="52"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="50">
-        <v>46297</v>
-      </c>
-      <c r="B31" s="50"/>
-      <c r="C31" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="D31" s="51"/>
-      <c r="E31" s="51"/>
-      <c r="F31" s="51"/>
-      <c r="G31" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="H31" s="51"/>
-      <c r="I31" s="51"/>
-      <c r="J31" s="51"/>
-      <c r="K31" s="52">
-        <v>200</v>
-      </c>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="50">
-        <v>46298</v>
-      </c>
-      <c r="B32" s="50"/>
-      <c r="C32" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="D32" s="51"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="51" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
-      <c r="J32" s="51"/>
-      <c r="K32" s="52">
-        <v>120</v>
-      </c>
-      <c r="L32" s="52"/>
-      <c r="M32" s="52"/>
-      <c r="N32" s="52"/>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="50">
-        <v>46298</v>
-      </c>
-      <c r="B33" s="50"/>
-      <c r="C33" s="51" t="s">
+      <c r="D31" s="47"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="47"/>
+      <c r="G31" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
+      <c r="K31" s="48">
+        <v>400</v>
+      </c>
+      <c r="L31" s="48"/>
+      <c r="M31" s="48"/>
+      <c r="N31" s="48"/>
+    </row>
+    <row r="32" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="46">
+        <v>46300</v>
+      </c>
+      <c r="B32" s="46"/>
+      <c r="C32" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="51"/>
-      <c r="E33" s="51"/>
-      <c r="F33" s="51"/>
-      <c r="G33" s="51" t="s">
-        <v>24</v>
-      </c>
-      <c r="H33" s="51"/>
-      <c r="I33" s="51"/>
-      <c r="J33" s="51"/>
-      <c r="K33" s="52">
-        <v>400</v>
-      </c>
-      <c r="L33" s="52"/>
-      <c r="M33" s="52"/>
-      <c r="N33" s="52"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="50">
-        <v>46300</v>
-      </c>
-      <c r="B34" s="50"/>
-      <c r="C34" s="51" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="51"/>
-      <c r="E34" s="51"/>
-      <c r="F34" s="51"/>
-      <c r="G34" s="51" t="s">
+      <c r="D32" s="47"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="H34" s="51"/>
-      <c r="I34" s="51"/>
-      <c r="J34" s="51"/>
-      <c r="K34" s="52">
+      <c r="H32" s="47"/>
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="48">
         <v>150</v>
       </c>
-      <c r="L34" s="52"/>
-      <c r="M34" s="52"/>
-      <c r="N34" s="52"/>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A35" s="53" t="s">
-        <v>52</v>
-      </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="53"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="53"/>
-      <c r="I35" s="53"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="54">
+      <c r="L32" s="48"/>
+      <c r="M32" s="48"/>
+      <c r="N32" s="48"/>
+    </row>
+    <row r="33" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="49"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="49"/>
+      <c r="J33" s="49"/>
+      <c r="K33" s="50">
         <v>2170</v>
       </c>
-      <c r="L35" s="54"/>
-      <c r="M35" s="54"/>
-      <c r="N35" s="54"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="50"/>
     </row>
   </sheetData>
-  <mergeCells count="64">
+  <mergeCells count="56">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A4:D5"/>
@@ -6565,32 +6112,32 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="K7:N7"/>
-    <mergeCell ref="A8:D9"/>
-    <mergeCell ref="E8:J9"/>
-    <mergeCell ref="K8:N9"/>
-    <mergeCell ref="A11:D12"/>
-    <mergeCell ref="F11:I12"/>
-    <mergeCell ref="K11:N12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A14:D15"/>
-    <mergeCell ref="F14:I15"/>
-    <mergeCell ref="K14:N15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="A17:D18"/>
-    <mergeCell ref="F17:I18"/>
+    <mergeCell ref="A8:D24"/>
+    <mergeCell ref="F8:I18"/>
+    <mergeCell ref="K8:N11"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="K12:N14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="J12:J14"/>
+    <mergeCell ref="K15:N16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="J15:J16"/>
     <mergeCell ref="K17:N18"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="J17:J18"/>
-    <mergeCell ref="A20:D21"/>
-    <mergeCell ref="E20:J21"/>
-    <mergeCell ref="K20:N21"/>
-    <mergeCell ref="A23:D24"/>
-    <mergeCell ref="F23:I24"/>
+    <mergeCell ref="E19:J22"/>
+    <mergeCell ref="K19:N22"/>
+    <mergeCell ref="E23:J24"/>
     <mergeCell ref="K23:N24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="A27:O27"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:N27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="G28:J28"/>
@@ -6611,16 +6158,8 @@
     <mergeCell ref="C32:F32"/>
     <mergeCell ref="G32:J32"/>
     <mergeCell ref="K32:N32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="A33:J33"/>
     <mergeCell ref="K33:N33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="G34:J34"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="A35:J35"/>
-    <mergeCell ref="K35:N35"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Recuperar gráficos de cuentas y crear mapa del dinero sin hoja Flujo
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -5,20 +5,22 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Flujo" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Gráficos" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Mapa del dinero" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Flujo'!$A1:$O33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Mapa del dinero'!$A1:$O35</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="63">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -113,96 +115,115 @@
     <t>Para añadir una inversión: escribe su nombre (y su titular) en la fila amarilla; al rellenarla sale la siguiente. Para quitarla: borra su nombre y desaparece. Entra al momento en los desplegables.</t>
   </si>
   <si>
-    <t>En las inversiones se escribe la rentabilidad en % (la celda amarilla, como en la app) y el saldo se calcula solo. «Exterior» es el dinero que entra o sale de fuera. La hoja está protegida: solo se puede escribir en los movimientos, en las filas nuevas y en el %.</t>
+    <t>La rentabilidad de cada cuenta o inversión se escribe en %. Para quitar un movimiento de este .xlsx, borra De, A e Importe y pon la fecha de hoy: escribir 0 solo oculta los datos. Al volver a descargar el Excel desde la app, los movimientos a cero se omiten de verdad.</t>
   </si>
   <si>
-    <t>Flujo del dinero</t>
+    <t>Gráficos</t>
   </si>
   <si>
-    <t>Gris: lo que llega de fuera · Azul: la cuenta por la que pasa · Verde: donde está hoy. Cada camino es más grueso cuanto más dinero lleva. Se dibuja con los movimientos de hoy.</t>
+    <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
   </si>
   <si>
-    <t xml:space="preserve">Entra de fuera
+    <t>Mapa del dinero</t>
+  </si>
+  <si>
+    <t>Lee cada recorrido de izquierda a derecha: origen → paso intermedio → destino. Una banda más larga significa más dinero.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENTRA DE FUERA
 1550,00 €</t>
   </si>
   <si>
-    <t xml:space="preserve">Sigue en las cuentas
+    <t xml:space="preserve">SIGUE EN CUENTAS
 380,00 €</t>
   </si>
   <si>
-    <t xml:space="preserve">Invertido
+    <t xml:space="preserve">ESTÁ INVERTIDO
 1170,00 €</t>
   </si>
   <si>
     <t>ORIGEN</t>
   </si>
   <si>
-    <t>PASOS</t>
+    <t>PASO INTERMEDIO</t>
   </si>
   <si>
-    <t>FINAL</t>
+    <t>DESTINO FINAL</t>
   </si>
   <si>
     <t xml:space="preserve">Exterior
-1550,00 €</t>
+400,00 €</t>
   </si>
   <si>
-    <t>380,00 €   ▶</t>
+    <t>400,00 €  ▶</t>
   </si>
   <si>
-    <t xml:space="preserve">Cuenta Myinvestor
-1000,00 €</t>
+    <t>Sin cuenta intermedia</t>
   </si>
   <si>
-    <t xml:space="preserve">Sigue en la cuenta
+    <t>▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondo indexado
+400,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exterior
 380,00 €</t>
   </si>
   <si>
-    <t>300,00 €   ▶</t>
+    <t>380,00 €  ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigue en Cuenta Myinvestor
+380,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exterior
+300,00 €</t>
+  </si>
+  <si>
+    <t>300,00 €  ▶</t>
   </si>
   <si>
     <t xml:space="preserve">Vanguard Global Stock Index
 300,00 €</t>
   </si>
   <si>
-    <t>200,00 €   ▶</t>
+    <t xml:space="preserve">Exterior
+200,00 €</t>
+  </si>
+  <si>
+    <t>200,00 €  ▶</t>
   </si>
   <si>
     <t xml:space="preserve">Fidelity MSCI World Index
 200,00 €</t>
   </si>
   <si>
-    <t>120,00 €   ▶</t>
+    <t xml:space="preserve">Exterior
+150,00 €</t>
+  </si>
+  <si>
+    <t>150,00 €  ▶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iShares Developed World Index
+150,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exterior
+120,00 €</t>
+  </si>
+  <si>
+    <t>120,00 €  ▶</t>
   </si>
   <si>
     <t xml:space="preserve">Cartera indexada Metal
 120,00 €</t>
   </si>
   <si>
-    <t>400,00 €   ▶▶▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fondo indexado
-400,00 €</t>
-  </si>
-  <si>
-    <t>150,00 €   ▶▶▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iShares Developed World Index
-150,00 €</t>
-  </si>
-  <si>
-    <t>Movimientos, uno a uno</t>
-  </si>
-  <si>
-    <t>De</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Total de los 6 movimientos</t>
+    <t>El mapa refleja los movimientos al descargar el Excel. Para actualizarlo tras editarlo, vuelve a descargarlo desde la app.</t>
   </si>
 </sst>
 </file>
@@ -298,25 +319,26 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF64748B"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1D4ED8"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <color rgb="FF64748B"/>
+      <color rgb="FF0F766E"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="12"/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -345,12 +367,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF64748B"/>
+        <fgColor rgb="FF475569"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF14B8A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -470,45 +512,41 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -660,6 +698,579 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="334155"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000"/>
+              <a:t>Marta</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Aportado</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$H$21</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E67E22"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$J$21</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Aportado + rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F766E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Marta</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$K$21</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="-20"/>
+        <c:axId val="100000001"/>
+        <c:axId val="100000002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="100000001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100000002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="D8DEE9"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="334155"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" sz="1000"/>
+              <a:t>Fondo ahorro</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Aportado</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$H$22</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E67E22"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$J$22</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Aportado + rentabilidad</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F766E"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0 &quot;€&quot;" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1"/>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="1"/>
+              <c:pt idx="0">
+                <c:v>Fondo ahorro</c:v>
+              </c:pt>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Movimientos!$K$22</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="-20"/>
+        <c:axId val="100000001"/>
+        <c:axId val="100000002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="100000001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100000002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100000001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="334155"/>
+              </a:solidFill>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:solidFill>
+        <a:srgbClr val="D8DEE9"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Grafico 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Grafico 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5407,7 +6018,7 @@
     <mergeCell ref="A25:K25"/>
     <mergeCell ref="A26:K26"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:D505">
+  <conditionalFormatting sqref="B6:D505">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($D6&lt;&gt;"",$D6=0)</formula>
     </cfRule>
@@ -5488,18 +6099,13 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
-    <col min="11" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="3" customWidth="1"/>
+    <col min="1" max="15" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
         <v>32</v>
       </c>
@@ -5518,7 +6124,7 @@
       <c r="N1" s="37"/>
       <c r="O1" s="37"/>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>33</v>
       </c>
@@ -5537,28 +6143,109 @@
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
     </row>
-    <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF0F766E"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="6" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+    </row>
+    <row r="2" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="38"/>
       <c r="C4" s="38"/>
       <c r="D4" s="38"/>
       <c r="F4" s="39" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G4" s="39"/>
       <c r="H4" s="39"/>
       <c r="I4" s="39"/>
       <c r="K4" s="40" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L4" s="40"/>
       <c r="M4" s="40"/>
       <c r="N4" s="40"/>
     </row>
-    <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="38"/>
       <c r="B5" s="38"/>
       <c r="C5" s="38"/>
@@ -5572,538 +6259,405 @@
       <c r="M5" s="40"/>
       <c r="N5" s="40"/>
     </row>
-    <row r="6" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="18" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="41"/>
       <c r="C7" s="41"/>
       <c r="D7" s="41"/>
       <c r="F7" s="41" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G7" s="41"/>
       <c r="H7" s="41"/>
       <c r="I7" s="41"/>
       <c r="K7" s="41" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L7" s="41"/>
       <c r="M7" s="41"/>
       <c r="N7" s="41"/>
     </row>
-    <row r="8" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="38" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="42" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" s="39" t="s">
+    <row r="8" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
-      <c r="K8" s="43" t="s">
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="39"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="38"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="39"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="38"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="42" t="s">
+      <c r="F9" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="42" t="s">
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="K9" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+    </row>
+    <row r="10" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="42"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+    </row>
+    <row r="11" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="47"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="47"/>
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="47"/>
+    </row>
+    <row r="12" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="48"/>
+      <c r="H13" s="48"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="K13" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="49"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="49"/>
+    </row>
+    <row r="14" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="42"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
+      <c r="N14" s="49"/>
+    </row>
+    <row r="15" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="47"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="47"/>
+      <c r="M15" s="47"/>
+      <c r="N15" s="50"/>
+    </row>
+    <row r="16" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="42" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="48"/>
+      <c r="H17" s="48"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="K17" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="L17" s="46"/>
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+    </row>
+    <row r="18" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+    </row>
+    <row r="19" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="47"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+    </row>
+    <row r="20" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="48" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="K21" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+    </row>
+    <row r="22" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="42"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="46"/>
+      <c r="L22" s="46"/>
+      <c r="M22" s="46"/>
+      <c r="N22" s="46"/>
+    </row>
+    <row r="23" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="47"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="50"/>
+      <c r="K23" s="50"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="50"/>
+    </row>
+    <row r="24" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="42" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="K12" s="40" t="s">
-        <v>45</v>
-      </c>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-    </row>
-    <row r="13" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="40"/>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="40"/>
-    </row>
-    <row r="14" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="40"/>
-    </row>
-    <row r="15" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
-      <c r="I15" s="39"/>
-      <c r="J15" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="K15" s="40" t="s">
-        <v>47</v>
-      </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-    </row>
-    <row r="16" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="40"/>
-      <c r="L16" s="40"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="40"/>
-    </row>
-    <row r="17" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="42" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="42" t="s">
-        <v>48</v>
-      </c>
-      <c r="K17" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="L17" s="40"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="40"/>
-    </row>
-    <row r="18" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="39"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="40"/>
-      <c r="L18" s="40"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-    </row>
-    <row r="19" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="42" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="42"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="L19" s="40"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="40"/>
-    </row>
-    <row r="20" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-    </row>
-    <row r="21" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="40"/>
-      <c r="N21" s="40"/>
-    </row>
-    <row r="22" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="40"/>
-    </row>
-    <row r="23" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="42"/>
-      <c r="K23" s="40" t="s">
-        <v>53</v>
-      </c>
-      <c r="L23" s="40"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="40"/>
-    </row>
-    <row r="24" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="42"/>
-      <c r="K24" s="40"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="40"/>
-      <c r="N24" s="40"/>
-    </row>
-    <row r="25" ht="16" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="44" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
       <c r="G25" s="44"/>
       <c r="H25" s="44"/>
       <c r="I25" s="44"/>
-      <c r="J25" s="44"/>
-      <c r="K25" s="44"/>
-      <c r="L25" s="44"/>
-      <c r="M25" s="44"/>
-      <c r="N25" s="44"/>
-      <c r="O25" s="44"/>
-    </row>
-    <row r="26" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45" t="s">
-        <v>56</v>
-      </c>
-      <c r="H26" s="45"/>
-      <c r="I26" s="45"/>
+      <c r="J25" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="K25" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+    </row>
+    <row r="26" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="42"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="44"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
       <c r="J26" s="45"/>
-      <c r="K26" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="L26" s="45"/>
-      <c r="M26" s="45"/>
-      <c r="N26" s="45"/>
-    </row>
-    <row r="27" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="46">
-        <v>46296</v>
-      </c>
-      <c r="B27" s="46"/>
-      <c r="C27" s="47" t="s">
-        <v>18</v>
-      </c>
+      <c r="K26" s="46"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+    </row>
+    <row r="27" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="47"/>
+      <c r="B27" s="47"/>
+      <c r="C27" s="47"/>
       <c r="D27" s="47"/>
       <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47" t="s">
+      <c r="F27" s="50"/>
+      <c r="G27" s="50"/>
+      <c r="H27" s="50"/>
+      <c r="I27" s="50"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="50"/>
+    </row>
+    <row r="28" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="42" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="48">
-        <v>1000</v>
-      </c>
-      <c r="L27" s="48"/>
-      <c r="M27" s="48"/>
-      <c r="N27" s="48"/>
-    </row>
-    <row r="28" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="46">
-        <v>46297</v>
-      </c>
-      <c r="B28" s="46"/>
-      <c r="C28" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="H28" s="47"/>
-      <c r="I28" s="47"/>
-      <c r="J28" s="47"/>
-      <c r="K28" s="48">
-        <v>300</v>
-      </c>
-      <c r="L28" s="48"/>
-      <c r="M28" s="48"/>
-      <c r="N28" s="48"/>
-    </row>
-    <row r="29" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="46">
-        <v>46297</v>
-      </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" s="47"/>
-      <c r="I29" s="47"/>
-      <c r="J29" s="47"/>
-      <c r="K29" s="48">
-        <v>200</v>
-      </c>
-      <c r="L29" s="48"/>
-      <c r="M29" s="48"/>
-      <c r="N29" s="48"/>
-    </row>
-    <row r="30" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="46">
-        <v>46298</v>
-      </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" s="47"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
-      <c r="K30" s="48">
-        <v>120</v>
-      </c>
-      <c r="L30" s="48"/>
-      <c r="M30" s="48"/>
-      <c r="N30" s="48"/>
-    </row>
-    <row r="31" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="46">
-        <v>46298</v>
-      </c>
-      <c r="B31" s="46"/>
-      <c r="C31" s="47" t="s">
-        <v>18</v>
-      </c>
+      <c r="G29" s="48"/>
+      <c r="H29" s="48"/>
+      <c r="I29" s="48"/>
+      <c r="J29" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="K29" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+    </row>
+    <row r="30" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="42"/>
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="48"/>
+      <c r="G30" s="48"/>
+      <c r="H30" s="48"/>
+      <c r="I30" s="48"/>
+      <c r="J30" s="45"/>
+      <c r="K30" s="46"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+    </row>
+    <row r="31" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="47"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
       <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
-      <c r="F31" s="47"/>
-      <c r="G31" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="H31" s="47"/>
-      <c r="I31" s="47"/>
-      <c r="J31" s="47"/>
-      <c r="K31" s="48">
-        <v>400</v>
-      </c>
-      <c r="L31" s="48"/>
-      <c r="M31" s="48"/>
-      <c r="N31" s="48"/>
-    </row>
-    <row r="32" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="46">
-        <v>46300</v>
-      </c>
-      <c r="B32" s="46"/>
-      <c r="C32" s="47" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="H32" s="47"/>
-      <c r="I32" s="47"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="48">
-        <v>150</v>
-      </c>
-      <c r="L32" s="48"/>
-      <c r="M32" s="48"/>
-      <c r="N32" s="48"/>
-    </row>
-    <row r="33" ht="16" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="49" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="49"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="50">
-        <v>2170</v>
-      </c>
-      <c r="L33" s="50"/>
-      <c r="M33" s="50"/>
-      <c r="N33" s="50"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="50"/>
+      <c r="G31" s="50"/>
+      <c r="H31" s="50"/>
+      <c r="I31" s="50"/>
+      <c r="J31" s="50"/>
+      <c r="K31" s="50"/>
+      <c r="L31" s="50"/>
+      <c r="M31" s="50"/>
+      <c r="N31" s="50"/>
+    </row>
+    <row r="32" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="56">
+  <mergeCells count="39">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A4:D5"/>
@@ -6112,54 +6666,37 @@
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="K7:N7"/>
-    <mergeCell ref="A8:D24"/>
-    <mergeCell ref="F8:I18"/>
-    <mergeCell ref="K8:N11"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="K12:N14"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="J12:J14"/>
-    <mergeCell ref="K15:N16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="A9:D10"/>
+    <mergeCell ref="F9:I10"/>
+    <mergeCell ref="K9:N10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="A13:D14"/>
+    <mergeCell ref="F13:I14"/>
+    <mergeCell ref="K13:N14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="A17:D18"/>
+    <mergeCell ref="F17:I18"/>
     <mergeCell ref="K17:N18"/>
     <mergeCell ref="E17:E18"/>
     <mergeCell ref="J17:J18"/>
-    <mergeCell ref="E19:J22"/>
-    <mergeCell ref="K19:N22"/>
-    <mergeCell ref="E23:J24"/>
-    <mergeCell ref="K23:N24"/>
-    <mergeCell ref="A25:O25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="A33:J33"/>
-    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="A21:D22"/>
+    <mergeCell ref="F21:I22"/>
+    <mergeCell ref="K21:N22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="A25:D26"/>
+    <mergeCell ref="F25:I26"/>
+    <mergeCell ref="K25:N26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="A29:D30"/>
+    <mergeCell ref="F29:I30"/>
+    <mergeCell ref="K29:N30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="A35:O35"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Distinguir ceros existentes y dibujar Sankey en el Excel
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -6,21 +6,21 @@
   <sheets>
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Gráficos" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Mapa del dinero" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="Gráfico del dinero" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Mapa del dinero'!$A1:$O35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Gráfico del dinero'!$A1:$M51</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -115,7 +115,7 @@
     <t>Para añadir una inversión: escribe su nombre (y su titular) en la fila amarilla; al rellenarla sale la siguiente. Para quitarla: borra su nombre y desaparece. Entra al momento en los desplegables.</t>
   </si>
   <si>
-    <t>La rentabilidad de cada cuenta o inversión se escribe en %. Para quitar un movimiento de este .xlsx, borra De, A e Importe y pon la fecha de hoy: escribir 0 solo oculta los datos. Al volver a descargar el Excel desde la app, los movimientos a cero se omiten de verdad.</t>
+    <t>Al poner 0 en un .xlsx no se borra solo. Para eliminarlo, borra De, A e Importe y pon Fecha a hoy. Si quieres que lo haga automáticamente SOLO al cambiar de positivo a 0, sigue las instrucciones de la macro opcional en README.md.</t>
   </si>
   <si>
     <t>Gráficos</t>
@@ -124,106 +124,34 @@
     <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
   </si>
   <si>
-    <t>Mapa del dinero</t>
+    <t>¿De dónde viene y a dónde va el dinero?</t>
   </si>
   <si>
-    <t>Lee cada recorrido de izquierda a derecha: origen → paso intermedio → destino. Una banda más larga significa más dinero.</t>
+    <t>El grosor de cada banda es proporcional al importe. Gris/azul/naranja: origen · colores: inversiones · azul oscuro: destino.</t>
   </si>
   <si>
-    <t xml:space="preserve">ENTRA DE FUERA
-1550,00 €</t>
+    <t>Origen</t>
   </si>
   <si>
-    <t xml:space="preserve">SIGUE EN CUENTAS
-380,00 €</t>
+    <t>Paso</t>
   </si>
   <si>
-    <t xml:space="preserve">ESTÁ INVERTIDO
-1170,00 €</t>
+    <t>Destino</t>
   </si>
   <si>
-    <t>ORIGEN</t>
+    <t>Aportaciones · Fondo ahorro</t>
   </si>
   <si>
-    <t>PASO INTERMEDIO</t>
+    <t>Sigue invertido · Fondo ahorro</t>
   </si>
   <si>
-    <t>DESTINO FINAL</t>
+    <t>Aportaciones · Marta</t>
   </si>
   <si>
-    <t xml:space="preserve">Exterior
-400,00 €</t>
+    <t>Sigue en cuenta · Marta</t>
   </si>
   <si>
-    <t>400,00 €  ▶</t>
-  </si>
-  <si>
-    <t>Sin cuenta intermedia</t>
-  </si>
-  <si>
-    <t>▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fondo indexado
-400,00 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exterior
-380,00 €</t>
-  </si>
-  <si>
-    <t>380,00 €  ▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sigue en Cuenta Myinvestor
-380,00 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exterior
-300,00 €</t>
-  </si>
-  <si>
-    <t>300,00 €  ▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vanguard Global Stock Index
-300,00 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exterior
-200,00 €</t>
-  </si>
-  <si>
-    <t>200,00 €  ▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fidelity MSCI World Index
-200,00 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exterior
-150,00 €</t>
-  </si>
-  <si>
-    <t>150,00 €  ▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iShares Developed World Index
-150,00 €</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exterior
-120,00 €</t>
-  </si>
-  <si>
-    <t>120,00 €  ▶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cartera indexada Metal
-120,00 €</t>
-  </si>
-  <si>
-    <t>El mapa refleja los movimientos al descargar el Excel. Para actualizarlo tras editarlo, vuelve a descargarlo desde la app.</t>
+    <t>Sigue invertido · Marta</t>
   </si>
 </sst>
 </file>
@@ -235,7 +163,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -319,26 +247,19 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
+      <color rgb="FF0F172A"/>
+      <sz val="17"/>
     </font>
     <font>
-      <b/>
       <color rgb="FF64748B"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF0F766E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1D4ED8"/>
-      <sz val="11"/>
+      <color rgb="FF0F172A"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -365,36 +286,6 @@
         <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF475569"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0F766E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCFBF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF14B8A6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2E8F0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -417,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -512,52 +403,15 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-        <sz val="10"/>
-      </font>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <font>
         <color rgb="FF0F172A"/>
@@ -1210,6 +1064,50 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="14287500" cy="9391650"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -6018,62 +5916,59 @@
     <mergeCell ref="A25:K25"/>
     <mergeCell ref="A26:K26"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:D505">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($D6&lt;&gt;"",$D6=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="A6:D505">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>AND($D5&lt;&gt;"",$D6="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$D5&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$D5=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F13:K19">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$F13&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>AND($F12&lt;&gt;"",$F13="")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>$F12=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I7:I12">
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="6" priority="4">
       <formula>AND($F7&lt;&gt;"",$H7&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I19">
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>$F13&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>AND($F12&lt;&gt;"",$F13="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F7:K12">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>$H7=""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F19">
-    <cfRule type="expression" dxfId="11" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="7">
+    <cfRule type="expression" dxfId="11" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:J19">
-    <cfRule type="cellIs" dxfId="13" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6175,530 +6070,151 @@
     <tabColor rgb="FF0F766E"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="3" customWidth="1"/>
+    <col min="1" max="13" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-    </row>
-    <row r="2" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+    </row>
+    <row r="2" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-    </row>
-    <row r="3" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="38" t="s">
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="F4" s="39" t="s">
+      <c r="E44" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="K4" s="40" t="s">
+      <c r="I44" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="L4" s="40"/>
-      <c r="M4" s="40"/>
-      <c r="N4" s="40"/>
-    </row>
-    <row r="5" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-    </row>
-    <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
+      <c r="M44" s="40" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="F7" s="41" t="s">
+      <c r="E45" t="s">
+        <v>24</v>
+      </c>
+      <c r="I45" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="K7" s="41" t="s">
+      <c r="M45" s="41">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>41</v>
       </c>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-    </row>
-    <row r="8" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="42" t="s">
+      <c r="E46" t="s">
+        <v>19</v>
+      </c>
+      <c r="I46" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="43" t="s">
+      <c r="M46" s="41">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>19</v>
+      </c>
+      <c r="E47" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="K9" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="L9" s="46"/>
-      <c r="M9" s="46"/>
-      <c r="N9" s="46"/>
-    </row>
-    <row r="10" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="42"/>
-      <c r="B10" s="42"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
-      <c r="N10" s="46"/>
-    </row>
-    <row r="11" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="47"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-    </row>
-    <row r="12" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="43" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="48" t="s">
+      <c r="M47" s="41">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="48"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="48"/>
-      <c r="J13" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="K13" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
-      <c r="N13" s="49"/>
-    </row>
-    <row r="14" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="42"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="49"/>
-      <c r="M14" s="49"/>
-      <c r="N14" s="49"/>
-    </row>
-    <row r="15" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="47"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="47"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="47"/>
-      <c r="M15" s="47"/>
-      <c r="N15" s="50"/>
-    </row>
-    <row r="16" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="43" t="s">
-        <v>51</v>
-      </c>
-      <c r="F17" s="48" t="s">
+      <c r="E48" t="s">
+        <v>22</v>
+      </c>
+      <c r="I48" t="s">
+        <v>43</v>
+      </c>
+      <c r="M48" s="41">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>39</v>
+      </c>
+      <c r="E49" t="s">
+        <v>25</v>
+      </c>
+      <c r="I49" t="s">
+        <v>40</v>
+      </c>
+      <c r="M49" s="41">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="48"/>
-      <c r="H17" s="48"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="K17" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="L17" s="46"/>
-      <c r="M17" s="46"/>
-      <c r="N17" s="46"/>
-    </row>
-    <row r="18" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="42"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="48"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="46"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="46"/>
-      <c r="N18" s="46"/>
-    </row>
-    <row r="19" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="47"/>
-      <c r="B19" s="47"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="47"/>
-      <c r="I19" s="47"/>
-      <c r="J19" s="47"/>
-      <c r="K19" s="47"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="50"/>
-    </row>
-    <row r="20" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="42"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="K21" s="46" t="s">
-        <v>55</v>
-      </c>
-      <c r="L21" s="46"/>
-      <c r="M21" s="46"/>
-      <c r="N21" s="46"/>
-    </row>
-    <row r="22" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="42"/>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="45"/>
-      <c r="K22" s="46"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="46"/>
-      <c r="N22" s="46"/>
-    </row>
-    <row r="23" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="47"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="47"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="50"/>
-      <c r="I23" s="50"/>
-      <c r="J23" s="50"/>
-      <c r="K23" s="50"/>
-      <c r="L23" s="50"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
-    </row>
-    <row r="24" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="42" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="43" t="s">
-        <v>57</v>
-      </c>
-      <c r="F25" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="G25" s="44"/>
-      <c r="H25" s="44"/>
-      <c r="I25" s="44"/>
-      <c r="J25" s="45" t="s">
-        <v>45</v>
-      </c>
-      <c r="K25" s="46" t="s">
-        <v>58</v>
-      </c>
-      <c r="L25" s="46"/>
-      <c r="M25" s="46"/>
-      <c r="N25" s="46"/>
-    </row>
-    <row r="26" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="42"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="45"/>
-      <c r="K26" s="46"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="46"/>
-      <c r="N26" s="46"/>
-    </row>
-    <row r="27" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="47"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="50"/>
-      <c r="K27" s="50"/>
-      <c r="L27" s="50"/>
-      <c r="M27" s="50"/>
-      <c r="N27" s="50"/>
-    </row>
-    <row r="28" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="42" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="F29" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="G29" s="48"/>
-      <c r="H29" s="48"/>
-      <c r="I29" s="48"/>
-      <c r="J29" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="K29" s="46" t="s">
-        <v>61</v>
-      </c>
-      <c r="L29" s="46"/>
-      <c r="M29" s="46"/>
-      <c r="N29" s="46"/>
-    </row>
-    <row r="30" ht="19" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="42"/>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="48"/>
-      <c r="I30" s="48"/>
-      <c r="J30" s="45"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="46"/>
-      <c r="N30" s="46"/>
-    </row>
-    <row r="31" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="47"/>
-      <c r="B31" s="47"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="50"/>
-      <c r="K31" s="50"/>
-      <c r="L31" s="50"/>
-      <c r="M31" s="50"/>
-      <c r="N31" s="50"/>
-    </row>
-    <row r="32" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="19" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="19" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
+      <c r="E50" t="s">
+        <v>23</v>
+      </c>
+      <c r="I50" t="s">
+        <v>43</v>
+      </c>
+      <c r="M50" s="41">
+        <v>120</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A4:D5"/>
-    <mergeCell ref="F4:I5"/>
-    <mergeCell ref="K4:N5"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="A9:D10"/>
-    <mergeCell ref="F9:I10"/>
-    <mergeCell ref="K9:N10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="A13:D14"/>
-    <mergeCell ref="F13:I14"/>
-    <mergeCell ref="K13:N14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="A17:D18"/>
-    <mergeCell ref="F17:I18"/>
-    <mergeCell ref="K17:N18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="A21:D22"/>
-    <mergeCell ref="F21:I22"/>
-    <mergeCell ref="K21:N22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="A25:D26"/>
-    <mergeCell ref="F25:I26"/>
-    <mergeCell ref="K25:N26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="A29:D30"/>
-    <mergeCell ref="F29:I30"/>
-    <mergeCell ref="K29:N30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="A35:O35"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reducir gráfico de bandas y separar etiquetas de gráficos de cuentas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -12,15 +12,15 @@
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Gráfico del dinero'!$A1:$M51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Gráfico del dinero'!$A1:$M40</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -124,6 +124,15 @@
     <t>Todo sale de la hoja «Movimientos»: lo que cambies allí, cambia aquí.</t>
   </si>
   <si>
+    <t>■ Aportado</t>
+  </si>
+  <si>
+    <t>■ Rentabilidad</t>
+  </si>
+  <si>
+    <t>■ Aportado + rentabilidad</t>
+  </si>
+  <si>
     <t>¿De dónde viene y a dónde va el dinero?</t>
   </si>
   <si>
@@ -163,7 +172,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -247,6 +256,21 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF2563EB"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFE67E22"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F766E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF0F172A"/>
       <sz val="17"/>
     </font>
@@ -308,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -403,9 +427,18 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -583,7 +616,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.18"/>
+          <c:y val="0.18"/>
+          <c:w val="0.76"/>
+          <c:h val="0.68"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -749,7 +792,7 @@
         <c:axPos val="b"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="none"/>
         <c:crossAx val="100000002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -764,7 +807,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines/>
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -774,24 +816,6 @@
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -837,7 +861,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.18"/>
+          <c:y val="0.18"/>
+          <c:w val="0.76"/>
+          <c:h val="0.68"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -1003,7 +1037,7 @@
         <c:axPos val="b"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="none"/>
         <c:crossAx val="100000002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
@@ -1018,7 +1052,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines/>
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1028,24 +1061,6 @@
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0">
-              <a:solidFill>
-                <a:srgbClr val="334155"/>
-              </a:solidFill>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -1066,12 +1081,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="14287500" cy="9391650"/>
+    <xdr:ext cx="10001250" cy="6574154"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -1110,15 +1125,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1140,15 +1155,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5994,7 +6009,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="15" customWidth="1"/>
@@ -6052,11 +6067,67 @@
     <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="J17" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="38"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="38"/>
+      <c r="N17" s="38"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="J18" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="K18" s="39"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="39"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B19" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
+      <c r="J19" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="K19" s="40"/>
+      <c r="L19" s="40"/>
+      <c r="M19" s="40"/>
+      <c r="N19" s="40"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="8">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="J17:N17"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="J18:N18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="J19:N19"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -6070,141 +6141,141 @@
     <tabColor rgb="FF0F766E"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="13" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
+      <c r="A1" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
     </row>
     <row r="2" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A44" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="E44" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="I44" s="40" t="s">
+      <c r="A2" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="M44" s="40" t="s">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>40</v>
+      </c>
+      <c r="I33" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="M33" s="43" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>39</v>
-      </c>
-      <c r="E45" t="s">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" t="s">
         <v>24</v>
       </c>
-      <c r="I45" t="s">
-        <v>40</v>
-      </c>
-      <c r="M45" s="41">
+      <c r="I34" t="s">
+        <v>43</v>
+      </c>
+      <c r="M34" s="44">
         <v>400</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>41</v>
-      </c>
-      <c r="E46" t="s">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" t="s">
         <v>19</v>
       </c>
-      <c r="I46" t="s">
+      <c r="I35" t="s">
+        <v>45</v>
+      </c>
+      <c r="M35" s="44">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" t="s">
+        <v>46</v>
+      </c>
+      <c r="M36" s="44">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" t="s">
+        <v>22</v>
+      </c>
+      <c r="I37" t="s">
+        <v>46</v>
+      </c>
+      <c r="M37" s="44">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>42</v>
       </c>
-      <c r="M46" s="41">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="E38" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" t="s">
+        <v>43</v>
+      </c>
+      <c r="M38" s="44">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>19</v>
       </c>
-      <c r="E47" t="s">
-        <v>20</v>
-      </c>
-      <c r="I47" t="s">
-        <v>43</v>
-      </c>
-      <c r="M47" s="41">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>19</v>
-      </c>
-      <c r="E48" t="s">
-        <v>22</v>
-      </c>
-      <c r="I48" t="s">
-        <v>43</v>
-      </c>
-      <c r="M48" s="41">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>39</v>
-      </c>
-      <c r="E49" t="s">
-        <v>25</v>
-      </c>
-      <c r="I49" t="s">
-        <v>40</v>
-      </c>
-      <c r="M49" s="41">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E50" t="s">
+      <c r="E39" t="s">
         <v>23</v>
       </c>
-      <c r="I50" t="s">
-        <v>43</v>
-      </c>
-      <c r="M50" s="41">
+      <c r="I39" t="s">
+        <v>46</v>
+      </c>
+      <c r="M39" s="44">
         <v>120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Quitar gráfico del dinero de las exportaciones Excel
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -6,21 +6,19 @@
   <sheets>
     <sheet sheetId="1" name="Movimientos" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Gráficos" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Gráfico del dinero" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Gráfico del dinero'!$A1:$M40</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -132,36 +130,6 @@
   <si>
     <t>■ Aportado + rentabilidad</t>
   </si>
-  <si>
-    <t>¿De dónde viene y a dónde va el dinero?</t>
-  </si>
-  <si>
-    <t>El grosor de cada banda es proporcional al importe. Gris/azul/naranja: origen · colores: inversiones · azul oscuro: destino.</t>
-  </si>
-  <si>
-    <t>Origen</t>
-  </si>
-  <si>
-    <t>Paso</t>
-  </si>
-  <si>
-    <t>Destino</t>
-  </si>
-  <si>
-    <t>Aportaciones · Fondo ahorro</t>
-  </si>
-  <si>
-    <t>Sigue invertido · Fondo ahorro</t>
-  </si>
-  <si>
-    <t>Aportaciones · Marta</t>
-  </si>
-  <si>
-    <t>Sigue en cuenta · Marta</t>
-  </si>
-  <si>
-    <t>Sigue invertido · Marta</t>
-  </si>
 </sst>
 </file>
 
@@ -172,7 +140,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00 %"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -269,19 +237,6 @@
       <color rgb="FF0F766E"/>
       <sz val="10"/>
     </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="17"/>
-    </font>
-    <font>
-      <color rgb="FF64748B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -332,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -436,10 +391,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1079,50 +1030,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="10001250" cy="6574154"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -6133,159 +6040,4 @@
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FF0F766E"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="13" width="17" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-    </row>
-    <row r="2" ht="25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="E33" s="43" t="s">
-        <v>40</v>
-      </c>
-      <c r="I33" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="M33" s="43" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E34" t="s">
-        <v>24</v>
-      </c>
-      <c r="I34" t="s">
-        <v>43</v>
-      </c>
-      <c r="M34" s="44">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>44</v>
-      </c>
-      <c r="E35" t="s">
-        <v>19</v>
-      </c>
-      <c r="I35" t="s">
-        <v>45</v>
-      </c>
-      <c r="M35" s="44">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" t="s">
-        <v>20</v>
-      </c>
-      <c r="I36" t="s">
-        <v>46</v>
-      </c>
-      <c r="M36" s="44">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" t="s">
-        <v>22</v>
-      </c>
-      <c r="I37" t="s">
-        <v>46</v>
-      </c>
-      <c r="M37" s="44">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>42</v>
-      </c>
-      <c r="E38" t="s">
-        <v>25</v>
-      </c>
-      <c r="I38" t="s">
-        <v>43</v>
-      </c>
-      <c r="M38" s="44">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>19</v>
-      </c>
-      <c r="E39" t="s">
-        <v>23</v>
-      </c>
-      <c r="I39" t="s">
-        <v>46</v>
-      </c>
-      <c r="M39" s="44">
-        <v>120</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-  </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustar gráficos y cuenta Luis con aportaciones netas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -11,14 +11,14 @@
     <definedName name="ListaNombres">OFFSET('Movimientos'!$F$6,0,0,MAX(COUNTA('Movimientos'!$F$6:$F$19),1),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Movimientos'!$A1:$O27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Movimientos'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Gráficos'!$A1:$O25</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="37">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -77,13 +77,16 @@
     <t>Exterior</t>
   </si>
   <si>
-    <t>Cuenta Myinvestor</t>
+    <t>Cuenta Luis</t>
+  </si>
+  <si>
+    <t>Fondo indexado</t>
+  </si>
+  <si>
+    <t>Luis</t>
   </si>
   <si>
     <t>Vanguard Global Stock Index</t>
-  </si>
-  <si>
-    <t>Marta</t>
   </si>
   <si>
     <t>Fidelity MSCI World Index</t>
@@ -92,16 +95,13 @@
     <t>Cartera indexada Metal</t>
   </si>
   <si>
-    <t>Fondo indexado</t>
+    <t>Fondo ahorro</t>
   </si>
   <si>
     <t>iShares Developed World Index</t>
   </si>
   <si>
-    <t>Fondo ahorro</t>
-  </si>
-  <si>
-    <t>Total Cuenta Myinvestor-Marta</t>
+    <t>Total Cuenta Luis</t>
   </si>
   <si>
     <t>Total Fondo ahorro</t>
@@ -557,7 +557,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-ES" sz="1000"/>
-              <a:t>Marta</a:t>
+              <a:t>Luis</a:t>
             </a:r>
             <a:endParaRPr/>
           </a:p>
@@ -572,10 +572,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.18"/>
-          <c:y val="0.18"/>
-          <c:w val="0.76"/>
-          <c:h val="0.68"/>
+          <c:x val="0.07"/>
+          <c:y val="0.14"/>
+          <c:w val="0.86"/>
+          <c:h val="0.75"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -604,7 +604,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -621,7 +621,7 @@
             <c:strLit>
               <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Marta</c:v>
+                <c:v>Luis</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
@@ -653,7 +653,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -670,7 +670,7 @@
             <c:strLit>
               <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Marta</c:v>
+                <c:v>Luis</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
@@ -702,7 +702,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -719,7 +719,7 @@
             <c:strLit>
               <c:ptCount val="1"/>
               <c:pt idx="0">
-                <c:v>Marta</c:v>
+                <c:v>Luis</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
@@ -761,7 +761,7 @@
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="none"/>
         <c:crossAx val="100000001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
@@ -817,10 +817,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.18"/>
-          <c:y val="0.18"/>
-          <c:w val="0.76"/>
-          <c:h val="0.68"/>
+          <c:x val="0.07"/>
+          <c:y val="0.14"/>
+          <c:w val="0.86"/>
+          <c:h val="0.75"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -849,7 +849,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -898,7 +898,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -947,7 +947,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="850" b="1"/>
+                  <a:defRPr sz="750" b="1"/>
                 </a:pPr>
                 <a:endParaRPr/>
               </a:p>
@@ -1006,7 +1006,7 @@
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="none"/>
         <c:crossAx val="100000001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
@@ -1032,16 +1032,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>838200</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>628650</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1062,16 +1062,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>838200</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>628650</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1569,7 +1569,7 @@
         <v>20</v>
       </c>
       <c r="D7" s="11">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>19</v>
@@ -1578,31 +1578,31 @@
         <v>21</v>
       </c>
       <c r="H7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor"))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis"))),"")</f>
       </c>
       <c r="I7" s="17"/>
       <c r="J7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$K7=""),"",$K7-$H7))),"")</f>
       </c>
       <c r="K7" s="16">
-        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Myinvestor",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Myinvestor")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Myinvestor")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$H7=0),"",IF($I7="",$H7,$H7*(1+$I7))))),"")</f>
+        <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",IF(OR($H7="",$H7=0),"",IF($I7="",$H7,$H7*(1+$I7))))),"")</f>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="11">
+        <v>620</v>
+      </c>
+      <c r="F8" s="18" t="s">
         <v>22</v>
-      </c>
-      <c r="D8" s="11">
-        <v>200</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>20</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>21</v>
@@ -1620,19 +1620,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="11">
+        <v>300</v>
+      </c>
+      <c r="F9" s="19" t="s">
         <v>23</v>
-      </c>
-      <c r="D9" s="11">
-        <v>120</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>22</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>21</v>
@@ -1650,19 +1650,19 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="11">
+        <v>200</v>
+      </c>
+      <c r="F10" s="19" t="s">
         <v>24</v>
-      </c>
-      <c r="D10" s="11">
-        <v>400</v>
-      </c>
-      <c r="F10" s="19" t="s">
-        <v>23</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>21</v>
@@ -1680,22 +1680,22 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="11">
+        <v>120</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="D11" s="11">
-        <v>150</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>26</v>
       </c>
       <c r="H11" s="23">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
@@ -1710,16 +1710,22 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
-        <v>46317</v>
-      </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
+        <v>46302</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="11">
+        <v>150</v>
+      </c>
       <c r="F12" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>26</v>
       </c>
       <c r="H12" s="23">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
@@ -1894,16 +1900,16 @@
         <v>21</v>
       </c>
       <c r="H21" s="31">
-        <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Luis")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Luis")),"")</f>
       </c>
       <c r="I21" s="32">
         <f>IFERROR(IF($H21=0,"",$J21/$H21),"")</f>
       </c>
       <c r="J21" s="31">
-        <f>IFERROR(IF(SUMIFS($J$6:$J$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($J$6:$J$19,$G$6:$G$19,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($J$6:$J$19,$G$6:$G$19,"Luis")=0,"",SUMIFS($J$6:$J$19,$G$6:$G$19,"Luis")),"")</f>
       </c>
       <c r="K21" s="31">
-        <f>IFERROR(IF(SUMIFS($K$6:$K$19,$G$6:$G$19,"Marta")=0,"",SUMIFS($K$6:$K$19,$G$6:$G$19,"Marta")),"")</f>
+        <f>IFERROR(IF(SUMIFS($K$6:$K$19,$G$6:$G$19,"Luis")=0,"",SUMIFS($K$6:$K$19,$G$6:$G$19,"Luis")),"")</f>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1917,7 +1923,7 @@
         <v>28</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H22" s="31">
         <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")),"")</f>
@@ -5880,7 +5886,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F19">
     <cfRule type="expression" dxfId="10" priority="6">
-      <formula>AND($F9&lt;&gt;"",$G9="Marta")</formula>
+      <formula>AND($F9&lt;&gt;"",$G9="Luis")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="11" priority="7">
       <formula>AND($F9&lt;&gt;"",$G9="Fondo ahorro")</formula>
@@ -5916,7 +5922,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="15" width="15" customWidth="1"/>
@@ -5974,67 +5980,70 @@
     <row r="14" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="38" t="s">
+    <row r="17" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B20" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
-      <c r="J17" s="38" t="s">
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
+      <c r="J20" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="K17" s="38"/>
-      <c r="L17" s="38"/>
-      <c r="M17" s="38"/>
-      <c r="N17" s="38"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="39" t="s">
+      <c r="K20" s="38"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="38"/>
+      <c r="N20" s="38"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="J18" s="39" t="s">
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="J21" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="K18" s="39"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="39"/>
-      <c r="N18" s="39"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="40" t="s">
+      <c r="K21" s="39"/>
+      <c r="L21" s="39"/>
+      <c r="M21" s="39"/>
+      <c r="N21" s="39"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="J19" s="40" t="s">
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="J22" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="K19" s="40"/>
-      <c r="L19" s="40"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="40"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
+      <c r="N22" s="40"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="J17:N17"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="J18:N18"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="J19:N19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="J21:N21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="J22:N22"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Exportar libro XLSM con limpieza y compactación automática
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Movimientos.xlsx
+++ b/Movimientos.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="39">
   <si>
     <t>Myinvestor</t>
   </si>
@@ -80,13 +80,19 @@
     <t>Cuenta Luis</t>
   </si>
   <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>cuenta</t>
+  </si>
+  <si>
     <t>Fondo indexado</t>
   </si>
   <si>
-    <t>Luis</t>
+    <t>Vanguard Global Stock Index</t>
   </si>
   <si>
-    <t>Vanguard Global Stock Index</t>
+    <t>inversion</t>
   </si>
   <si>
     <t>Fidelity MSCI World Index</t>
@@ -113,7 +119,7 @@
     <t>Para añadir un fondo o cartera: escribe un nombre nuevo en De/A (hasta siete). Se refleja en el resumen; para quitarlo, elimina todas sus referencias De/A. Revisa el titular y % al borrar nombres anteriores.</t>
   </si>
   <si>
-    <t>Al poner 0 en un .xlsx no se borra solo. Para eliminarlo, borra De, A e Importe y pon Fecha a hoy. Si quieres que lo haga automáticamente SOLO al cambiar de positivo a 0, sigue las instrucciones de la macro opcional en README.md.</t>
+    <t>En el .xlsm, habilita macros en Excel de escritorio: al pasar un importe positivo a 0, De/A se limpian y los movimientos restantes suben. En el .xlsx sin macros hay que hacerlo a mano. Un movimiento que ya venía a 0 se conserva.</t>
   </si>
   <si>
     <t>Gráficos</t>
@@ -325,8 +331,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
@@ -1418,7 +1425,7 @@
     <tabColor rgb="FF1D4ED8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R505"/>
+  <dimension ref="A1:W505"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -1435,6 +1442,11 @@
     <col min="16" max="16" width="9" hidden="1" customWidth="1"/>
     <col min="17" max="17" width="9" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="9" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="9" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="9" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="9" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="9" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1538,7 +1550,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>46296</v>
       </c>
@@ -1568,8 +1580,20 @@
       <c r="R6" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S6" t="s">
+        <v>19</v>
+      </c>
+      <c r="T6" t="s">
+        <v>20</v>
+      </c>
+      <c r="V6" t="s">
+        <v>21</v>
+      </c>
+      <c r="W6">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>46297</v>
       </c>
@@ -1577,7 +1601,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D7" s="11">
         <v>400</v>
@@ -1586,7 +1610,7 @@
         <v>19</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H7" s="16">
         <f>IFERROR(IF($F7="","",IF(AND(COUNTIFS($C$6:$C$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")+COUNTIFS($B$6:$B$505,"Cuenta Luis",$D$6:$D$505,"&gt;0")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis")&lt;=0,SUMPRODUCT(--($H8:$H10&lt;&gt;""))=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cuenta Luis")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cuenta Luis"))),"")</f>
@@ -1607,8 +1631,17 @@
       <c r="R7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S7" t="s">
+        <v>23</v>
+      </c>
+      <c r="T7" t="s">
+        <v>20</v>
+      </c>
+      <c r="V7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>46298</v>
       </c>
@@ -1622,10 +1655,10 @@
         <v>620</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H8" s="16">
         <f>IFERROR(IF($F8="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Vanguard Global Stock Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Vanguard Global Stock Index"))),"")</f>
@@ -1644,10 +1677,22 @@
         <f>IFERROR(IF(AND($C8&lt;&gt;"",$C8&lt;&gt;"Exterior",COUNTIF($C$6:C8,$C8)=1,COUNTIF($R$6:$R$12,$C8)=0,COUNTIF($B$6:$B$505,$C8)=0),$C8,""),"")</f>
       </c>
       <c r="R8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="S8" t="s">
+        <v>25</v>
+      </c>
+      <c r="T8" t="s">
+        <v>20</v>
+      </c>
+      <c r="V8" t="s">
+        <v>24</v>
+      </c>
+      <c r="W8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>46299</v>
       </c>
@@ -1655,16 +1700,16 @@
         <v>19</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="11">
         <v>300</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H9" s="20">
         <f>IFERROR(IF($F9="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fidelity MSCI World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fidelity MSCI World Index"))),"")</f>
@@ -1683,10 +1728,19 @@
         <f>IFERROR(IF(AND($C9&lt;&gt;"",$C9&lt;&gt;"Exterior",COUNTIF($C$6:C9,$C9)=1,COUNTIF($R$6:$R$12,$C9)=0,COUNTIF($B$6:$B$505,$C9)=0),$C9,""),"")</f>
       </c>
       <c r="R9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="S9" t="s">
+        <v>26</v>
+      </c>
+      <c r="T9" t="s">
+        <v>20</v>
+      </c>
+      <c r="V9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>46300</v>
       </c>
@@ -1694,16 +1748,16 @@
         <v>19</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D10" s="11">
         <v>200</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H10" s="20">
         <f>IFERROR(IF($F10="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Cartera indexada Metal")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Cartera indexada Metal"))),"")</f>
@@ -1722,10 +1776,19 @@
         <f>IFERROR(IF(AND($C10&lt;&gt;"",$C10&lt;&gt;"Exterior",COUNTIF($C$6:C10,$C10)=1,COUNTIF($R$6:$R$12,$C10)=0,COUNTIF($B$6:$B$505,$C10)=0),$C10,""),"")</f>
       </c>
       <c r="R10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S10" t="s">
+        <v>22</v>
+      </c>
+      <c r="T10" t="s">
+        <v>27</v>
+      </c>
+      <c r="V10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>46301</v>
       </c>
@@ -1733,16 +1796,16 @@
         <v>19</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D11" s="11">
         <v>120</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H11" s="23">
         <f>IFERROR(IF($F11="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"Fondo indexado")-SUMIFS($D$6:$D$505,$B$6:$B$505,"Fondo indexado"))),"")</f>
@@ -1761,7 +1824,16 @@
         <f>IFERROR(IF(AND($C11&lt;&gt;"",$C11&lt;&gt;"Exterior",COUNTIF($C$6:C11,$C11)=1,COUNTIF($R$6:$R$12,$C11)=0,COUNTIF($B$6:$B$505,$C11)=0),$C11,""),"")</f>
       </c>
       <c r="R11" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="S11" t="s">
+        <v>28</v>
+      </c>
+      <c r="T11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V11" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -1772,16 +1844,16 @@
         <v>18</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D12" s="11">
         <v>150</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H12" s="23">
         <f>IFERROR(IF($F12="","",IF(AND(SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")&gt;0,SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index")&lt;=0),"",SUMIFS($D$6:$D$505,$C$6:$C$505,"iShares Developed World Index")-SUMIFS($D$6:$D$505,$B$6:$B$505,"iShares Developed World Index"))),"")</f>
@@ -1800,7 +1872,7 @@
         <f>IFERROR(IF(AND($C12&lt;&gt;"",$C12&lt;&gt;"Exterior",COUNTIF($C$6:C12,$C12)=1,COUNTIF($R$6:$R$12,$C12)=0,COUNTIF($B$6:$B$505,$C12)=0),$C12,""),"")</f>
       </c>
       <c r="R12" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -2035,10 +2107,10 @@
       <c r="C21" s="10"/>
       <c r="D21" s="11"/>
       <c r="F21" s="29" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G21" s="30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H21" s="31">
         <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Luis")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Luis")),"")</f>
@@ -2067,10 +2139,10 @@
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
       <c r="F22" s="29" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H22" s="31">
         <f>IFERROR(IF(SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")=0,"",SUMIFS($H$6:$H$19,$G$6:$G$19,"Fondo ahorro")),"")</f>
@@ -2099,7 +2171,7 @@
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
       <c r="F23" s="33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G23" s="33"/>
       <c r="H23" s="34">
@@ -2137,7 +2209,7 @@
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="36" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B25" s="36"/>
       <c r="C25" s="36"/>
@@ -2158,7 +2230,7 @@
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="36" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B26" s="36"/>
       <c r="C26" s="36"/>
@@ -8981,7 +9053,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -9000,7 +9072,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -9036,14 +9108,14 @@
     <row r="19" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C20" s="38"/>
       <c r="D20" s="38"/>
       <c r="E20" s="38"/>
       <c r="F20" s="38"/>
       <c r="J20" s="38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K20" s="38"/>
       <c r="L20" s="38"/>
@@ -9052,14 +9124,14 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="39" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="39"/>
       <c r="E21" s="39"/>
       <c r="F21" s="39"/>
       <c r="J21" s="39" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K21" s="39"/>
       <c r="L21" s="39"/>
@@ -9068,14 +9140,14 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" s="40" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C22" s="40"/>
       <c r="D22" s="40"/>
       <c r="E22" s="40"/>
       <c r="F22" s="40"/>
       <c r="J22" s="40" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K22" s="40"/>
       <c r="L22" s="40"/>

</xml_diff>